<commit_message>
Monitor update 2026-06-23 20:24 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A3:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -583,8 +583,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add three live test sources + fix Node.js 24 action versions
- actions/checkout@v4 -> v7, actions/setup-python@v5 -> v6 (no more warning)
- Add Competitor B: CoinGecko crypto prices (changes every ~5 min, ideal demo)
- Add Competitor C: EUR exchange rates via Frankfurter API
- Config now shows 3 university tabs in TEST_MODE
- Dashboard already shows 6 real Bitcoin/Ethereum changes from first test run

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WORLDOMETERS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXCHANGE_RATES" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRYPTO_MARKETS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR_RATES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -575,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A3:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -583,6 +585,58 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:13</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>USD / GBP</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>1.32437</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1.32437</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
     <row r="1"/>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -593,33 +647,163 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:13</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>23-Jun 21:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>USD / GBP</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>1.32437</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>1.32437</t>
+          <t>GBP 47,257.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>GBP 1,257.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BNB</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>GBP 435.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>GBP 52.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Hyperliquid</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>GBP 47.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Zcash</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>GBP 316.54</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Monitor update 2026-06-23 21:54 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -630,11 +630,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -650,8 +651,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Bitcoin</t>
@@ -660,6 +666,11 @@
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>GBP 47,257.00</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>GBP 47,395.00</t>
         </is>
       </c>
     </row>
@@ -675,8 +686,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Ethereum</t>
@@ -685,6 +701,11 @@
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>GBP 1,257.76</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>GBP 1,261.23</t>
         </is>
       </c>
     </row>
@@ -700,8 +721,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>BNB</t>
@@ -710,6 +736,11 @@
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>GBP 435.92</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>GBP 436.71</t>
         </is>
       </c>
     </row>
@@ -725,8 +756,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Solana</t>
@@ -735,6 +771,11 @@
       <c r="B13" s="4" t="inlineStr">
         <is>
           <t>GBP 52.18</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>GBP 52.38</t>
         </is>
       </c>
     </row>
@@ -750,8 +791,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Hyperliquid</t>
@@ -762,7 +808,13 @@
           <t>GBP 47.40</t>
         </is>
       </c>
-    </row>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>GBP 47.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -774,8 +826,13 @@
           <t>23-Jun 21:37</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>23-Jun 21:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Zcash</t>
@@ -784,6 +841,11 @@
       <c r="B19" s="4" t="inlineStr">
         <is>
           <t>GBP 316.54</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>GBP 316.33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace test sources with realistic clearing simulation + tabbed dashboard
- 3 simulated universities with real UK course names and A-level/UCAS grades
- Grades drop in clearing order (ABB→BBB→BBC) staggered across courses
- 3 changes will appear on next Actions poll (BSc Computing, Computer Science, Data Science)
- Dashboard rebuilt with clickable tabs (one per university)
- Every course table now shows first-seen timestamp and initial requirement
- Changed cells highlighted; Node.js 24 action warning already fixed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -11,6 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXCHANGE_RATES" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRYPTO_MARKETS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR_RATES" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_A" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_C" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -630,15 +633,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A3:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -663,7 +664,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -688,7 +688,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -713,7 +712,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -738,7 +736,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -806,4 +803,52 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add clearing day test + demo dashboard with multi-column layout
- run_clearing_day_test.py: simulates BCU/Coventry/DMU across 09:00-10:30
  verifying multi-column layout, new/removed courses, and requirement drops
- Generated demo dashboard showing 3 universities × 4-6 courses each,
  with up to 3 timestamp columns per course row and horizontal scroll
- Data files updated with realistic clearing-day change history

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -7,13 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WORLDOMETERS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXCHANGE_RATES" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRYPTO_MARKETS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EUR_RATES" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_A" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_B" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_C" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_C" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,12 +475,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C10"/>
+  <dimension ref="A3:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="3" ht="22" customHeight="1">
@@ -495,29 +492,39 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 20:56</t>
+          <t>14-Aug 09:30</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 20:58</t>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>BSc (Hons) Computing</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Total: 111,820,082</t>
+          <t>BBC or 112 UCAS tariff points. GCSE Mathematics B/5 and English C/4. Non-standard qualifications considered – call 0121 331 5595.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Total: 111,820,082</t>
+          <t>CLEARING VACANCY – BCC or 104 UCAS tariff points. GCSE Mathematics essential. Call BCU Clearing: 0121 331 5595.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING – limited spaces remaining. 96 UCAS tariff points or above. GCSE Mathematics required. Call NOW: 0121 331 5595.</t>
         </is>
       </c>
     </row>
@@ -529,19 +536,19 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 20:56</t>
+          <t>14-Aug 09:30</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>BA (Hons) Business Management</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Total: 38,828,995</t>
+          <t>CCC or 96 UCAS tariff points. GCSE Maths and English C/4. BTEC MMP accepted.</t>
         </is>
       </c>
     </row>
@@ -553,19 +560,131 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 20:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>BSc (Hons) Nursing (Adult)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Total: 24,910,387</t>
+          <t>BBC or 112 UCAS tariff points. Science A-level no longer mandatory for clearing. Relevant care experience required. Enhanced DBS and Occupational Health check.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Care experience required. Enhanced DBS check required. Call 0121 331 5595.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>LLB Law</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>BBB or 120 UCAS tariff points. GCSE English Language B/5.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BBC or 112 tariff points. GCSE English Language C/4 accepted. All A-levels welcome. Call 0121 331 5595.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>BEng (Hons) Civil Engineering</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>BBC or 112 UCAS tariff points. Mathematics A-level required. GCSE Maths 4.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Mathematics A-level required. GCSE Maths 4. Call 0121 331 5595.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>BSc (Hons) Psychology</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>BBC or 112 UCAS tariff points. GCSE English Language and Maths C/4. Psychology or Biology A-level desirable.</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Open to all A-level combinations. GCSE English and Maths required. Call 0121 331 5595.</t>
         </is>
       </c>
     </row>
@@ -580,12 +699,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C4"/>
+  <dimension ref="A3:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="3" ht="22" customHeight="1">
@@ -596,29 +716,175 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:13</t>
+          <t>14-Aug 09:30</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:14</t>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>USD / GBP</t>
+          <t>BSc (Hons) Computer Science</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>1.32437</t>
+          <t>BBB or 120 UCAS tariff points. Mathematics A-level required. GCSE Maths 4.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>1.32437</t>
+          <t>CLEARING VACANCY – BBC or 112 tariff points. Mathematics A-level required. Call Coventry Clearing: 02477 655 645.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING – final spaces. BCC or equivalent. Mathematics A-level required. Call 02477 655 645.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>BA (Hons) International Business</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>BBC or 112 UCAS tariff points. GCSE English Language and Maths 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BSc (Hons) Sport and Exercise Science</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>BCC or 104 UCAS tariff points. GCSE English Language and Maths 4.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – CCC or 96 tariff points. Call 02477 655 645.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>MPharm Pharmacy (4 years)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ABB or 136 UCAS tariff points. Chemistry A-level required. Interview required.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>BBB or 120 UCAS tariff points. Chemistry A-level required. Interview required.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BBB or 120 tariff points. Chemistry A-level required. Interview required. Call 02477 655 645.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>BA (Hons) Criminology</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>BCC or 104 UCAS tariff points. No specific A-levels. GCSE English Language and Maths 4.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>CCC or 96 UCAS tariff points. GCSE English Language and Maths 4.</t>
         </is>
       </c>
     </row>
@@ -633,13 +899,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -648,22 +918,33 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>BSc (Hons) Data Science</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>GBP 47,257.00</t>
-        </is>
-      </c>
-    </row>
+          <t>BBC or 112 UCAS tariff points. Mathematics A-level recommended but not required. GCSE Maths 4.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. GCSE Maths essential. Call DMU Clearing: 0116 250 6070.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -672,22 +953,43 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>BA (Hons) Accounting and Finance</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>GBP 1,257.76</t>
-        </is>
-      </c>
-    </row>
+          <t>BBC or 112 UCAS tariff points. Maths or Business background preferred. GCSE Maths B/5.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Call 0116 250 6070.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING – final spaces. CCC or 96 tariff points. Call 0116 250 6070.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -696,22 +998,43 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>BEng (Hons) Electronic Engineering</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>GBP 435.92</t>
-        </is>
-      </c>
-    </row>
+          <t>BBC or 112 UCAS tariff points. Mathematics A-level required. GCSE Maths 5.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Mathematics A-level required. Call 0116 250 6070.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING – final spaces. BBC or equivalent. Mathematics required. Call 0116 250 6070.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -720,22 +1043,43 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+          <t>14-Aug 09:30</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>BSc (Hons) Architecture (ARB/RIBA Part 1)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>GBP 52.18</t>
-        </is>
-      </c>
-    </row>
+          <t>ABB or 128 UCAS tariff points. Portfolio required. GCSE English and Maths C/4.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>BBB or 120 UCAS tariff points. Portfolio required. Creative or scientific A-level preferred.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BBC or 112 tariff points. Portfolio required. Call 0116 250 6070.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -744,19 +1088,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
+          <t>14-Aug 10:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>14-Aug 10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Hyperliquid</t>
+          <t>BSc (Hons) Environmental Science</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>GBP 47.40</t>
+          <t>BBC or 112 UCAS tariff points. Science A-level preferred. GCSE Maths and English C/4.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>CLEARING VACANCY – BCC or 104 tariff points. Science A-level welcomed. Call 0116 250 6070.</t>
         </is>
       </c>
     </row>
@@ -768,87 +1122,23 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>23-Jun 21:37</t>
+          <t>14-Aug 10:30</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Zcash</t>
+          <t>BA (Hons) Fashion Design</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>GBP 316.54</t>
+          <t>CCC or 96 UCAS tariff points. Art or Design A-level. Portfolio required. GCSE English C/4.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Switch to real live data: ClinicalTrials.gov API integration
Replaces simulation with 3 tabs of real UK clinical trials data:
- UK Cancer Trials / UK Cardiovascular Trials / UK Diabetes Trials
- Eligibility criteria text = descriptive entry requirements
- Status/criteria changes → new timestamp columns (same pipeline as clearing)
- No browser needed; free public JSON API; runs on GitHub Actions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_A" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_B" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLEARING_UNI_C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIALS_CANCER" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIALS_CARDIO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIALS_DIABETES" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -899,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A3:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -908,8 +911,6 @@
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -944,7 +945,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -989,7 +989,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -1034,7 +1033,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -1079,7 +1077,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -1141,4 +1138,52 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Monitor update 2026-06-24 13:33 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,12 +1146,350 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A3:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A Clinical Study to Investigate the Efficacy and Safety of an Investigational Combination Therapy With BNT324 and BNT327 in Patients With Advanced Lung Cancer [NCT06892548]</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Aged ≥18 years at the time of giving informed consent.
+* Histological or cytological confirmed unresectable advanced/metastatic lung cancer. Histological classification may be based on tumor samples prior to metastatic disease. Participants with mixed histology must be classified based on the main component. Participants with NSCLC are eligible with any or no PD-L1 expression. Participants with AGA-positive disease must have received targeted therapy prior to enrollment in this study.
+  * Part 1: Participants with NSCLC and SCLC
+  * Part 2 Cohort 1: Participants with NSCLC (subpopulation 1) AGA negative, 1L
+  * Part 2 Cohort 2: Participants with SCLC, 2L+
+  * Part 2 Cohort 3: Participants with NSCLC (subpopulation 1) AGA negative, 2L+
+  * Part 2 Cohort 4: Participants with NSCLC (subpopulation 2) AGA negative, 1L
+  * Part 2 Cohort 5: Participants with NSCLC (subpopulation 2) AGA negative, 2L+
+  * Part 2 Cohort 6: Participants with NSCLC AGA positive
+  * Part 2 Cohort 7: Participants with SCLC, 1L
+* Have measurable disease defined by RECIST version 1.1.
+* Have an Eastern Cooperative Oncology Group performance status of 0 or 1.
+* Have a life expectancy of ≥12 weeks.
+Exclusion Criteria:
+* Prior treatment with B7-H3 targeted therapy.
+* Prior treatment with ADC with topoisomerase inhibitor (e.g., datopotamab deruxtecan, trastuzumab deruxtecan). Note: This exclusion applies to participants in the first-line/treatment-naïve cohorts in the advanced/metastatic setting. Prior treatment with ADC with topoisomerase inhibitor payload is only allowed for participants in the second-line plus cohorts in the advanced/metastatic setting.
+* Is a candidate to locoregional treatment (including surgical resection, stereotactic radiotherapy or tumor ablation) with potential to induce complete or near complete response and prolonged tumor control (sometimes described as "radical" intent), per investigator's assessment.
+* Has a history of significant hematologic toxicity to prior lines of therapy, as assessed by investigator, e.g., Grade 4 febrile neutropenia or recurrent/persistent Grade 3 to 4 neutropenia.
+NOTE: Other protocol defined Inclusion/Exclusion criteria may apply to all or some participants depending on the cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Study of Revumenib in Combination With Intensive Chemotherapy in Newly Diagnosed Acute Myeloid Leukemia (AML) With a NPM1 Mutation [NCT07211958]</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 12 Years – Not specified  |  All
+Key Inclusion Criteria:
+* Participants must have newly diagnosed and previously untreated AML and be candidates for intensive chemotherapy.
+* Presence of an NPM1 mutation.
+* Eastern Cooperative Oncology Group performance status ≤2 (≤1 if \&gt;65 years old); Karnofsky or Lansky ≥40.
+* Have a life expectancy of ≥3 months as judged by the Investigator.
+* Negative serum pregnancy test.
+* Adequate liver, kidney, and cardiac function.
+Key Exclusion Criteria:
+* Diagnosis of active acute promyelocytic leukemia.
+* Active central nervous system disease.
+* Fridericia's corrected QT interval (QTcF) \&gt;450 milliseconds at screening, diagnosis or suspicion of Long QT syndrome or family history of Long QT syndrome.
+* Any gastrointestinal (GI) issue of the upper GI tract likely to affect oral drug absorption or ingestion.
+* Any concurrent malignancy requiring active therapy (except breast or prostate cancer stable on or responding to endocrine therapy).
+* Inability to swallow oral medication.
+* Pregnant or nursing females.
+* Participant has known active or chronic hepatitis B or active hepatitis C (HCV) infection or human immunodeficiency virus (HIV)-positive with detectable viral load.
+Note: Additional inclusion/exclusion criteria may apply, per protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>SPECTA: Screening Cancer Patients for Efficient Clinical Trial Access [NCT02834884]</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 12 Years – Not specified  |  All
+* Patients with pathologically confirmed selected tumor types (at site or centrally);
+* Mandatory availability of adequate human biological material (HBM);
+* Centrally performed confirmation of HBM adequacy in terms of quality and quantity for SPECTA downstream project requirements;
+* Age ≥ 12 years;
+* Absence of any psychological, familial, sociological or geographical condition potentially hampering compliance with the study protocol and follow-up schedule;
+* Written informed consent according to applicable legal and ethical requirements;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Beamion LUNG-2: A Study to Test Whether Zongertinib (BI 1810631) Helps People With Advanced Non-small Cell Lung Cancer With HER2 Mutations Compared With Standard Treatment [NCT06151574]</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion criteria:
+1. Signed and dated written informed consent form (ICF) in accordance with International Council for Harmonisation of Technical Requirements for Pharmaceuticals for Human Use - Good Clinical Practice (ICH-GCP) and local legislation prior to admission to the trial.
+2. Patients ≥18 years of age or over the legal age of consent in countries where that is greater than 18 years at the time of signature of the ICF.
+3. Histologically or cytologically confirmed diagnosis of an advanced and/or metastatic non-squamous Non-small cell lung cancer (NSCLC).
+4. Documented Human epidermal growth factor receptor 2 (HER2) mutation in the Tyrosine kinase domain (TKD) as per local lab results.
+5. An archival tumor tissue sample must be submitted to the central laboratory after inclusion of the patient to retrospectively confirm the HER2 status. If no archival tissue is available, this may be acceptable in exceptional cases after written agreement with the sponsor.
+6. Patients who have not received any systemic treatment for unresectable, locally advanced or metastatic disease and are not eligible for curative therapy.
+7. Presence of at least one measurable lesion according to Response evaluation criteria in solid tumors (RECIST) 1.1, as determined by the local site investigator/radiology assessment.
+8. Eligible to receive treatment with the selected platinum-based doublet-chemotherapy (i.e. cisplatin/pemetrexed or carboplatin/pemetrexed) and pembrolizumab in accordance with the Summaries of Product Characteristics (SmPC)/Product Information.
+Further inclusion criteria apply.
+Exclusion criteria:
+1. Previous or concomitant malignancies other than the one treated in this trial within the last 5 years, except;
+   * effectively treated non-melanoma skin cancers
+   * effectively treated carcinoma in situ of the cervix
+   * effectively treated ductal carcinoma in situ
+   * other effectively treated malignancy that is considered cured by local treatment
+2. Tumors with targetable alterations with approved available therapy.
+3. Lung-specific intercurrent clinically significant severe illness based on investigators assessment.
+4. Patients who must or wish to continue the intake of restricted medications or any drug considered likely to interfere with the safe conduct of the trial.
+5. Major surgery (major according to the investigator's assessment) performed within 4 weeks prior to randomization or planned within 6 months after screening, e.g. hip replacement.
+6. Any history of or concomitant condition that, in the opinion of the investigator, would compromise the patient's ability to comply with the trial or interfere with the evaluation of the safety and efficacy of the test drug.
+7. History or presence of cardiovascular abnormalities such as uncontrolled hypertension, congestive heart failure New York Heart Association (NYHA) classification of ≥ III or IV, unstable angina or poorly controlled arrhythmia which are considered as clinically relevant by the investigator. Myocardial infarction, stroke, or pulmonary embolism within 6 months prior to randomization.
+8. Any clinically important abnormalities (as assessed by the investigator) in rhythm, conduction, or morphology of resting electrocardiograms, e.g. complete left bundle branch block, third degree heart block.
+Further exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>A Study Evaluating the Efficacy and Safety of Inavolisib Plus Fulvestrant Compared With Alpelisib Plus Fulvestrant in Participants With HR-Positive, HER2-Negative, PIK3CA Mutated, Locally Advanced or Metastatic Breast Cancer Post CDK4/6i and Endocrine Combination Therapy [NCT05646862]</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria for Main Study and Sub-study:
+* If pre/perimenopausal women and men treatment with luteinizing hormone-releasing hormone (LHRH) agonist therapy beginning at least 2 weeks prior to Day 1 of Cycle 1
+* Histologically or cytologically confirmed adenocarcinoma of the breast that is locally advanced or metastatic and is not amenable to surgical or radiation therapy with curative intent
+* Documented HR +/ HER2- tumor according to American Society of Clinical Oncology/College of American Pathologists (ASCO/CAP) guidelines
+* Confirmation of biomarker eligibility: detection of specified mutation(s) of PIK3CA via specified test
+* Disease progression after or during treatment with a combination of CDK4/6i and endocrine therapy: \&lt;= 2 prior lines of systemic therapy in mBC setting; CDK4/6i based therapy does not need to be the last one received prior study entry; one line of chemotherapy in mBC setting allowed
+* Measurable or evaluable disease per Response Evaluation Criteria in Solid Tumors version 1.1 (RECIST v1.1)
+* Participants for whom endocrine-based therapy is recommended and treatment with cytotoxic chemotherapy is not indicated at time of entry into the study, as per national or local treatment guidelines
+* Eastern Cooperative Oncology Group (ECOG) Performance Status of 0, 1, or 2
+* Life expectancy of \&gt; 6 months
+* Adequate hematologic and organ function prior to initiation of study treatment
+Exclusion Criteria for both Main Study and Sub-study:
+* Metaplastic breast cancer
+* Prior treatment in locally advanced or metastatic setting with any PI3K, AKT, or mTOR inhibitor or any agent whose mechanism of action is to inhibit the PI3K/-AKT/-mTOR pathway
+* Participant who relapsed with documented evidence of progression \&gt; 12 months from completion of adjuvant CDK4/6i based therapy with no treatment for metastatic disease
+* Type 2 diabetes requiring ongoing systemic treatment at the time of study entry; or any history of Type 1 diabetes
+* Inability or unwillingness to swallow pills
+* Malabsorption syndrome or other condition that would interfere with enteral absorption
+* Any history of leptomeningeal disease or carcinomatous meningitis
+* Known and untreated, or active central nervous system (CNS) metastases. Participants with a history of treated CNS metastases are eligible if they meet specific certain criteria
+* Any concurrent ocular or intraocular condition that, in the opinion of the investigator, would require medical or surgical intervention during the study period to prevent or treat vision loss that might result from that condition
+* Active inflammatory or infectious conditions in either eye or history of idiopathic or autoimmune-associated uveitis in either eye
+* Requirement for daily supplemental oxygen
+* Symptomatic active lung disease, including pneumonitis
+* History of or active inflammatory bowel disease
+* Any active bowel inflammation
+* Clinically significant and active liver disease, including severe liver impairment, viral or other hepatitis, current alcohol abuse, or cirrhosis
+* Participants with known human immunodeficiency virus infection that meet specific criteria
+* History of other malignancy within 5 years prior to screening, except for cancers with very low risk of recurrence
+* Chronic therapy of \&gt;= 10 mg of prednisone per day or an equivalent dose of other anti-inflammatory corticosteroids or immunosuppressants for a chronic disease
+* Active ongoing osteonecrosis of the jaw
+Exclusion Criteria for Main Study Only:
+* Pregnant, lactating, or breastfeeding, or intending to become pregnant during the study or at least 60 days after the final dose of study treatment
+* Known active, systemic infection at study enrollment, or any major episode of infection requiring treatment with intravenous antibiotics or hospitalization within 7 days prior to Day 1 of Cycle 1
+* Investigational drug(s) within 4 weeks before randomization or within 5 half-lives of the investigational drug(s), whichever is longer
+* Allergy or hypersensitivity to components or excipients of the inavolisib, fulvestrant, or alpelisib formulations
+* History of severe cutaneous reactions like Stevens-Johnson Syndrome, Erythema Multiforme, Toxic Epidermal Necrolysis, or Drug Reaction with Eosinphilia and Systemic Symptoms
+Exclusion Criteria for Sub-study Only:
+* Pregnant, lactating, or breastfeeding, or intending to become pregnant during the substudy or within 2 weeks after the final dose of inavolisib and within 2 years after the final dose of fulvestrant, whichever is longer
+* Known active, systemic infection at study enrollment, or any major episode of infection requiring treatment with intravenous antibiotics or hospitalization within 7 days prior to Day -4 of Cycle 1
+* Investigational drug(s) within 4 weeks prior to Day -4 or within 5 half-lives of the investigational drug(s), whichever is longer
+* Allergy or hypersensitivity to components or excipients of the inavolisib, fulvestrant formulations
+* Treatment with mild, moderate, or strong inducers of CYP2B6, CYP3A4, and/or CYP2C19 (including St. John's Wort) within 14 days or 5 drug-elimination half-lives, whichever is longer, prior to initiation of study treatment on Day -4 until after the final PK sample has been collected on Day 15 of Cycle 1
+* Treatment with mild, moderate, or strong inhibitors of CYP2B6, CYP3A4, and/or CYP2C19 (including grapefruit juice or supplements) within 14 days or 5 drug-elimination half-lives, whichever is longer, prior to initiation of study treatment on Day -4 until after the final PK sample has been collected on Day 15 of Cycle 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>DAREON™-5: A Study to Test Whether Different Doses of BI 764532 Help People With Small Cell Lung Cancer or Other Neuroendocrine Cancers [NCT05882058]</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion criteria:
+1. Male or female participants ≥18 years old and at least at the legal age of consent in countries where it is greater than 18 years at the time of signature of the informed consent form (ICF).
+2. Signed and dated written informed consent in accordance with International Council for Harmonisation-Good Clinical Practice (ICH-GCP) and local legislation prior to admission to the trial.
+3. Part 1: Histologically or cytologically confirmed, cancer of the following histologies:
+   * Small cell lung cancer (SCLC)
+   * Extra-pulmonary neuroendocrine carcinoma (epNEC) (except Merkel cell carcinoma (MCC), Medullary thyroid cancer (MTC) and Neuroendocrine prostate cancer (NEPC))
+   * Large cell neuroendocrine carcinoma (LCNEC) of the lung Patients with tumours with mixed histologies for any above type are eligible only if the neuroendocrine carcinoma/small tumour cells component is predominant and represents at least 50% of the overall tumour tissue.
+   Patients must have progressed or recurred after standard of care therapy
+   * SCLC: after at least two prior lines of therapy, including at least one platinum-based regimen; in countries where standard of care in first line therapy includes PD-L1 inhibitor treatment patients should have received the combination of platinum-based regimen plus PD-L1 inhibitor unless they have been unable to receive checkpoint inhibitor treatment.
+   * Therapy includes PD-L1 inhibitor treatment; patients should have received the combination of platinum-based regimen plus PD-L1 inhibitor unless they have been unable to receive checkpoint inhibitor treatment.
+   * epNEC/LCNEC: after at least one platinum-based regimen. Part 2 and part 3: Histologically or cytologically confirmed epNEC (except MCC, MTC and NEPC) with centrally assessed DLL3 high expression status. Patients must have progressed or recurred after at least one platinum-based regimen.
+4. Eastern Cooperative Oncology Group (ECOG) score of 0 or 1.,
+5. Measurable lesions as defined per Response Evaluation Criteria In Solid Tumours (RECIST) v 1.1 within 21 days prior to the first dose of BI 764532.
+6. Part 1: Availability of archival tumour tissue sample Part 2 and part 3: Availability of archival formalin-fixed paraffin-embedded (FFPE) tumour tissue sample. Following specimens are not allowed: Fine Needle Aspiration (FNA), Cytology samples, decalcified bone samples.
+7. Adequate organ function as defined in the protocol.
+8. All toxicities related to previous anti-cancer therapies have resolved = Common Terminology Criteria for Adverse Events (CTCAE) Grade 1 prior to trial treatment administration (except for alopecia, peripheral neuropathy, fatigue and endocrinopathies controlled by replacement therapy which must be = CTCAE Grade 2 and amenorrhea/menstrual disorders which can be any grade).
+9. Women of childbearing potential (WOCBP) and men able to father a child must be ready and able to use acceptable methods of birth control per ICH M3 (R2) that result in a low failure rate of less than 1% per year when used consistently and correctly. A list of contraception methods meeting these criteria and instructions on the duration of their use is provided in the participant information
+10. Only for Part 3, at the timepoint of Screening 02:
+    * For Cycle 1, patients should be willing to stay within 1 hour driving distance for 48 hours after IMP administration and confirm availability of a caregiver for the same timeframe.
+    * Patients should be considered suitable by the investigator to follow instructions applicable to the reduced monitoring cohort, such as taking their temperature and administration of oral medication at home if needed.
+Exclusion criteria:
+1. Untreated or symptomatic brain metastases. (Part 2 and part 3: identified during the mandatory assessment by brain MRI within 21 days before first trial drug administration.) Participants with treated, stable brain metastases are eligible provided they meet the following criteria:
+   * Radiotherapy or surgery for brain metastases was completed at least 2 weeks prior to the first administration of BI 764532.
+   * Patient is off steroids for at least 7 days (physiologic doses of steroids are permitted), and the patient is off anti-epileptic drugs for at least 7 days or on stable doses of anti-epileptic drugs for malignant central nervous system (CNS) disease.
+2. Presence of leptomeningeal disease or, part 2 and part 3: epidural disease including spinal cord compression.
+3. Part 1: Active/previous history of interstitial lung disease or non-infectious pneumonitis (any grade).
+   Part 2 and part 3: Active/previous history of interstitial lung disease, pulmonary fibrosis, organizing pneumonia or non-infectious pneumonitis (any grade). Patients with a history of therapy-related pneumonitis that is considered clinically resolved are eligible.
+4. Participants who experienced severe, life-threatening immune-mediated adverse events or infusion-related reactions including those that lead to permanent discontinuation while on treatment with immuno-oncology agents.
+5. Prior anti-cancer therapy:
+   * Patients who have been treated with any other anti-cancer drug within 4 weeks or within 5 half-life periods (whichever is shorter) prior to first administration of BI 764532.
+   * Patients who have been treated with extensive field radiotherapy including whole brain irradiation within 2 weeks prior to first administration of BI 764532.
+6. Previous treatment with Delta-like ligand 3 (DLL3)-targeting T cell engagers or cell therapies.
+7. Diagnosis of immunodeficiency or systemic steroid therapy or any other form of immunosuppressive therapy within 7 days prior to the first dose of BI 764532. Physiological replacement of steroids is allowed.
+8. Unresolved toxicity from prior anti-tumour therapy, defined in the inclusion criteria.
+Further exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Study to Evaluate Adverse Events, Change in Disease Activity, and How Oral ABBV-101 Moves Through the Body in Adult Participants With B-Cell Malignancies [NCT05753501]</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* For Dose Escalation (Part 1) only (including backfill): Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have a documented diagnosis for one of the following third line or later B-cell malignancies, from one of the following world health organization (WHO)-defined histologies (Swerdlow et al 2016):
+  * Chronic lymphocytic leukemia (CLL)/small lymphocytic lymphoma (SLL)
+    1. For Dose Escalation (Part 1) backfill only - Bruton's tyrosine kinase inhibitor (BTKi)/Bruton's tyrosine kinase degrader (BTKd)-naïve CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received at least one prior systemic therapy that cannot be a BTK inhibitor or degrader, and, with the exception of BTK pathway agents, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+    2. For Dose Escalation (Part 1) backfill only - BTKi/BCL-2i combination regimen-exposed 2L CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received one prior systemic therapy with a BTKi and BCL-2i combination regimen, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+  * Chimeric antigen receptor T-cells (CAR-T)/hematopoietic cell transplant (HCT) relapsed/refractory (R/R) or ineligible diffuse large b-cell lymphoma (DLBCL) from the following histologies: DLBCL not otherwise specified (NOS) (germinal center B cell \[GCB\] and non-GCB DLBCL), T-cell/histiocyte-rich large B-cell lymphoma, primary mediastinal (thymic) large B-cell lymphoma, intravascular large B-cell lymphoma, anaplastic lymphoma kinase positive (ALK+) large B-cell lymphoma, high-grade B-cell lymphoma with MYC and BCL2 and/or BCL6 rearrangements, and high-grade B-cell lymphoma NOS.
+  * Mantle cell lymphoma (MCL)
+  * Follicular lymphoma \[FL\] (grades 1-3b)
+  * Marginal zone lymphoma \[MZL\] (splenic, extranodal, and nodal)
+  * Waldenström macroglobulinemia (WM)
+  * Transformed indolent non-Hodgkin's lymphoma (iNHL)
+* For Dose Expansion (Part 2a) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment.
+* For Dose Expansion (Part 2a) DLBCL only: Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have documented diagnosis of CAR-T/HCT R/R or ineligible non-GCB DLBCL who are in their third line or later treatment with histology based on criteria established by the WHO.
+* For Dose Exploration of ABBV-101 combination with venetoclax (Part 2b) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment: In safety lead-in for each dose level, participants must have received at least one prior systemic therapy.
+* Has an Eastern Cooperative Oncology Group (ECOG) Performance Status (PS) of 0, 1, or 2. For EU only: Participant has an ECOG PS of 0 or 1.
+* Participant has a life expectancy \&gt;= 12 weeks.
+* Prior Bruton's tyrosine kinase inhibitor (BTKi) is allowed.
+* Adequate hematologic, renal, and hepatic function per the protocol.
+Exclusion Criteria:
+* Previously treated with a Bruton's tyrosine kinase (BTK) degrader.
+* Known active central nervous system (CNS) disease, or primary CNS lymphoma. Participants with prior CNS disease that have been effectively treated may be eligible.
+* Uncontrolled active systemic infection requiring systemic treatment that is ongoing or was completed \&lt;= 14 days before the first dose of study drug, or active cytomegalovirus infection.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1162,12 +1500,383 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A3:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Effect of Venglustat Tablets on Left Ventricular Mass Index in Male and Female Adult Participants With Fabry Disease [NCT05280548]</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 65 Years  |  All
+Inclusion Criteria:
+* Male and female participants aged 18 to 65 with previously confirmed diagnosis of Fabry disease and a history of clinical symptoms of Fabry disease.
+* Participants may be receiving treatment with agalsidase alfa, agalsidase beta, or migalastat, or may be untreated.
+* Left ventricular hypertrophy.
+* Contraception for male or female participants: not pregnant or breastfeeding; no sperm donating for male participant.
+* A signed informed consent must be provided prior to any study-related procedures.
+Exclusion Criteria:
+* History of transient ischemic attack, stroke, myocardial infarction, heart failure, major cardiovascular surgery or kidney transplantation.
+* History of seizures currently requiring treatment.
+* Underlying medical condition that may cause or contribute to left ventricular hypertrophy.
+* Asymmetric hypertrophy by cardiac MRI at screening if considered by central reader to be not related to Fabry disease.
+* Advanced cardiac fibrosis, defined as significant late gadolinium enhancement affecting 3 or more segments involving \&gt;50% of myocardial thickness on screening cardiac MRI.
+* History of clinically significant cardiac arrhythmia. Atrial fibrillation that is well controlled on a stable medical regimen for at least 12 months is not an exclusion if the CHA2DS2-VASc score is 0 for males or 1 for females.
+* Estimated glomerular filtration rate \&lt;45 mL/min/1.73m2.
+* Presence of severe depression as measured by Beck's Depression Inventory (BDI)-II \&gt;28 and/or a history of an untreated, unstable major affective disorder within 1 year of the screening visit.
+* Patients with hepatitis C, HIV, or hepatitis B infection.
+* Positive SARS-CoV-2 virus test within 2 weeks of enrollment, or COVID-19 requiring hospitalization within 6 months of enrollment.
+* History of drug and/or alcohol abuse.
+* Moderate to severe hepatic impairment.
+* History of or active hepatobiliary disease.
+* Liver enzymes (alanine aminotransferase/aspartate aminotransferase) or total bilirubin \&gt;2 times the upper limit of normal.
+* Strong or moderate inducers or inhibitors of cytochrome P450 CYP3A4 within 14 days or 5 half-lives, whichever is longer, prior to randomization.
+* Known contraindication to undergoing MRI or known hypersensitivity to gadolinium-based contrast agents.
+The above information is not intended to contain all considerations relevant to a potential participation in a clinical trial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Assess the Safety and Efficacy of Sovateltide in Patients With Acute Cerebral Ischemic Stroke [NCT05691244]</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 80 Years  |  All
+Inclusion Criteria:
+A patient will be eligible for inclusion in the study if he/she fulfills the following criteria:
+1. Adult males or females aged 18 - 80 years of age.
+2. Consent obtained per national laws and regulations, and in accordance with the applicable ethics committee requirements prior to study procedures.
+3. A stroke is ischemic in origin that is diagnosed clinically and/or radiologically confirmed by Computed Tomography (CT) scan or diagnostic magnetic resonance imaging (MRI) prior to enrolment. No hemorrhage as proved by cerebral CT/MRI scan.
+4. Cerebral ischemic stroke patients presenting within 24 hours after the onset of symptoms with NIHSS score of ≥8 and \&lt;20, NIHSS Level of Consciousness (1A) score \&lt;2 at the time of screening. This includes cerebral ischemic stroke patients who completely recovered from earlier episodes before having a new or fresh stroke having a pre-stroke historical measure of mRS score of 0-2.
+5. The patient is \&lt;24 hours from the time of stroke onset when the first dose of sovateltide is administered. Time of onset is when symptoms began; for stroke that occurred during sleep, time of onset is when the patient was last seen or was self- reported to be normal.
+6. Reasonable expectation of availability to receive the full sovateltide/placebo course of therapy and to be available for subsequent follow-up visits.
+Exclusion Criteria:
+A patient will not be eligible for inclusion in this study if they meet any of the following exclusion criteria:
+1. Patients receiving endovascular therapy or is a candidate for any surgical intervention for the treatment of stroke, which may include but not limited to endovascular techniques.
+2. Patients classified as comatose are defined as a patient who requires repeated stimulation to attend or is obtunded and requires strong or painful stimulation to make movements (NIHSS Level of Consciousness (1A) score ≥2).
+3. Evidence of intracranial hemorrhage (intracerebral hematoma, intraventricular hemorrhage, subarachnoid hemorrhage (SAH), epidural hemorrhage, acute or chronic subdural hematoma (SDH)) on the baseline CT or MRI scan.
+4. Known pregnancy and lactating women.
+5. Known medical history of neurological (other than current acute ischemic stroke) or psychiatric condition that, in the investigator's opinion, would confound the neurological and functional evaluations, lead to further deterioration of neurological status, or interfere with participation in this study.
+6. Concurrent participation in any other therapeutic clinical trial.
+7. Evidence of any other major life-threatening or serious medical condition that would prevent completion of the study protocol impair the assessment of outcome, or in which sovateltide therapy would be contraindicated or might cause harm to the patient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Study With Omecamtiv Mecarbil (CK-1827452) to Treat Chronic Heart Failure With Severely Reduced Ejection Fraction [NCT06736574]</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 85 Years  |  All
+Inclusion Criteria:
+Adult patients who meet all the following criteria at screening may be included in the study:
+* Are between ≥ 18 years and ≤ 85 years at the signing of informed consent
+* Have a history of chronic HFrEF, defined as requiring treatment for HF for a minimum of 3 months prior to screening
+* Are receiving oral loop diuretics on a regular schedule
+* Patients without AFF on screening ECG:
+  * LVEF \&lt; 30% within 6 months of screening
+  * Elevated N-terminal prohormone of B-type natriuretic peptide (NT-proBNP) ≥ 1000 pg/mL (BNP ≥ 300 pg/mL)
+* Patients with AFF on screening ECG:
+  * LVEF \&lt; 25% within 6 months of screening
+  * Elevated N-terminal prohormone of B-type natriuretic peptide (NT-proBNP) ≥ 3000 pg/mL (BNP ≥ 900 pg/mL)
+  * Not currently taking digoxin
+* Meet one of the following criteria for a recent HF event:
+  * Are currently hospitalized with the primary reason of HF
+  * Had an HF event (as defined in the primary endpoint) within 12 months prior to screening. For the purposes of a qualifying HF event, subcutaneous furosemide will be treated as equivalent to intravenous furosemide Or
+  * Had outpatient escalation of oral diuretics due to worsening signs and symptoms of heart failure plus one of two additional criteria sustained for at least 1 week: (1) at least 50% or 1.5-fold increase in daily loop-diuretic-equivalent dose; (2) the addition of a new diuretic class to a loop diuretic.
+* Are established on regional standard-of-care HF therapies for at least 30 days prior to screening
+* Systolic blood pressure ≤ 140 mmHg
+Exclusion Criteria:
+Any of the following criteria will exclude potential patients from the study:
+* Have AFF on the screening ECG and are currently taking digoxin
+* Have had any event or procedure that may have resulted in a change in ejection fraction, including, but not limited to, acute coronary syndrome and/or any coronary revascularization, cardiac surgery, valve surgery, any coronary revascularization, and/or cardiac resynchronization, or cardiac contractility modulation therapy within 3 months of screening
+* Are admitted to a long-term care facility or hospice
+* Have a projected survival of \&lt; 12 months due to non-cardiovascular causes based on clinical judgment
+* Are receiving intravenous inotropes or intravenous vasopressors ≤ 3 days prior to screening
+* Are receiving mechanical hemodynamic support or mechanical ventilation ≤ 7 days prior to screening
+* Are receiving intravenous diuretics, intravenous vasodilators, or supplemental oxygen therapy ≤ 12 hours prior to screening (except for nocturnal supplemental oxygen for sleep apnea or heart failure)
+* Have an estimated glomerular filtration rate (eGFR) \&lt; 20 mL/min/1.73m2 or receiving dialysis at screening
+* Have previously had a solid organ transplant
+* Are receiving treatment in another investigational device or drug study or are within 30 days of ending such investigational treatment at screening
+* Have received omecamtiv mecarbil in a previous clinical trial
+* Are pregnant or planning pregnancy during the study period, or planning to breastfeed during treatment with IP or within 5 days after the end of treatment with IP
+* Have primary infiltrative cardiomyopathy (e.g. cardiac amyloidosis) or severe stenotic valvular disease</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Percutaneous or Surgical Repair In Mitral Prolapse And Regurgitation for ≥60 Year-olds (PRIMARY) [NCT05051033]</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 60 Years – Not specified  |  All
+The patient population for this trial consists of adults with severe, primary degenerative MR for whom the local heart team has verified that an indication for MV intervention is present and for whom both transcatheter edge-to-edge and surgical repair strategies are anatomically feasible. Specific inclusion and exclusion criteria are listed below. All patients who meet eligibility criteria will be included in the study regardless of gender, race, or ethnicity.
+Inclusion Criteria:
+* Adult patients ≥60 years with moderately-severe or severe (3+ or 4+/4+) primary degenerative (Carpentier type II) MR defined by transthoracic echocardiography
+* Clinical indication for MV intervention and anatomic candidate for both surgical MV repair and transcatheter edge-to-edge repair (TEER) per local heart team assessment with central eligibility committee verification
+* Patients across the surgical risk spectrum (low, intermediate, and high risk) depending on local heart team assessment and central eligibility committee verification (see ACC/AHA 2020 guidelines for the management of patients with valvular heart disease)
+* Patients with AF who meet an indication for a concomitant ablation procedure be included provided the local heart team and central eligibility committee decide they are eligible for both catheter-based and surgical ablation.
+* Ability to perform 6-minute walk test (6MWT) and complete Kansas City Cardiomyopathy Questionnaire (KCCQ) instrument
+Exclusion Criteria:
+* Non-degenerative types of primary MR (e.g., cleft leaflet)
+* Secondary or functional MR
+* Hypertrophic obstructive cardiomyopathy
+* Presence of an IVC filter or permanent pacing/ICD leads that would interfere with TEER per local heart team assessment
+* Known allergic reactions to intravenous contrast
+* Febrile illness within 30-days prior to randomization
+* Any absolute contraindication to transesophageal echocardiography
+* Any contraindication to systemic heparinization including active bleeding diatheses, and heparin induced thrombocytopenia
+* Patients with CAD requiring revascularization
+* Any prior mitral valve intervention or any prior repair of atrial septal defect
+* Any prior MV intervention or any prior repair of atrial septal defect
+* Need for any of the following concomitant procedures: aortic valve or aortic surgery, tricuspid valve surgery
+* Need for any emergency intervention or surgery
+* Active endocarditis
+* Hemodynamic instability defined as cardiac index \&lt;2.0 l/min/m2 or systolic blood pressure \&lt;90mmHg or need for inotropic support or any mechanical circulatory support
+* Left ventricular ejection fraction \&lt;25%
+* Intracardiac mass or thrombus
+* Co-morbid medical or oncologic condition for which local heart team believes that survival beyond 2 years is unlikely
+* Active substance abuse
+* Suspected inability to adhere to follow-up
+* Treatment with another investigational drug or other intervention, assessment of which has not completed the primary endpoint or that clinically interferes with the present study endpoints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Study to Evaluate Adverse Events, Change in Disease Activity, and How Oral ABBV-101 Moves Through the Body in Adult Participants With B-Cell Malignancies [NCT05753501]</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* For Dose Escalation (Part 1) only (including backfill): Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have a documented diagnosis for one of the following third line or later B-cell malignancies, from one of the following world health organization (WHO)-defined histologies (Swerdlow et al 2016):
+  * Chronic lymphocytic leukemia (CLL)/small lymphocytic lymphoma (SLL)
+    1. For Dose Escalation (Part 1) backfill only - Bruton's tyrosine kinase inhibitor (BTKi)/Bruton's tyrosine kinase degrader (BTKd)-naïve CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received at least one prior systemic therapy that cannot be a BTK inhibitor or degrader, and, with the exception of BTK pathway agents, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+    2. For Dose Escalation (Part 1) backfill only - BTKi/BCL-2i combination regimen-exposed 2L CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received one prior systemic therapy with a BTKi and BCL-2i combination regimen, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+  * Chimeric antigen receptor T-cells (CAR-T)/hematopoietic cell transplant (HCT) relapsed/refractory (R/R) or ineligible diffuse large b-cell lymphoma (DLBCL) from the following histologies: DLBCL not otherwise specified (NOS) (germinal center B cell \[GCB\] and non-GCB DLBCL), T-cell/histiocyte-rich large B-cell lymphoma, primary mediastinal (thymic) large B-cell lymphoma, intravascular large B-cell lymphoma, anaplastic lymphoma kinase positive (ALK+) large B-cell lymphoma, high-grade B-cell lymphoma with MYC and BCL2 and/or BCL6 rearrangements, and high-grade B-cell lymphoma NOS.
+  * Mantle cell lymphoma (MCL)
+  * Follicular lymphoma \[FL\] (grades 1-3b)
+  * Marginal zone lymphoma \[MZL\] (splenic, extranodal, and nodal)
+  * Waldenström macroglobulinemia (WM)
+  * Transformed indolent non-Hodgkin's lymphoma (iNHL)
+* For Dose Expansion (Part 2a) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment.
+* For Dose Expansion (Part 2a) DLBCL only: Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have documented diagnosis of CAR-T/HCT R/R or ineligible non-GCB DLBCL who are in their third line or later treatment with histology based on criteria established by the WHO.
+* For Dose Exploration of ABBV-101 combination with venetoclax (Part 2b) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment: In safety lead-in for each dose level, participants must have received at least one prior systemic therapy.
+* Has an Eastern Cooperative Oncology Group (ECOG) Performance Status (PS) of 0, 1, or 2. For EU only: Participant has an ECOG PS of 0 or 1.
+* Participant has a life expectancy \&gt;= 12 weeks.
+* Prior Bruton's tyrosine kinase inhibitor (BTKi) is allowed.
+* Adequate hematologic, renal, and hepatic function per the protocol.
+Exclusion Criteria:
+* Previously treated with a Bruton's tyrosine kinase (BTK) degrader.
+* Known active central nervous system (CNS) disease, or primary CNS lymphoma. Participants with prior CNS disease that have been effectively treated may be eligible.
+* Uncontrolled active systemic infection requiring systemic treatment that is ongoing or was completed \&lt;= 14 days before the first dose of study drug, or active cytomegalovirus infection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Safety and Efficacy Study of the Medtronic CoreValve® System in the Treatment of Severe, Symptomatic Aortic Stenosis in Intermediate Risk Subjects Who Need Aortic Valve Replacement (SURTAVI). [NCT01586910]</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: Not specified – Not specified  |  All
+Inclusion Criteria:
+* Subject must have co-morbidities such that Heart Team agrees predicted risk of operative mortality is ≥3% and \&lt;15% at 30 days (Intermediate Clinical Risk classification). Heart team evaluation of clinical surgical mortality risk for each patient includes the calculated STS score for predicted risk of surgical mortality augmented by consideration of the overall clinical status and co-morbidities unmeasured by the STS risk calculation;
+* Heart Team unanimously agree on treatment proposal and eligibility for randomization\* based on their clinical judgement (including anatomy assessment, risk factors, etc.);
+* Subject has severe aortic stenosis presenting with;
+  1. Critical aortic valve area defined as an initial aortic valve area of ≤1.0cm2 or aortic valve area index \&lt; 0.6cm2/m2 AND
+  2. Mean gradient \&gt; 40mmHg or Vmax \&gt; 4m/sec by resting echocardiogram or simultaneous pressure recordings at cardiac catherization \[or with dobutamine stress, if subject has left ventricular ejection fraction (LVEF) \&lt;55%\] or velocity ratio \&lt; 0.25;
+* Subject is symptomatic from his/her aortic valve stenosis, as demonstrated by New York Heart Association (NYHA) Functional Class II or greater;
+* Subject and the treating physician agree that the subject will return for all required post-procedure follow-up visits;
+* Subject meets the legal minimum age to provide informed consent based on local regulatory requirements;
+Exclusion Criteria:
+* Subject has refused surgical aortic valve replacement (SAVR) as a treatment option; (not applicable for Single Arm)
+* Any condition considered a contraindication for placement of a bioprosthetic valve (i.e., subject requires a mechanical valve);
+* A known hypersensitivity or contraindication to all anticoagulation/antiplatelet regimens (or inability to be anticoagulated for the index procedure), nitinol, or sensitivity to contrast media which cannot be adequately pre-medicated;
+* Blood dyscrasias as defined: leukopenia (WBC \&lt;1000mm3), thrombocytopenia (platelet count \&lt;50,000 cells/mm3), history of bleeding diathesis or coagulopathy;
+* Ongoing sepsis, including active endocarditis;
+* Any condition considered a contraindication to extracorporeal assistance;
+* Any percutaneous coronary or peripheral interventional procedure performed within 30 days prior to randomization\* (Subjects with recent placement of drug eluting stent(s) should be assessed for ability to safely proceed with SAVR within the protocol timeframe);
+* Symptomatic carotid or vertebral artery disease or successful treatment of carotid stenosis within six weeks of randomization\*;
+* Cardiogenic shock manifested by low cardiac output, vasopressor dependence, or mechanical hemodynamic support;
+* Recent (within 6 months of randomization\*) cerebrovascular accident (CVA) or transient ischemic attack (TIA);
+* Active gastrointestinal (GI) bleeding that would preclude anticoagulation;
+* Subject refuses a blood transfusion;
+* Severe dementia (resulting in either inability to provide informed consent for the trial/procedure, prevents independent lifestyle outside of a chronic care facility, or will fundamentally complicate rehabilitation from the procedure or compliance with follow-up visits);
+* Multivessel coronary artery disease with a Syntax score \&gt;22 and/or unprotected left main coronary artery (Syntax score calculation is not required for patients with history of previous revascularization if repeat revascularization is not planned);
+* Estimated life expectancy of less than 24 months due to associated non-cardiac comorbid conditions;
+* Other medical, social, or psychological conditions that in the opinion of the Investigator precludes the subject from appropriate consent or adherence to the protocol required follow-up exams;
+* Currently participating in an investigational drug or another device trial (excluding registries);
+* Evidence of an acute myocardial infarction ≤30 days before the index procedure;
+* Need for emergency surgery for any reason;
+* True porcelain aorta (i.e. Heart Team agrees the aorta is not clampable for SAVR);
+* Extensive mediastinal radiation;
+* Liver failure (Child-C);
+* Reduced ventricular function with left ventricular ejection fraction (LVEF) \&lt;20% as measured by resting echocardiogram;
+* Uncontrolled atrial fibrillation (e.g. resting heart rate \&gt; 120 bpm);
+* Pregnancy or intent to become pregnant prior to completion of all protocol follow-up requirements;
+* End stage renal disease requiring chronic dialysis or creatinine clearance \&lt; 20 cc/min;
+* Pulmonary Hypertension (systolic pressure\&gt; 80mmHg);
+* Severe Chronic Obstructive Pulmonary Disease (COPD) demonstrated by Forced Expiratory Volume (FEV1) \&lt; 750cc;
+* Frailty assessments identify:
+  1. Subject is \&lt; 80 years of age and three or more of the following apply
+  2. Subject is ≥ 80 years of age and two or more of the following apply
+     * Wheelchair bound
+     * Resides in an institutional care facility (e.g., nursing home, skilled care center)
+     * Body Mass Index \&lt; 20 kg/m2
+     * Grip Strength \&lt; 16 kg
+     * Katz Index Score ≤ 4
+     * Albumin \&lt; 3.5 g/dL;
+* Marfan syndrome or other known connective tissue disease that would necessitate aortic root replacement/intervention; (Not applicable for Single Arm)
+Note: Additional anatomical and vascular exclusion criteria may apply.
+Note: \* For purposes of the single arm phase of the trial, "randomization" will refer to trial enrollment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Efficacy and Safety of Depemokimab Compared With Mepolizumab in Adults With Relapsing or Refractory Eosinophilic Granulomatosis With Polyangiitis (EGPA) [NCT05263934]</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Participant (male or female) must be 18 years of age or older at the time of signing the informed consent.
+* Participants who are \&gt;=40 kilogram at Screening Visit 1.
+* Participants with a documented diagnosis of EGPA for at least 6 months based on the history or presence of: asthma plus eosinophilia defined as \&gt;1.0\*10\^9/Liter (L) and/or \&gt;10 percentage (%) of leucocytes plus at least 2 of the following additional features of EGPA: a biopsy showing histopathological evidence of eosinophilic vasculitis, or perivascular eosinophilic infiltration, or eosinophil-rich granulomatous inflammation, neuropathy, mono or poly (motor deficit or nerve conduction abnormality), pulmonary infiltrates, non-fixed, sino-nasal abnormality, cardiomyopathy (established by echocardiography or magnetic resonance imaging), glomerulonephritis (hematuria, red cell casts, proteinuria), alveolar hemorrhage (by bronchoalveolar lavage), palpable purpura, anti-neutrophil cytoplasmic antibodies positive Myeloperoxidase or Proteinase 3.
+* History of relapsing OR refractory disease.
+* Participants must be on a stable dose of oral prednisolone or prednisone of \&gt;=7.5 mg/day (but not \&gt;50 mg/day) or equivalent for at least 4 weeks prior to Baseline (Visit 2).
+* If participants receiving immunosuppressive therapy (excluding cyclophosphamide) the dosage must be stable for the 4 weeks prior to Baseline (Visit 2) and during the study.
+* A female participant is eligible to participate if she is not pregnant or breastfeeding, and one of the following conditions applies: Is a woman of non-childbearing potential (WONCBP) OR Is a woman of childbearing potential (WOCBP) and using a contraceptive method that is highly effective, with a failure rate of \&lt;1%.
+* Capable of giving signed informed consent
+Exclusion Criteria:
+* Participants diagnosed with granulomatosis with polyangiitis; previously known as Wegener's granulomatosis or microscopic polyangiitis.
+* Participants with organ-threatening EGPA as per EULAR criteria,
+* Imminently life-threatening EGPA disease within 3 months prior to Screening (Visit 1).
+* A current malignancy or previous history of cancer in remission for less than 12 months prior to Screening.
+* Participants with alanine aminotransferase \&gt;2\*upper limit of normal (ULN) or if participant is on background methotrexate or azathioprine \&gt;3\*ULN, aspartate aminotransferase \&gt;2\*ULN or if participant is on background methotrexate or azathioprine \&gt;3\*ULN, alkaline phosphatase \&gt;=2.0\*ULN, total bilirubin \&gt;1.5\*ULN (isolated bilirubin \&gt;1.5\*ULN is acceptable if bilirubin is fractionated and direct bilirubin \&lt;35%), Cirrhosis or current unstable liver or biliary disease per investigator assessment.
+* Participants who have severe or clinically significant cardiovascular disease uncontrolled with standard treatment.
+* Participants who have known, pre-existing, clinically significant system abnormalities that are not associated with EGPA and are uncontrolled with standard treatment.
+* Clinically significant abnormality in the hematological, biochemical or urinalysis screen at Visit 1.
+* Chronic or ongoing active infectious disease requiring systemic treatment.
+* Participants with a known, pre-existing parasitic infestation within 6 months prior to Screening Visit 1.
+* A known immunodeficiency (e.g., human immunodeficiency virus \[HIV\]).
+* Participants that, according to the investigator's medical judgment, are likely to have active coronavirus disease 2019 (COVID-19) infection. Participants with known COVID-19 positive contacts within the past 14 days must be excluded for at least 14 days following the exposure during which the participant must remain symptom-free.
+* Participants with a known allergy or intolerance to a monoclonal antibody or biologic therapy or any of the excipients of the investigational products.
+* Participants who have a previous documented failure with anti-Interleukin-5 /Interleukin-5 receptor therapy (e.g., mepolizumab, reslizumab, benralizumab). Participants who have received monoclonal antibodies (mAb) and who have not undergone the required washout periods, prior to Visit 1.
+* Participants receiving any of the following: Oral corticosteroids: Participant requires an oral corticosteroid dose of \&gt;50 mg/day prednisolone/prednisone in the 4-week period prior to Baseline (Visit 2), Intravenous (IV), intramuscular or subcutaneous (SC) corticosteroids in the 4-week period prior to Baseline (Visit 2), Omalizumab within 130 days prior to Screening (Visit 1), Cyclophosphamide (CYC): oral CYC within 4 weeks prior to Baseline (Visit 2) and IV CYC within 3 weeks prior to Baseline (Visit 2), if their total white blood cells is \&gt;=4\*10\^9/L (measured using the local laboratory if necessary), Rituximab within 12 months prior to Screening (Visit 1); in addition, the Participant must have shown recovery of peripheral B-cell count to within the normal range, Tezepelumab and Dupilumab with a washout period of 5 half-lives prior to Screening Visit 1, IV or SC immunoglobulin within 6 months prior to Screening (Visit 1); For China and Japan only within 12 weeks prior to Screening (Visit 1), Interferon-alpha within 6 months prior to Screening Visit 1, Anti-tumor necrosis factor therapy within 12 weeks prior to Screening Visit 1, Anti-CD52 (alemtuzumab) within 6 months prior to Screening Visit 1.
+* Participants with QT interval corrected for heart rate according to Fridericia's formula (QTcF) \&gt;=450 milliseconds (msec) or QTcF \&gt;=480 msec for participants with Bundle Branch Block in the 12-lead ECG central over-read from at Screening Visit 1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1178,12 +1887,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun 13:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>EASi-PROTKT™ - A Study to Test Vicadrostat (BI 690517) Taken Together With Empagliflozin in People With Type 2 Diabetes, High Blood Pressure, and Cardiovascular Disease [NCT07064473]</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria :
+* At least 18 years old at time of consent
+* Signed and dated written informed consent in accordance with ICH-GCP and local legislation prior to admission to the trial
+* Women of childbearing potential (WOCBP) must be ready and able to use highly effective methods of birth control per ICH M3 (R2).
+* Participants with medical history of hypertension and on active pharmacological treatment
+* Participants with medical history of type 2 diabetes mellitus (T2DM) and on active pharmacological treatment
+* Established cardiovascular (CV) disease and on active pharmacological treatment
+* At least one additional risk factor for developing heart failure (HF)
+Exclusion Criteria:
+* History of HF or hospitalization for HF or treatment of HF
+* Atrial fibrillation or Atrial flutter with a resting heart rate \&gt;110 beats per minute (bpm) documented by echocardiogram (ECG) at Visit 1 (screening)
+* Advanced untreated conduction disease or untreated clinically relevant ventricular arrhythmia at Visit 1 (screening)
+* Treatment with an Mineralocorticoid receptor antagonist (MRA)
+* Treatment with amiloride or other potassium-sparing diuretic
+* Receiving the following treatments at Visit 1 (screening) or requiring such treatment before Visit 2 (randomisation), or planned during the trial:
+  * A direct renin inhibitor (e.g. aliskiren)
+  * More than one Angiotensin-converting enzyme inhibitor (ACEi) and/or Angiotensin receptor blocker (ARB) (including Angiotensin receptor-neprilysin inhibitor (ARNi)) used simultaneously
+  * Other aldosterone synthase inhibitors (e.g. baxdrostat)
+  * Systemic mineralocorticoid replacement therapy (e.g. fludrocortisone) Further exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Monitor update 2026-06-25 12:37 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B22"/>
+  <dimension ref="A3:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1489,6 +1489,407 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>First-Time-in-Human Study of GSK4381562 in Participants With Advanced Solid Tumors [NCT05277051]</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion criteria:
+* A female participant is eligible to participate if she is not pregnant or breastfeeding, and at least 1 of the following conditions applies:
+  * Is not a woman of childbearing potential (WOCBP) or
+  * Is a WOCBP and using a contraceptive method that is highly effective with a failure rate of less than (\&lt;)1 percent (\[%\] per year), during the intervention period and for specified time after end of study treatment.
+  * A WOCBP must have a negative highly sensitive pregnancy test within 24-48 hours before the first dose of study intervention.
+  * Requirement for Arm I only: Male participants agree to use contraception and for their female partner to use contraception, if applicable.
+* Histological or cytological documentation of loco-regionally recurrent solid tumors where curative treatment options have been exhausted, or metastatic solid tumors; types as follows:
+  * head and neck squamous cell carcinoma (HNSCC)
+  * non-small-cell lung cancer (NSCLC)
+  * breast cancer (BC)
+  * clear cell renal cell cancer (ccRCC)
+  * gastric cancer (GC)
+  * colorectal cancer (CRC)
+  * endometrial cancer (EC)
+  * epithelial ovarian, fallopian tube, and primary peritoneal cancers- Disease that has progressed after standard therapy for the specific tumor type, or for which standard therapy has proven to be ineffective, intolerable, or is considered inappropriate, or if no further standard therapy exists.
+  * Measurable disease per RECIST 1.1.
+* Eastern Cooperative Oncology Group (ECOG) performance status (PS) 0-1.
+* Life expectancy of at least 12 weeks.
+* Adequate organ function, as defined in the protocol.
+* For participants enrolled in a PK/PD cohort, participant agrees to a fresh tumor biopsy during Screening and at approximately 6-weeks after treatment initiation.
+Exclusion Criteria:
+* Prior treatment with the following therapies (specified time periods are from last dose of prior treatment to first dose of study intervention):
+  * Any therapy directed against Polio virus receptor (PVR)-related immunoglobulin domain-containing (PVRIG) (COM701 or other anti-PVRIG monoclonal antibody \[mAb\]) or other cluster of differentiation (CD)226 axis receptor (T-cell immunoglobulin and immunoreceptor tyrosine-based inhibition motif domain \[TIGIT\] or CD96) at any time.
+  * For Arm I only, prior treatment with orlotamab, enoblituzumab, I-Dxd, or other B7-H3 targeted agents.
+  * Other prior immunotherapy, chemotherapy, targeted therapy, biological therapy or radiation therapy within specified periods as defined in the protocol.
+  * Investigational therapy: if the participant has participated in a clinical study and has received an investigational product within 4 weeks or 5 half-lives of the investigational product (whichever is shorter).
+* Prior allogenic or autologous bone marrow transplantation or other solid organ transplantation.
+* Toxicity from previous anticancer treatment, including:
+  * Greater than or equal to Grade 3 immune-mediated toxicity considered related to prior immunotherapy and that led to treatment discontinuation; or
+  * History of myocarditis of any grade during a previous treatment with immunotherapy
+  * Toxicity related to prior treatment that has not resolved to less than or equal to (\&lt;=) Grade 1. Non clinically relevant Grade 2 toxicities, not constituting a safety risk by investigator judgment are allowed.
+* Participant has a known additional malignancy that progressed or required active treatment within the last 2 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>ROSETTA Breast-01: The Effects and Safety of Pumitamig in Patients With Triple-Negative Breast Cancer [NCT07173751]</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Are considered ineligible for combination treatment with a monospecific PD(L)1 targeting immunotherapy plus chemotherapy as per their tumor PD-L1 expression status.
+* Have confirmed locally recurrent inoperable or metastatic TNBC, or estrogen receptor (ER)-low, human epidermal growth factor receptor 2 (HER2)-negative breast cancer (ER and/or progesterone receptor \[PgR\]) 1% to 10%, HER2 immunohistochemistry \[IHC\] 0, 1+, or 2+ with fluorescence in situ hybridization \[FISH\] negative for HER2 gene amplification) documented prior to trial screening as part of standard of care.
+* Have at least one measurable lesion as the targeted lesion based on RECIST v1.1.
+* Have provided a tissue sample, archival or fresh, during the screening period (bone biopsies, fine needle aspiration biopsies, and samples from pleural or peritoneal fluid are not acceptable; participants with only one target lesion are not eligible to participate in the trial).
+* Eastern cooperative oncology group (ECOG) performance status of 0 or 1.
+Exclusion Criteria:
+* Have received any of the following therapies or drugs prior to the initiation of trial:
+  * Have received prior systemic anticancer therapy for advanced disease.
+  * Have received prior treatment with a PD(L)-1/vascular endothelial growth factor (VEGF) bispecific antibody.
+  * Have received systemic corticosteroids (at a dosage greater than 10 milligrams \[mg\]/day of prednisone or an equivalent dose of other corticosteroids) within 7 days prior to the initiation of trial treatment. Exception: excluding local, intranasal, intraocular, intra-articular or inhaled corticosteroids, short-term use (\&lt;= 7 days) of corticosteroids for prophylaxis (for example, prevention of contrast agent allergy) or treatment of non-autoimmune conditions (for example, delayed hypersensitivity reactions caused by exposure to allergens).
+  * Have been vaccinated with live attenuated vaccine(s) within 4 weeks prior to initiation of trial treatment.
+  * Have received broad-spectrum intravenous antibiotics therapy within 2 weeks prior to initiation of trial treatment.
+* Are pregnant or breastfeeding or are planning pregnancy or planning to father children during the trial or within 6 months after the last dose of pumitamig or placebo.
+* Have undergone major organ surgery, significant trauma, or invasive dental procedures (such as dental implants) within 28 days prior to the initiation of trial treatment or plan to undergo elective surgery during the trial. Placement of vascular infusion devices is allowed.
+* Have received allogeneic hematopoietic stem cell transplantation or organ transplantation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>An Adjuvant Endocrine-based Therapy Study of Camizestrant (AZD9833) in ER+/HER2- Early Breast Cancer (CAMBRIA-2) [NCT05952557]</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 130 Years  |  All
+Inclusion Criteria:
+* Women and Men; ≥18 years at the time of screening (or per national guidelines)
+* Histologically confirmed ER+/HER2- early-stage resected invasive breast cancer with absence of any evidence of metastatic disease as defined in the protocol.
+* Completed adequate (definitive) locoregional therapy (surgery with or without radiotherapy) for the primary breast tumour(s), with or without (neo)adjuvant chemotherapy.
+* Patients must be randomised within 12 months of definitive breast surgery.
+* Patients may have received up to 12 weeks of endocrine therapy prior to randomisation.
+* Eastern Cooperative Oncology Group (ECOG) performance status of ≤ 1
+* Adequate organ and bone marrow function
+Exclusion Criteria:
+* Inoperable locally advanced or metastatic breast cancer
+* Pathological complete response following treatment with neoadjuvant therapy
+* History of any other cancer (except non-melanoma skin cancer or carcinoma in situ of the cervix or considered a very low risk of recurrence per investigator judgement) unless in complete remission with no therapy for a minimum of 5 years from the date of randomisation
+* Any evidence of severe or uncontrolled systemic diseases which, in the investigator's opinion precludes participation in the study or compliance "
+* Known LVEF \&lt;50% with heart failure NYHA Grade ≥2.
+* Mean resting QTcF interval \&gt; 480 ms at screening
+* Concurrent exogenous reproductive hormone therapy or non topical hormonal therapy for non-cancer-related conditions
+* Any concurrent anti-cancer treatment not specified in the protocol with the exception of bisphosphonates (e.g. zoledronic acid) or RANKL inhibitors ( eg, denosumab)
+* Previous treatment with camizestrant, investigational SERDs/investigational ER targeting agents, or fulvestrant
+* Currently pregnant (confirmed with positive serum pregnancy test) or breastfeeding.
+* Patients with known hypersensitivity to active or inactive excipients of camizestrant or drugs with a similar chemical structure or class to camizestrant. In pre-/peri-menopausal female and male patients, known hypersensitivity or intolerance to LHRH agonists that would preclude the patient from receiving any LHRH agonist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>AMG 410 Alone and in Combination With Other Agents in Participants With KRAS Altered Advanced or Metastatic Solid Tumors [NCT07094113]</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Age ≥ 18 years (or \&gt; legal age within the country if it is older than 18 years).
+2. Pathologically documented, locally-advanced or metastatic malignancy with any missense mutation in the KRAS gene or evidence of KRAS amplification using an analytically validated KRASWT amplification assay.
+3. Participants must have no standard of care treatment options or have actively refused such therapy.
+4. Able to swallow and retain per oral administered study treatment.
+5. Eastern Cooperative Oncology Group (ECOG) Performance Status of 0 or 1.
+6. Disease measurable as defined by Response Evaluation Criteria in Solid Tumors Version 1.1 (RECIST v1.1), as determined by the site investigator.
+7. Adequate organ function.
+8. Archival (formalin-fixed, paraffin-embedded \[FFPE\]) tumor tissue or block collected within 5 years before screening must be available. Participants without archived tumor tissue may undergo tumor biopsy before AMG 410 dosing (Day1).
+Exclusion Criteria:
+1. Untreated symptomatic central nervous system or leptomeningeal metastases.
+2. Uncontrolled pleural effusion and/or ascites.
+3. History of other malignancy within the past 5 years.
+4. Active systemic infection or symptoms that indicate an acute and/or uncontrolled infection requiring IV antibiotics within 7days prior to the first dose of study treatment.
+5. History of arterial or venous thrombosis (eg, stroke, transient ischemic attack, pulmonary embolism, or deep vein thrombosis).
+6. Live and live-attenuated vaccines are prohibited within 28 days prior to the first dose of study treatment.
+7. History of solid organ transplant.
+8. Anti-tumor therapy (chemotherapy, antibody therapy, molecular targeted therapy, hormonal therapy, or investigational agent) within 28 days of first dose of study treatment.
+9. Presence or history of any of the following viral infections: HIV, Hepatitis C, Hepatitis B, and active severe acute respiratory syndrome coronavirus 2 (SARS-CoV-2).
+10. Toxicities from prior anti-tumor therapy (including radiotherapy) not having improved to at least Common Terminology Criteria for Adverse Events (CTCAE) version 5.0 grade 1.
+11. Therapeutic or palliative radiation therapy within 2 weeks of first dose of study treatment.
+12. Major surgery within 28 days of first dose of study treatment.
+13. History or evidence of any other clinically significant disorder, condition, or disease that, in the opinion of the investigator, would pose a risk to participant safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>A Study of Xaluritamig Plus Abiraterone Versus Investigator's Choice in Participants With Chemotherapy-naïve Metastatic Castration-resistant Prostate Cancer [NCT07213674]</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  Male
+Inclusion Criteria:
+* Participant has provided informed consent before initiation of any study-specific activities/procedures.
+* Age ≥ 18 years (or ≥ legal age within the country if it is older than 18 years) at the time of signing the informed consent.
+* Participant must have histological, pathological, and/or cytological confirmation of adenocarcinoma of the prostate. Mixed histologies (eg, adenocarcinoma with neuroendocrine component) are not permitted.
+* Metastatic castration-resistant prostate cancer (mCRPC) with ≥ 1 metastatic lesion that is present on baseline computed tomography (CT), magnetic resonance imaging (MRI), or bone scan imaging obtained within 28 days before enrollment.
+* Evidence of progressive disease (PD), defined as 1 or more PCWG3-modified RECIST 1.1 criteria:
+  * Serum PSA progression is defined as 2 consecutive increases in PSA over a previous reference value measured at least 1 week prior. The minimum start value is 2.0 ng/mL.
+  * Soft-tissue progression defined as an increase ≥ 20% in the sum of the diameter (SOD) (short axis for nodal lesions and long axis for non-nodal lesions) of all target lesions based on the smallest SOD since treatment started or the appearance of 1 or more new lesions or unequivocal progression of existing non-target lesions.
+  * Progression of bone disease defined by the appearance of at least 2 new bone lesions(s) by bone scan (as per the 2+2 PCWG3-modified RECIST 1.1 criteria).
+* Participants must have had prior orchiectomy and/or ongoing androgen-deprivation therapy (ADT) and a castrate level of serum testosterone (\&lt; 50 ng/dL or \&lt; 1.7 nmol/L).
+* Prior disease progression on 1, and only 1, androgen receptor pathway inhibitor (ARPI) (either enzalutamide, apalutamide, or darolutamide) is required.
+* Participants intended to receive cabazitaxel must have previously received ≤ 6 cycles of docetaxel in the metastatic hormone-sensitive prostate cancer (mHSPC) setting.
+* Eastern Cooperative Oncology Group (ECOG) performance status (PS) of 0 or 1.
+* Adequate organ function.
+Exclusion Criteria:
+Disease Related:
+* Participants with a history of central nervous system (CNS) metastases.
+* Unresolved toxicities from prior antitumor therapy not having resolved to CTCAE version 5.0 grade 1 or baseline, with the exception of alopecia or toxicities that are stable and well-controlled AND there is an agreement to allow inclusion by both the investigator and the sponsor.
+Prior/Concomitant Therapy:
+* Prior six transmembrane epithelial antigen of the prostate 1 (STEAP1)-targeted therapy.
+* Prior disease progression on or intolerance to abiraterone.
+* Prior treatment with any chemotherapy regimen in the mCRPC setting and/or \&gt; 6 cycles of docetaxel treatment in the mHSPC setting.
+* Any anticancer therapy, immunotherapy, or investigational agent within 4 weeks before first dose of study treatment with the following exceptions:
+  * Androgen receptor pathway inhibitors (ARPIs; enzalutamide, darolutamide, apalutamide): minimum washout of 2 weeks prior to the first dose of study treatment.
+  * Androgen suppression therapy (eg, luteinizing hormone-releasing hormone/gonadotrophin releasing hormone \[LHRH/GnRH\] analogue \[agonist/antagonist\]) is permitted.
+* Prior radioligand therapy (RLT) within 8 weeks of first dose of study treatment.
+* Prior radionuclide therapy (radium-223) within 2 months of first dose of study treatment.
+* Prior palliative radiotherapy within 2 weeks before first dose of study treatment. Participants must have recovered from all radiation-related toxicities.
+* Concurrent cytotoxic chemotherapy, ARPI, immunotherapy, RLT, poly adenosine diphosphate ribose polymerase (PARP) inhibitor, biological therapy, investigational therapy.
+* Treatment with live and live-attenuated vaccines within 4 weeks before the first dose of study treatment.
+* Prior CD3-directed therapy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Study of Vimseltinib (DCC-3014) in Patients With Advanced Tumors and Tenosynovial Giant Cell Tumor [NCT03069469]</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+Dose Escalation Phase:
+1. Patients ≥18 years of age
+2. Patients must have:
+   1. advanced malignant solid tumors; or
+   2. symptomatic TGCT for which surgical resection is not an option (tumor biopsy to confirm diagnosis required if no histology/pathology available at screening)
+3. Malignant solid tumor patients only: Able to provide a tumor tissue sample
+4. Must have 1 measurable lesion according to RECIST Version 1.1
+5. Malignant solid tumor patients only: Must have Eastern Cooperative Oncology Group (ECOG) performance status of 0-1
+6. Adequate organ and bone marrow function
+7. If a female of childbearing potential, must have a negative pregnancy test prior to enrollment and agree to follow the contraception requirements.
+8. Must provide signed consent to participate in the study and is willing to comply with study-specific procedures.
+Expansion Phase (Cohorts A and B)
+1. Patients ≥18 years of age
+2. Patients must have symptomatic TGCT for which surgical resection is not an option (tumor biopsy to confirm diagnosis required if no histology/pathology available at screening)
+   a) Expansion Cohort B: patients must have prior systemic treatment with anti-CSF1 or anti-CSF1R therapy, with the exception of imatinib or nilotinib
+3. Adequate organ and bone marrow function
+4. Must have at least 1 measurable lesion according to RECIST Version 1.1
+5. If a female of childbearing potential, must have a negative pregnancy test prior to enrollment and agree to follow the contraception requirements.
+6. Must provide signed consent to participate in the study and is willing to comply with study-specific procedures.
+Exclusion Criteria
+Dose Escalation Phase:
+1. Received anticancer therapy or therapy for TGCT, including investigational therapy, within 2 weeks or 28 days for therapies with half-life (t1/2) longer than 3 days prior to the administration of study drug.
+2. Unresolved toxicity (Grade \&gt;1 or baseline) from previous anticancer therapy or TGCT therapy, excluding alopecia.
+3. Known active central nervous system (CNS) metastases.
+4. History or presence of clinically relevant cardiovascular abnormalities.
+5. Systemic arterial or venous thrombotic or embolic events.
+6. QT interval corrected by Fridericia's formula (QTcF) \&gt;450 ms in males or \&gt;470 ms in females or history of long QT syndrome.
+7. Left ventricular ejection fraction (LVEF) \&lt;50%.
+8. Concurrent treatment with proton-pump inhibitor(s).
+9. Major surgery within 2 weeks of the first dose of study drug.
+10. Malabsorption syndrome or other illness that could affect oral absorption.
+11. Known human immunodeficiency virus, active hepatitis B, active hepatitis C, or active mycobacterium tuberculosis infection.
+12. If female, the patient is pregnant or lactating.
+13. Known allergy or hypersensitivity to any component of the study drug.
+14. Any other clinically significant comorbidities.
+Expansion Phase (Cohorts A and B)
+1. Expansion Cohort A: received systemic therapy targeting CSF1 or CSF1R; previous therapy with imatinib and nilotinib is allowed.
+2. Expansion Cohort B: discontinued systemic therapy targeting anti-CSF1 or anti-CSF1R due to drug-induced liver injury.
+3. Treatment with therapy for TGCT, including investigational therapy, within 2 weeks or 28 days for therapies with a t1/2 longer than 3 days prior to the administration of the study drug.
+4. Known metastatic TGCT or other active cancer that requires concurrent treatment.
+5. QT interval corrected by Fridericia's formula (QTcF) \&gt;450 ms in males or \&gt;470 ms in females or history of long QT syndrome.
+6. Left ventricular ejection fraction (LVEF) \&lt;55%.
+7. Concurrent treatment with proton-pump inhibitor(s).
+8. Major surgery within 2 weeks of the first dose of study drug.
+9. Any clinically significant comorbidities
+10. Malabsorption syndrome or other illness that could affect oral absorption.
+11. Known human immunodeficiency virus (HIV), active or chronic hepatitis B, active or chronic hepatitis C, or active mycobacterium tuberculosis infection.
+12. If female, the patient is pregnant or lactating.
+13. Known allergy or hypersensitivity to any component of the study drug.
+14. Contraindication for MRI
+15. Active liver or biliary disease, including evidence of fatty liver, nonalcoholic steatohepatitis (NASH), or cirrhosis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Carcinoid Syndrome Efficacy Study Featuring an Oral Daily Paltusotine Regimen [NCT07087054]</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Male or female ≥18 years of age, at the time of Screening.
+* Willing and able to comply with the study procedures as specified in the protocol, including at least 70% compliance with the study diary for the 2-week period.
+* Documented carcinoid syndrome requiring medical therapy. Participants must exhibit symptoms of flushing with or without frequent BMs as follows:
+  * For participants who are naïve/not currently treated with somatostatin receptors ligands (SRL), they must exhibit an average of \&gt;1 flushing episode/day over a period of 14 days
+  * For participants who will wash out from SRL treatment, they must be symptomatically controlled and exhibit an increase in daily average flushing episodes and an average of \&gt;1 flushing episode/day over a period of 14 days during the Washout Period.
+* Evaluable documentation of locally advanced or metastatic histopathologically confirmed well-differentiated neuroendocrine tumor(s) \[NETs\].
+* No significant disease progression as assessed by the Investigator within the last 6 months before randomization.
+Exclusion Criteria:
+* Diarrhea attributed to any condition(s) other than carcinoid syndrome.
+* Uncontrolled/severe diarrhea associated with significant volume contraction, dehydration, or hypotension.
+* Requires second line treatments (eg, telotristat) for control of carcinoid syndrome symptoms in the opinion of the Investigator.
+* Treatment with specific NET therapy \&lt;4 weeks before Screening (such as everolimus or sunitinib) or hepatic embolization, radiotherapy, peptide receptor radionuclide therapy (PRRT), and/or tumor debulking \&lt;12 weeks before Screening.
+* Major surgery within 8 weeks before Screening.
+* History of another primary malignancy \&lt;3 years prior to the date of randomization, except for adequately treated basal or squamous cell carcinoma of the skin, cancer of the breast has been completely locally excised and carcinoma in situ of the cervix has also been resected, previously treated malignancy, if all treatment for that malignancy was completed at least 3 years prior to first dose of study treatment, and no current evidence of disease, concurrent malignancy determined to be clinically stable and not requiring treatment.
+* Diabetes mellitus treated with insulin for less than 6 weeks prior to the study entry.
+* Poorly controlled diabetes mellitus defined as having a hemoglobin A1c (HbA1c) ≥8.5%
+* Unable to administer short-acting (SA) octreotide (octreotide acetate injection), or prior nonresponse documented with somatostatin agonists.
+* Clinically significant concomitant disease or indicator of disease that is not a result of the primary disease under study, including but not limited to cardiovascular disease, estimated glomerular filtration rate 2×upper limit of normal \[ULN\], and/or total bilirubin (TB) \&gt;1.5×ULN. (Participants with previously diagnosed Gilbert's syndrome not accompanied by other hepatobiliary disorders and associated with TB
+* Alcohol or drug abuse is not permitted at any time during the study
+* Diagnosed with symptomatic cholelithiasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Rollover Study to Provide Continued Treatment for Participants With B-Cell Malignancies Previously Enrolled in Studies of Parsaclisib (INCB050465) [NCT04509700]</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Currently enrolled and receiving treatment in an Incyte-sponsored clinical study of parsaclisib.
+* Currently tolerating treatment in the parent Protocol.
+* Currently receiving clinical benefit from treatment with parsaclisib as monotherapy or in combination therapy with Itacitinib, ruxolitinib, or ibrutinib as determined by the investigator.
+* Has at least stable disease, as determined by the investigator.
+* Has demonstrated compliance, as assessed by the investigator, with the parent Protocol requirements.
+* Willingness and ability to comply with scheduled visits, treatment plans, including PJP prophylaxis, and any other study procedures indicated in this Protocol.
+* Willingness to avoid pregnancy or fathering children
+* Ability to comprehend and willingness to sign an ICF
+Exclusion Criteria:
+* Has been permanently discontinued from study treatment in the parent Protocol for any reason.
+* Able to access parsaclisib as monotherapy or in combination with itacitinib, ruxolitinib, or ibrutinib therapy outside a clinical study.
+* Participants with an uncontrolled intercurrent illness or any concurrent condition that, in the investigator's opinion, would jeopardize the safety of the participant or compliance with the Protocol.
+* Pregnant or breastfeeding women.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1500,7 +1901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B22"/>
+  <dimension ref="A3:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1876,6 +2277,354 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PLatform Study for INTracerebral Haemorrhage (PLINTH): Community-based Feasibility Study [NCT06078020]</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* People aged ≥18 years at the time of diagnosis with symptomatic stroke due to first-ever or recurrent spontaneous (non-traumatic) ICH, most likely to be due to cerebral small vessel disease, confirmed by brain imaging between 1 October 2023 and 30 June 2025 inclusive
+* One or more management uncertainties exist about the patient's management according to the patient/nearest relative and their responsible clinician
+* Patient or their nearest relative can be approached for consent to participation in this feasibility study with the aid of simple information delivered by Tailored Talks
+* Residential postcode in the National Health Service (NHS) Lothian or NHS Lanarkshire regions of Scotland
+Exclusion Criteria:
+* People aged \&lt;18 years at the time of ICH diagnosis
+* Exclusively extra-axial intracranial haemorrhage or ICH definitely attributable to a macrovascular cause (e.g. aneurysm, arteriovenous malformation, cavernoma, cerebral venous sinus thrombosis), tumour, trauma or haemorrhagic transformation of an ischaemic stroke
+* Responsible clinician deems it inappropriate to approach the patient or their nearest relative (e.g. death appears imminent)
+* Mental incapacity and no nearest relative, welfare attorney or welfare guardian available at the time of approach
+* Patient died before approached for consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Convergent Ablation Plus Left Atrial Appendage Isolation for the Treatment of Persistent Atrial Fibrillation [NCT06165510]</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 80 Years  |  All
+Inclusion Criteria:
+* Age \&gt; 18 years; \&lt; 80 years
+* Persistent AF \&gt; 1-year duration
+* Left atrium size \&lt; 6cm
+* Pts should be able to provide written informed consent.
+Exclusion Criteria:
+* Subjects currently enrolled in another investigational study except in case of observational registry with no associated treatments.
+* Subject has a reversible cause of AF or transient AF
+* Subject is absent of LAA or if the LAA is previously surgically ligated
+* Subject has had previous cardiac surgery or abdominal surgery.
+* Subject has contraindication to anticoagulation.
+* Patients with hypertrophic cardiomyopathy.
+* Patients with significant valve disease.
+* Subject has had previous catheter or surgical ablation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>REdo Transcatheter Aortic VALVE Implantation for the Management of Transcatheter Aortic Valve Failure [NCT06557798]</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1\. Bio-prosthetic Valve Failure (BVF) of a Transcatheter Aortic Valve requiring possible reintervention
+Exclusion Criteria:
+1. Bio-prosthetic Valve Failure due solely to paravalvular aortic regurgitation
+2. Active endocarditis
+3. Untreated acute valve thrombosis
+4. Life-expectancy less than 1 year
+5. Subject is less than legal age of consent, legally incompetent, or otherwise vulnerable
+6. Pregnant or nursing</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>A Randomised, Controlled Trial of a Low-energy Diet for Improving Functional Status in Heart Failure With PRESERVED Ejection Fraction Preserved Ejection Fraction [NCT05887271]</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Established clinical diagnosis of heart failure with preserved ejection fraction HFpEF (EF\&gt;45%) made by a cardiologist or a primary care physician with heart failure expertise, or a heart failure nurse
+2. Clinically stable for ≥ 3 months (no admissions to hospital)
+3. Obesity (BMI ≥30kg/m2 if white European or ≥27kg/m2 if Asian, Middle Eastern or Black ethnicity)
+4. Age ≥18
+Exclusion Criteria:
+1. Inability to walk/undertake 6-minute walk test
+2. Inability to follow a low-energy MRP
+3. HFpEF due to infiltrative cardiomyopathy (cardiac amyloidosis or sarcoidosis), genetic hypertrophic cardiomyopathy, restrictive cardiomyopathy/pericardial disease or congenital heart disease.
+4. Recovered EF (previous EF \&lt; 40%) unless reduced EF was in context of tachycardia induced cardiomyopathy (eg AF/Aflutter).
+5. Known heritable, idiopathic or drug-induced pulmonary arterial hypertension
+6. Severe chronic obstructive pulmonary disease (FEV1\&lt; 1.0L)
+7. Severe primary valvular heart disease
+8. Anaemia (Hb\&lt;100g/L)
+9. Severe renal disease (eGFR \&lt; 30 ml/min/1.73 m2)
+10. Weight loss \&gt; 5kg in preceding 3 months.
+11. Symptomatic gallstones (including biliary colic) or cholecystitis within last 3 months
+12. Active substance abuse (drugs or alcohol)
+13. History of bariatric surgery in the last 3 years
+14. Active illness likely to cause change in weight
+15. Women who are pregnant or are considering pregnancy
+16. People currently participating in another clinical research trial that is likely to affect diet or weight change.
+17. History of a severe mental illness including an eating disorder
+17\. Individuals with a diagnosis of Type 1 diabetes mellitus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Perivenous Dexamethasone Therapy: Examining Reduction of Inflammation After Thrombus Removal to Yield Benefit in Subacute and Chronic Iliofemoral DVT [NCT04858776]</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 89 Years  |  All
+Inclusion Criteria:
+1. Provision of signed and dated informed consent form prior to receiving any non-standard of care, protocol-specific procedures.
+2. Stated willingness to comply with all study procedures including completion of questionnaires and follow-up visits and availability for the duration of the study.
+3. Male or female, aged 18 to 89 years.
+4. For females of reproductive potential: negative pregnancy test ≤7 days before the procedure, use of highly effective contraception for at least 1 month prior to screening, and agreement to use such a method during study participation.
+5. Negative COVID-19 test result within 5 days prior to procedure or evidence of COVID-19 vaccine or booster within past 12 months.
+6. Onset of DVT symptoms 14 to 60 days prior to intervention in the study limb with need for stenting of the iliofemoral segment.
+7. Ability to take oral medication and be willing to adhere to the prescribed anti-coagulant regimen.
+8. Prescription for at least 14 days low molecular weight heparin followed by therapeutic anticoagulant of investigator's choice for 12-month minimum as part of post-interventional medication regimen.
+9. Minimum of 30 days of prescribed antiplatelet agent (aspirin or P2Y12 inhibitor).
+10. Hemodynamically significant DVT (\&gt;50% area obstruction) spanning at least (a) the iliofemoral and common femoral veins or (b) the common femoral vein with extension into the femoral vein and/or profunda vein. Extent of thrombus in the popliteal and calf veins is allowed.
+11. Successful recanalization of the target vein with at least one patent inflow vein (femoral or profunda).
+Exclusion Criteria:
+1. Current enrollment in another non-registry clinical study of systemic drug therapy or another device study that has not completed its primary endpoint, including prior enrollment in this study. Concurrent enrollment in registry studies of approved devices or drugs are acceptable.
+2. Lack of capability of understanding the nature, significance and implications of the clinical trial.
+3. Body Mass Index \&gt; 40 kg/m2.
+4. Non-ambulatory status prior to DVT occurrence.
+5. In the target vein segment: previously treated symptomatic DVT within the previous 12 months.
+6. In the contralateral (non-study) leg: symptomatic DVT that, in the opinion of the operating physician, will require surgery in the following 30 days.
+7. Limb-threatening circulatory compromise with ankle-brachial index \&lt;0.4, absolute ankle pressure \&lt;50 mmHg or absolute toe pressure \&lt;30 mmHg.
+8. Pulmonary embolism (PE) defined as either massive (Systolic blood pressure \&lt; 90 mmHg and/or patient on IV vasoactive medication to support blood pressure), or intermediate high-risk PE, as defined by the European Society Guideline on management of PE. Low-risk PE and/or intermediate low-risk PE can be enrolled.
+9. Inability to tolerate contemporary venous intervention procedure due to severe dyspnea or acute systemic illness.
+10. Allergy, hypersensitivity, or thrombocytopenia from heparin, Recombinant tissue plasminogen activator (rtPA), dexamethasone sodium phosphate or iodinated contrast, except for mild-moderate contrast allergies for which steroid pre-medication can be used.
+11. History of, or active heparin-induced thrombocytopenia (HIT).
+12. Haemoglobin \&lt; 9.0 mg/dl, INR \&gt; 1.6 before starting anticoagulation, or platelets \&lt; 100,000/ml. Moderate renal impairment in diabetic patients (estimated glomerular filtration rate \&lt; 60 ml/min) or severe renal impairment in non-diabetic patients (estimated glomerular filtration rate \&lt; 30 ml/min).
+13. Active bleeding, recent (\&lt; 3 mo) GI bleeding, severe liver dysfunction, bleeding diathesis.
+14. Recent (\&lt; 3 mo) internal eye surgery or haemorrhagic retinopathy; recent (\&lt; 10 days) major surgery, cataract surgery, trauma, cardiopulmonary resuscitation, obstetrical delivery, or other invasive procedure.
+15. History of hemorrhagic stroke or intracranial/intraspinal bleed, tumor, vascular malformation, aneurysm.
+16. Active cancer with a life expectancy of \&lt;2 years.
+17. Severe hypertension on repeated readings (systolic blood pressure \&gt; 180 mmHg or diastolic blood pressure \&gt; 105 mmHg). This can be treated, and blood pressure must be stable before venous access is obtained (systolic blood pressure \&lt;140 mmHg).
+18. Pregnant or breastfeeding.
+19. Life expectancy \&lt; 2 years.
+20. Thrombus of the inferior vena cava (IVC) extending at least one centimeter above the common iliac confluence.
+21. Inability to obtain venous access.
+22. Inability to recanalize the target vein segment(s).
+23. History of ipsilateral venous stent.
+24. DVT length to be targeted for perivascular drug therapy exceeds 50 cm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Real World Data Collection in Subjects Treated With the FARAPULSE Pulsed Field Ablation System [NCT05501873]</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Subjects intended to be treated with the FARAPULSE™ Pulsed Field Ablation system for cardiac tissue ablation, per physician's medical judgement, and as per hospitals' standard of care
+2. Subjects who are willing and capable of providing informed consent
+3. Subjects who are willing and capable of participating in all testing associated with this clinical study at an approved clinical investigational center
+4. Subjects whose age is 18 years or above, or who are of legal age to give informed consent specific to state and national law
+Exclusion Criteria:
+1. Subjects with a current interatrial baffle or patch
+2. Subjects with a known or suspected atrial myxoma
+3. Subjects with a myocardial infarction within 14 days prior to enrollment
+4. Subjects with a recent (within 30 days prior to enrollment) Cerebral Vascular Accident (CVA)
+5. Subjects who do not tolerate anticoagulation therapy
+6. Subjects with an active systemic infection \*
+7. Subjects with a presence of atrial known thrombus \*
+8. Subjects with a known inability to obtain vascular access
+9. Subjects who are pregnant or planning to be pregnant
+10. Subjects with atrial fibrillation that is secondary to electrolyte imbalance, thyroid disease, alcohol, or other reversible / non-cardiac causes
+11. Subjects with any prosthetic heart valve, ring or repair including balloon aortic valvuloplasty
+12. Subjects with a contraindication to an invasive electrophysiology procedure where insertion or manipulation of a catheter in the cardiac chambers is deemed unsafe per physician's medical judgement, such as, but not limited to, a recent previous cardiac surgery (eg. ventriculotomy or atriotomy, CABG, PTCA/PCI/coronary stent procedure/unstable angina) and/or in patients with congenital heart disease where the underlying abnormality increases the risk of the ablation (e.g., severe rotational anomalies of the heart or great vessels)
+13. Subjects with a life expectancy of ≤ 1 year per investigator's opinion
+14. Subjects who are currently enrolled in another investigational study or registry that would directly interfere with the current study, except when the subject is participating in a mandatory governmental registry, or a purely observational registry with no associated treatments. Each instance must be brought to the attention of the sponsor to determine eligibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>A Study of Migalastat in Pediatric Subjects (2 to &lt;12 Yrs) With Fabry Disease and Amenable GLA Variants [NCT06904261]</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 2 Years – 11 Years  |  All
+Inclusion Criteria
+* Male or female subjects, diagnosed with Fabry disease who are between ages 2 and \&lt; 12 years at randomization (subjects aged 11 years must have birthdays \&gt; 30 days after randomization)
+* Subject's parent or legally authorized representative is willing and able to provide written informed consent and authorization for use and disclosure of personal health information or research-related health information, and subject provides assent, if applicable.
+* Subject has a GLA variant documented in his/her medical record that is amenable to migalastat prior to Visit 2.
+* Subject has not received ERT (eg, Replagal® \[agalsidase alfa\] or Fabrazyme® \[agalsidase beta\]) for at least 14 days prior to Baseline visit.
+* Subject has at least 1 documented complication (ie, historical or current laboratory abnormality or sign/symptom) of Fabry disease
+* If of reproductive potential, both male and female subjects agree to use a medically accepted method of contraception throughout the duration of the study and for up to 30 days after their last dose of migalastat.
+Exclusion Criteria
+* Has moderate or severe renal impairment (eGFR \&lt; 60 mL/min/1.73 m2 at Visit 1 \[screening\]).
+* Has advanced kidney disease requiring dialysis or kidney transplantation.
+* History of allergy or sensitivity to migalastat (including excipients) or other iminosugars (eg, miglustat, miglitol).
+* Has received any investigational/experimental drug, biologic, or device within 30 days or 5 half-lives of the investigational product (whichever is longer) before Visit 1 (screening).
+* Has received any gene therapy at any time or anticipates starting gene therapy during the study period.
+* Requires treatment with Glyset (miglitol) or Zavesca (miglustat), within 6 months before Visit 1(screening) or throughout the study.
+* Has any intercurrent illness or condition at Visit 1 (screening) or Visit 2 (baseline) that may preclude the subject from fulfilling the protocol requirements or suggests to the investigator that the potential subject may have an unacceptable risk by participating in this study.
+* Pregnant or breastfeeding
+* Otherwise unsuitable for the study in the opinion of the investigator</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Thrombectomy in Pulmonary Embolism [NCT07650435]</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Clinical signs and symptoms consistent with acute pulmonary embolism with duration of 14 days or less
+* Patients who present with computed tomography confirmed pulmonary embolism
+* Defined as intermediate or high-risk pulmonary embolism (according to European Society of Cardiology guidelines)
+* Date of computed tomography imaging from within a two-year period
+* Patient is greater than or equal to 18 years of age
+* Informed consent obtained
+* Evidence of cardiac dysfunction (either biochemical or imaging features of right heart strain)
+Exclusion Criteria:
+* Known serious, uncontrolled sensitivity to radiographic agents
+* Computed tomography not available to evaluate pulmonary embolism
+* Low-risk pulmonary embolism as defined by European Society of Cardiology guidelines
+* Current participation in another investigational drug or device study that may confound the results of this study. Studies requiring extended follow-up for products that were investigational but have since become commercially available are not considered investigational
+* Other medical, social, or psychological conditions that, in the opinion of the investigator, preclude the patient from appropriate consent, could limit the patient's ability to participate in the study, including compliance with follow-up requirements, or that could impact the scientific integrity of the study
+Inclusion Criteria:
+1. Clinical signs and symptoms consistent with acute PE with duration of 14 days or less
+2. Patients who present with CT confirmed PE
+3. Defined as intermediate or high-risk PE (according to ESC guidelines1)
+4. Date of CT imaging from within a two-year period
+5. Patient is ≥ 18 years of age
+6. Informed consent obtained
+7. Evidence of cardiac dysfunction (Either biochemical or imaging features of RHS)
+Exclusion Criteria:
+* 1\. Known serious, uncontrolled sensitivity to radiographic agents 2. CT not available to evaluate PE 3. Low Risk PE as defined by ESC guidelines1 4. Current participation in another investigational drug or device study that may confound the results of this study. Studies requiring extended follow-up for products that were investigational but have since become commercially available are not considered investigational studies 5. Other medical, social, or psychological conditions that, in the opinion of the Investigator, precludes the patient from appropriate consent, could limit the patient's ability to participate in the study, including compliance with follow-up requirements, or that could impact the scientific integrity of the study</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1887,13 +2636,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B4"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -1937,6 +2688,97 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>A Randomised, Controlled Trial of a Low-energy Diet for Improving Functional Status in Heart Failure With PRESERVED Ejection Fraction Preserved Ejection Fraction [NCT05887271]</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Established clinical diagnosis of heart failure with preserved ejection fraction HFpEF (EF\&gt;45%) made by a cardiologist or a primary care physician with heart failure expertise, or a heart failure nurse
+2. Clinically stable for ≥ 3 months (no admissions to hospital)
+3. Obesity (BMI ≥30kg/m2 if white European or ≥27kg/m2 if Asian, Middle Eastern or Black ethnicity)
+4. Age ≥18
+Exclusion Criteria:
+1. Inability to walk/undertake 6-minute walk test
+2. Inability to follow a low-energy MRP
+3. HFpEF due to infiltrative cardiomyopathy (cardiac amyloidosis or sarcoidosis), genetic hypertrophic cardiomyopathy, restrictive cardiomyopathy/pericardial disease or congenital heart disease.
+4. Recovered EF (previous EF \&lt; 40%) unless reduced EF was in context of tachycardia induced cardiomyopathy (eg AF/Aflutter).
+5. Known heritable, idiopathic or drug-induced pulmonary arterial hypertension
+6. Severe chronic obstructive pulmonary disease (FEV1\&lt; 1.0L)
+7. Severe primary valvular heart disease
+8. Anaemia (Hb\&lt;100g/L)
+9. Severe renal disease (eGFR \&lt; 30 ml/min/1.73 m2)
+10. Weight loss \&gt; 5kg in preceding 3 months.
+11. Symptomatic gallstones (including biliary colic) or cholecystitis within last 3 months
+12. Active substance abuse (drugs or alcohol)
+13. History of bariatric surgery in the last 3 years
+14. Active illness likely to cause change in weight
+15. Women who are pregnant or are considering pregnancy
+16. People currently participating in another clinical research trial that is likely to affect diet or weight change.
+17. History of a severe mental illness including an eating disorder
+17\. Individuals with a diagnosis of Type 1 diabetes mellitus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>25-Jun 12:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>A Pan-European Post-Authorisation Safety Study: Risk of Pancreatic Cancer Among Type 2 Diabetes Patients Who Initiated Exenatide as Compared With Those Who Initiated Other Non-Glucagon-Like Peptide 1 Receptor Agonists Based Glucose Lowering Drugs [NCT05663515]</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 99 Years  |  All
+For inclusion in either exposure group, all of the following inclusion criteria must be fulfilled:
+1. Aged 18 years or older at the index date
+2. Individual level data on prescriptions, diagnoses and medical history is available for a minimum of 12 months prior to the index date
+3. A diagnosis of T2DM on index date or prior to index date
+For inclusion in the overall exenatide exposure group, the following criterion must be fulfilled:
+1. One incident prescription (or incident dispensed prescription) for exenatide (BYETTA or BYDUREON/ BYDUREON BCise) between the start and 12 months before the end of the study period. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+   For inclusion in the BYDUREON/ BYDUREON BCise exposure group, for the analyses of the secondary objective, the criterion a) is substituted with criterion b):
+2. One incident prescription (or incident dispensed prescription) for BYDUREON/ BYDUREON BCise between the start and 12 months before the end of the study period. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+   For inclusion in the comparator group, the following criterion must be fulfilled:
+3. One incident prescription (or incident dispensed prescription) of a GLD between the start and 12 months before the end of the study period. The GLD must not be a DPP-4i, a GLP-1 RA, or a combination with either a DPP-4i or a GLP-1 RA. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+Patients are not eligible for any of the study population groups if they fulfil any of the following exclusion criteria:
+1. A diagnosis of type 1 diabetes mellitus (T1DM) on index date or a diagnosis of T1DM during the baseline period that is not succeeded by a T2DM diagnosis during the remaining part of the baseline period.
+2. A diagnosis of gestational diabetes during the baseline period or on index date.
+3. A diagnosis of polycystic ovarian syndrome during the baseline period or on index date in combination with exposure to metformin (Anatomical Therapeutic Chemical Classification System (ATC) code of the World Health Organization (WHO): A10BA02) as the only GLD on index date or during the baseline period.
+4. History of any cancer on or prior to index date. The only exception is that nonmelanoma skin cancer does not lead to exclusion.
+5. History of any acute pancreatitis, other diseases of the pancreas, or disorders of the pancreas on or prior to index date.
+6. One or more prescriptions (or dispensed prescriptions) of a GLP-1 RA (incretin mimetics) other than exenatide on or prior to index date.
+7. One or more prescriptions (or dispensed prescriptions) of DPP-4i (incretin mimetics) on or prior to the index date.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitor update 2026-06-25 15:32 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -2636,15 +2636,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A3:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -2688,7 +2686,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Monitor update 2026-06-26 13:27 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B46"/>
+  <dimension ref="A3:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1890,6 +1890,336 @@
         </is>
       </c>
     </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Efficacy of Pumitamig Versus Pembrolizumab in Participants With Previously Untreated Advanced Non-Small Cell Lung Cancer and PD-L1 ≥ 50%. (ROSETTA Lung-202) [NCT07361510]</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Participants must have a histologically or cytologically confirmed diagnosis of Non-Small Cell Lung Cancer (NSCLC) (squamous and nonsquamous) with Stage IIIB/IIIC or Stage IV disease.
+* Participants must have a programmed death ligand-1 (PD-L1) expression ≥ 50%.
+* Participants must have measurable disease as defined by Response Evaluation Criteria in Solid Tumors (RECIST) v1.1.
+* Participants must have no prior systemic anti-tumor therapy for locally advanced or metastatic NSCLC.
+* Participants must have an Eastern Cooperative Oncology Group (ECOG) Performance Status 0-1.
+Exclusion Criteria
+* Participants must not have any documented actionable genomic alteration (AGA) for which first-line (1L) approved therapies are indicated.
+* Participants must not have any symptomatic untreated central nervous system (CNS) metastases, leptomeningeal metastases (carcinomatous meningitis) or spinal cord compression.
+* Participants must not have any significant cardiovascular impairment as evidenced by uncontrolled hypertension (despite optimal medical treatment), congestive heart failure, active coronary disease (within 6 months prior to randomization), ventricular arrhythmias, or major thrombotic or embolic events or major hemorrhagic events (within 6 months prior to randomization), or significant risk of pulmonary hemorrhage.
+* Participants must not an active autoimmune disease.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Compare the Combination of Navlimetostat (BMS-986504) With Pembrolizumab and Chemotherapy Versus Placebo Plus Pembrolizumab and Chemotherapy in First-line Metastatic Non-small Cell Lung Cancer Participants With Homozygous MTAP Deletion [NCT07063745]</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Participants must have Metastatic (Stage IV or recurrent) non-small cell lung cancer (NSCLC) (as defined by the American Joint Committee on Cancer, Ninth Edition) with no prior systemic anti-cancer therapy for metastatic disease.
+* Participants must have histologically confirmed diagnosis of NSCLC and homozygous methylthioadenosine phosphorylase (MTAP) deletion or MTAP loss.
+* Participants must have an Eastern Cooperative Oncology Group (ECOG) performance status of 0-1.
+* Participants must have at least 1 measurable lesion as per RECIST v1.1.
+Exclusion Criteria
+* Nonsquamous participants must not have documented targetable oncogenic mutation or actionable genetic alterations (AGAs) for which there is a standard of care (SoC) available as first-line (1L) therapy.
+* Participants must not have symptomatic brain metastases or spinal cord compression.
+* Participants must not have any prior systemic therapy (chemotherapy, immunotherapy, targeted therapy, or biological therapy) for metastatic non-small cell lung cancer (mNSCLC).
+Note: One cycle of SoC treatment prior to randomization will be allowed for participants who require immediate treatment if clinically indicated.
+* Participants must not have any known or suspected impairment of gastrointestinal function that may prohibit the ability to absorb or swallow an oral medication without chewing or crushing.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Study to Assess Safety, Efficacy, and Cellular Kinetics of YTB323 in Generalized Myasthenia Gravis [NCT06704269]</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 65 Years  |  All
+Inclusion Criteria:
+1. Confirmed gMG diagnosis supported by the following:
+   * Documented report of positive serology testing for either AChR antibodies or MuSK antibodies at screening AND at least one of the following:
+   * History of abnormal neuromuscular transmission test demonstrated by repetitive nerve stimulation or single-fiber electromyography
+   * History of positive acetylcholinesterase inhibitor test
+   * Improvement in MG signs on an oral acetylcholinesterase inhibitor as assessed by the treating physician
+2. MGFA Class III-IVa (gMG) at screening
+3. Treatment-resistant gMG as defined by: MG-ADL score ≥ 6 (≥50% non-ocular) at screening despite adequate treatment trials with at least two different non-steroidal immunosuppressive drugs given at adequate doses and duration of therapy.
+4. If on chronic corticosteroids, must be on a stable dose of corticosteroids for ≥1 month prior to screening and have the ability and willingness to taper to a maximum dose of 10 mg prednisolone daily or equivalent at least one week before leukapheresis
+5. If treated with cholinesterase inhibitors, patients must be on a stable dose for at least two weeks prior to screening
+Exclusion Criteria:
+1. Exclusively ocular myasthenia gravis (MGFA I), mild symptoms (MGFA II), or severe bulbar disease or MG crisis, MGFA Class IVb or V at screening
+2. History of bone marrow/hematopoietic stem cell or solid organ transplantation.
+3. Clinically significant active, opportunistic, chronic or recurrent infection (including positive for hepatitis B or hepatitis C) confirmed by clinical evidence, imaging, or positive laboratory tests one month prior to leukapheresis
+4. Other uncontrolled disease states, such as asthma, or inflammatory bowel disease, where flares are commonly treated with oral or parenteral corticosteroids, at screening
+5. Participants with a known immunodeficiency syndrome (AIDS, hereditary immune deficiency, drug induced immune deficiency), or tested positive for HIV antibody, at screening
+6. Prior treatment with anti-CD19 therapy, adoptive T cell therapy or any prior gene therapy product (e.g. CAR-T cell therapy).
+Other protocol-defined inclusion/exclusion criteria may apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Pediatric Long-Term Follow-up and Rollover Study [NCT03975829]</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 1 Year – 99 Years  |  All
+Key Inclusion Criteria:
+All Subjects:
+* Written informed consent, according to local guidelines, signed by the subjects and/or by the parents or legal guardian prior to any study related screening procedures are performed.
+* Participation in a Novartis sponsored study such as CTMT212X2101, CDRB436G2201, CDRB436A2102, regardless of current age.
+* Parent study (or cohort of parent study) is planned to be closed.
+* Subject has demonstrated compliance, as assessed by the investigator, within the parent study protocol requirement(s).
+* Willingness and ability to comply with scheduled visits, treatment plans and any other study procedures.
+For Subjects Entering the Treatment Period:
+* Subject is currently receiving treatment with dabrafenib/trametinib monotherapy or combination within a Novartis Sponsored Drug Development study. Note that subjects who were on the chemotherapy arm of the CDRB436G2201 study are eligible for treatment period of this study only after crossing over into the experimental treatment arm of the CDRB436G2201 study
+* In the opinion of the investigator is likely to benefit from continued treatment.
+Key Exclusion Criteria:
+All Subjects:
+\- Subject has participated in a combination trial where dabrafenib and/or trametinib was dispensed in combination with another study medication.
+For Subjects Entering the Treatment Period:
+* Subject has permanently discontinued from study treatment in the parent protocol due to any reason.
+* Treatment with dabrafenib and/or trametinib for the subject's indication is approved for marketing and the appropriate dosage form is commercially available and reimbursed in the local country
+* Subject currently has unresolved drug related severe toxicities for which dabrafenib and/or trametinib dosing has been interrupted in the parent study. If the subject should meet criteria to resume treatment on the parent protocol then they may be eligible for treatment in this study.
+Other protocol-defined inclusion/exclusion may apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>A Study Comparing Pre- and Post-Change Teclistamab in Participants With Relapsed or Refractory Multiple Myeloma [NCT06425991]</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Documented diagnosis of multiple myeloma as defined by the criteria below: (a) Multiple myeloma diagnosis according to International Myeloma Working Group (IMWG) diagnostic criteria (b) Measurable disease at screening as defined by any of the following: (1) Serum M-protein level greater than or equal to (\&gt;=) 0.5 grams per deciliter (g/dL) (central laboratory); or (2) Urine M-protein level \&gt;=200 milligrams (mg)/24 hours (central laboratory); or (3) Serum immunoglobulin free light chain \&gt;=10 milligrams per deciliter (mg/dL) (central laboratory) and abnormal serum immunoglobulin kappa lambda free light chain ratio
+* Received 1 to 3 prior lines of antimyeloma therapy, including a minimum of 2 consecutive cycles each of a protease inhibitor (PI), lenalidomide, and an anti-cluster of differentiation 38 (CD38) monoclonal antibody (or minimum of 6 doses if anti CD38 monoclonal antibody was only part of a maintenance regimen) in any prior line
+* Documented evidence of progressive disease or failure to achieve a response to last line of therapy based on investigator's determination of response by IMWG criteria
+* Have an eastern cooperative oncology group (ECOG) performance status score of 0 to 2
+* A female participant of childbearing potential must have a negative highly sensitive serum pregnancy test at screening and within 24 hours of the start of study treatment and must agree to further serum or urine pregnancy tests during the study
+Exclusion Criteria:
+* Received any bispecific antibody and/or chimeric antigen receptor T cell (CAR-T) cell therapy
+* Contraindications or life-threatening allergies, hypersensitivity, or intolerance to any study drug or its excipients
+* Received a live, attenuated vaccine within 4 weeks before the first dose of study drug. Non-live or non-replicating vaccines authorized for emergency use by local health authorities are allowed
+* Central nervous system involvement or clinical signs of meningeal involvement of multiple myeloma. If either is suspected, negative whole brain magnetic resonance imaging (MRI) and lumbar cytology may be required
+* Participant had major surgery or had significant traumatic injury within 2 weeks prior to randomization, or will not have fully recovered from surgery, or has major surgery planned during the time the participant is expected to be treated in the study</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Pancreatic Cancer Early Detection Consortium [NCT04970056]</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 90 Years  |  All
+Inclusion Criteria:
+Individuals from the following groups who present for clinical evaluation and assessment of PDAC risk at any of the participating sites can be offered participation in the PRECEDE database:
+Cohort 1
+Individuals without history of PDAC meeting any of the following criteria:
+1. 2+ relatives with PDAC on same side of family where 2 affected are first degree related to each other and at least 1 affected is first degree related to subject; age 50+ or ≤10 years younger than earliest PDAC in family at time of diagnosis.
+2. 2 affected first degree relatives with PDAC; age 50+ or 10 years younger than earliest PDAC in family
+3. BRCA1, BRCA2, PALB2, ATM, MLH1, MSH2, MSH6, PMS2, EPCAM pathogenic or likely pathogenic variant AND 1 first or second degree relative with PDAC; age 50+ or 10 years younger than earliest PDAC in family
+4. Familial Atypical Moles and Malignant Melanoma (FAMMM) with pathogenic or likely pathogenic CDKN2A variant; age 40+
+5. Peutz-Jegher syndrome with STK11 pathogenic or likely pathogenic variant; age 35+
+6. Hereditary pancreatitis with PRSS1 pathogenic or likely pathogenic variant and history of pancreatitis; age 40+
+Cohort 2
+Individuals without history of PDAC meeting any of the following criteria:
+1. ATM, BRCA1, BRCA2, or PALB2 pathogenic or likely pathogenic variant regardless of family history, age 50+
+2. 2+ relatives with PDAC on the same side of family, any degree of relation, not meeting other criteria above; age 50+ or 10 years younger than earliest PDAC in family
+3. 1 first degree relative with PDAC ≤ age 45; age up to 10 years younger than PDAC diagnosis in family member
+Cohort 3 Individual meeting criteria for Cohorts 1 or 2 EXCEPT age (i.e. too young to qualify for Cohorts 1 or 2)
+Cohort 4 Individuals without history of PDAC presenting for evaluation who do not meet any criteria for 1-3, 6, or the Cyst Cohort.
+Cohort 5 Individuals without history of PDAC who are not otherwise engaged in pancreas surveillance at a participating site may be invited to participate in the PRECEDE database and to donate a biosample (e.g. blood, saliva, and/or buccal swab) for discovery studies. This may include relatives of individuals in Cohorts 1-4,6, and the Cyst Cohort.
+Cohort 6a
+Individuals diagnosed with PDAC or pancreatic high-grade dysplasia after enrollment in PRECEDE meeting any of the following criteria:
+1. Family history includes at least one first degree relative with PDAC, or 2 relatives with PDAC who are first degree related to each other
+2. Personal or family history of a pathogenic or likely pathogenic germline variant in ATM, BRCA1, BRCA2, CDKN2A, EPCAM, MLH1, MSH2, MSH6, PALB2,PMS2, PRSS1, STK11
+Cohort 6b
+Individuals with a personal history of PDAC or pancreatic high-grade dysplasia meeting any of the following criteria:
+1. Family history includes at least one first degree relative with PDAC, or 2 relatives with PDAC who are first degree related to each other
+2. Personal or family history of a pathogenic or likely pathogenic germline variant in ATM, BRCA1, BRCA2, CDKN2A, EPCAM, MLH1, MSH2, MSH6, PALB2,PMS2, PRSS1, STK11
+3. Diagnosed ≤ age 45
+Cohort 6c Individuals with newly diagnosed early stage (stage I or stage II) PDAC seen at a PRECEDE site that do not meet the criteria for 6a or 6b.
+Cohort 6d Individuals with PDAC seen at a PRECEDE site that do not meet the criteria for 6a, 6b, or 6c.
+Cyst Cohort Individuals with a personal history of a pancreatic cystic neoplasm not meeting any criteria for Cohorts 1-3 or 6 (no known family history of PDAC, no known pathogenic germline variants linked to PDAC risk)
+Exclusion Criteria:
+* Individuals not meeting the criteria above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="36" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Safety and Efficacy of Pumitamig in Combination With Chemotherapy Versus Nivolumab in Combination With Chemotherapy in Participants With Previously Untreated Advanced or Metastatic Gastric, Gastroesophageal Junction, or Esophageal Adenocarcinoma (ROSETTA Gastric-204) [NCT07221149]</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Participants must be previously untreated with systemic treatment for advanced/metastatic disease, histologically or cytologically confirmed advanced or metastatic gastric cancer (GC), gastroesophageal junction adenocarcinoma (GEJC) or distal esophageal adenocarcinoma (EAC). GEJ involvement can be confirmed via biopsy, endoscopy, or imaging.
+* Participants must have a documented programmed cell death-(ligand)1 (PD-L1) ≥ 1 or \&lt; 1 status for Phase 2, and document PD-L1 ≥ 1 status for the Phase 3 part of the study.
+* Participants must have documented human epidermal growth factor receptor 2 (HER2)-negative cancer, as determined according to local guidelines.
+* Participants must have measurable disease as defined by RECIST v1.1.
+Exclusion Criteria
+* Participants must not have untreated known central nervous system (CNS) metastases.
+* Participants must not have significant cardiovascular disease, such as myocardial infarction, unstable angina, arterial thrombosis, cerebrovascular accident within 6 months prior to randomization, uncontrolled hypertension (≥ 160 systolic, ≥ 100 diastolic mm Hg) despite optimal medical management, or congenital long QT syndrome.
+* Participants must not have evidence of major coagulation disorders (eg, hemophilia).
+* Participants must not have a history of deep vein thrombosis, pulmonary embolism, or any other significant thromboembolism within 3 months prior to randomization, unless the participant has been fully treated (eg, inferior vena cava filter placed) and/or adequately anticoagulated on a stable dose.
+* Participants must not have a history of abdominal fistula or gastrointestinal (GI) perforation within 6 months of randomization.
+* Participants must not have had major surgery, open biopsy, or significant traumatic injury within 28 days prior to randomization, or anticipation of the need for major surgery during the course of study intervention.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="36" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Safety, Tolerability, and Efficacy of Pumitamig Alone or in Combination With Ipilimumab or Cabozantinib in Participants With Advanced Renal Cell Carcinoma (RCC) (ROSETTA RCC-208) [NCT07293351]</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Participants must have a histologically confirmed diagnosis of locally advanced, unresectable (not amenable to curative surgery or radiation therapy) or metastatic Renal Cell Carcinoma (RCC).
+* Participants must have clear cell RCC (ccRCC) or non-clear cell RCC (nccRCC) may be enrolled in Part 1. Note: Part 2 may only enroll participants with ccRCC.
+* Participants may have favorable, intermediate or poor risk disease categories.
+* Participants must not have received prior systemic therapy for metastatic RCC, with the following exceptions:
+  i) One prior adjuvant or neoadjuvant therapy for completely resectable RCC is allowed if such therapy did not include an agent that targets vascular endothelial growth factor (VEGF) or VEGF receptors and if recurrence occurred at least 6 months after the last dose of adjuvant or neoadjuvant therapy.
+ii) For Part 1A participants: Prior systemic therapy in the metastatic setting is allowed if the participant has not received any therapy targeting cytotoxic T-lymphocyte antigen 4 (CTLA-4) (e.g., ipilimumab).
+iii) For Part 1B participants: Prior systemic therapy in the metastatic setting is allowed if the participant has not received prior treatment with cabozantinib.
+\- Participants must have measurable disease as per Response Evaluation Criteria in Solid Tumors (RECIST) v1.1.
+Exclusion Criteria
+* Participants must not have any untreated known CNS metastases.
+* Participants must not have a condition requiring systemic treatment with either corticosteroids (\&gt; 10 mg daily prednisone equivalent) or other immunosuppressive medications within 14 days of Cycle 1 Day1 (C1D1).
+* Participants must not have a history of interstitial lung disease or pneumonitis.
+* Participants must not have an uncontrolled pleural or pericardial effusion requiring recurrent therapeutic drainage procedures.
+* Participants must not have significant cardiovascular disease, such as myocardial infarction, unstable angina, arterial thrombosis, cerebrovascular accident within 6 months prior to C1D1, uncontrolled hypertension (≥ 150 systolic, ≥ 90 diastolic mm Hg) despite optimal medical management, or congenital long QT syndrome.
+* Participants must not have a urine protein ≥ 2+ and 24 hour urine protein ≥ 1 g at baseline.
+* Participants must not have evidence of major coagulation disorders.
+* Participants must not have a history of deep vein thrombosis, pulmonary embolism, or any other significant thromboembolism within 6 months prior to C1D1.
+* Participants must not have a history of abdominal fistula or gastrointestinal (GI) perforation within 6 months.
+* Participants must not have had a major surgery or trauma within 28 days prior to C1D1.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1901,11 +2231,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B46"/>
+  <dimension ref="A3:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="3" ht="22" customHeight="1">
@@ -2118,14 +2449,46 @@
           <t>24-Jun 13:33</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Study to Evaluate Adverse Events, Change in Disease Activity, and How Oral ABBV-101 Moves Through the Body in Adult Participants With B-Cell Malignancies [NCT05753501]</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* For Dose Escalation (Part 1) only (including backfill): Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have a documented diagnosis for one of the following third line or later B-cell malignancies, from one of the following world health organization (WHO)-defined histologies (Swerdlow et al 2016):
+  * Chronic lymphocytic leukemia (CLL)/small lymphocytic lymphoma (SLL)
+    1. For Dose Escalation (Part 1) backfill only - Bruton's tyrosine kinase inhibitor (BTKi)/Bruton's tyrosine kinase degrader (BTKd)-naïve CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received at least one prior systemic therapy that cannot be a BTK inhibitor or degrader, and, with the exception of BTK pathway agents, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+    2. For Dose Escalation (Part 1) backfill only - BTKi/BCL-2i combination regimen-exposed 2L CLL/SLL. Participants with a documented diagnosis of CLL/SLL who have received one prior systemic therapy with a BTKi and BCL-2i combination regimen, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), and have measurable disease requiring treatment.
+  * Chimeric antigen receptor T-cells (CAR-T)/hematopoietic cell transplant (HCT) relapsed/refractory (R/R) or ineligible diffuse large b-cell lymphoma (DLBCL) from the following histologies: DLBCL not otherwise specified (NOS) (germinal center B cell \[GCB\] and non-GCB DLBCL), T-cell/histiocyte-rich large B-cell lymphoma, primary mediastinal (thymic) large B-cell lymphoma, intravascular large B-cell lymphoma, anaplastic lymphoma kinase positive (ALK+) large B-cell lymphoma, high-grade B-cell lymphoma with MYC and BCL2 and/or BCL6 rearrangements, and high-grade B-cell lymphoma NOS.
+  * Mantle cell lymphoma (MCL)
+  * Follicular lymphoma \[FL\] (grades 1-3b)
+  * Marginal zone lymphoma \[MZL\] (splenic, extranodal, and nodal)
+  * Waldenström macroglobulinemia (WM)
+  * Transformed indolent non-Hodgkin's lymphoma (iNHL)
+* For Dose Expansion (Part 2a) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment.
+* For Dose Expansion (Part 2a) DLBCL only: Participants have received at least two prior systemic therapies, have no available therapies known to provide clinical benefit (e.g., standard chemotherapy or HCT), have measurable disease requiring treatment, and have documented diagnosis of CAR-T/HCT R/R or ineligible non-GCB DLBCL who are in their third line or later treatment with histology based on criteria established by the WHO.
+* For Dose Exploration of ABBV-101 combination with venetoclax (Part 2b) CLL/SLL only: Participants with a documented diagnosis of CLL/SLL in their first-line or later treatment: In safety lead-in for each dose level, participants must have received at least one prior systemic therapy.
+* Has an Eastern Cooperative Oncology Group (ECOG) Performance Status (PS) of 0, 1, or 2. For EU only: Participant has an ECOG PS of 0 or 1.
+* Participant has a life expectancy \&gt;= 12 weeks.
+* Prior Bruton's tyrosine kinase inhibitor (BTKi) is allowed.
+* Adequate hematologic, renal, and hepatic function per the protocol.
+Exclusion Criteria:
+* Previously treated with a Bruton's tyrosine kinase (BTK) degrader.
+* Known active central nervous system (CNS) disease, or primary CNS lymphoma. Participants with prior CNS disease that have been effectively treated may be eligible.
+* Uncontrolled active systemic infection requiring systemic treatment that is ongoing or was completed \&lt;= 14 days before the first dose of study drug, or active cytomegalovirus infection.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
 Inclusion Criteria:
@@ -2625,6 +2988,322 @@
         </is>
       </c>
     </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>A Study Comparing Pre- and Post-Change Teclistamab in Participants With Relapsed or Refractory Multiple Myeloma [NCT06425991]</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Documented diagnosis of multiple myeloma as defined by the criteria below: (a) Multiple myeloma diagnosis according to International Myeloma Working Group (IMWG) diagnostic criteria (b) Measurable disease at screening as defined by any of the following: (1) Serum M-protein level greater than or equal to (\&gt;=) 0.5 grams per deciliter (g/dL) (central laboratory); or (2) Urine M-protein level \&gt;=200 milligrams (mg)/24 hours (central laboratory); or (3) Serum immunoglobulin free light chain \&gt;=10 milligrams per deciliter (mg/dL) (central laboratory) and abnormal serum immunoglobulin kappa lambda free light chain ratio
+* Received 1 to 3 prior lines of antimyeloma therapy, including a minimum of 2 consecutive cycles each of a protease inhibitor (PI), lenalidomide, and an anti-cluster of differentiation 38 (CD38) monoclonal antibody (or minimum of 6 doses if anti CD38 monoclonal antibody was only part of a maintenance regimen) in any prior line
+* Documented evidence of progressive disease or failure to achieve a response to last line of therapy based on investigator's determination of response by IMWG criteria
+* Have an eastern cooperative oncology group (ECOG) performance status score of 0 to 2
+* A female participant of childbearing potential must have a negative highly sensitive serum pregnancy test at screening and within 24 hours of the start of study treatment and must agree to further serum or urine pregnancy tests during the study
+Exclusion Criteria:
+* Received any bispecific antibody and/or chimeric antigen receptor T cell (CAR-T) cell therapy
+* Contraindications or life-threatening allergies, hypersensitivity, or intolerance to any study drug or its excipients
+* Received a live, attenuated vaccine within 4 weeks before the first dose of study drug. Non-live or non-replicating vaccines authorized for emergency use by local health authorities are allowed
+* Central nervous system involvement or clinical signs of meningeal involvement of multiple myeloma. If either is suspected, negative whole brain magnetic resonance imaging (MRI) and lumbar cytology may be required
+* Participant had major surgery or had significant traumatic injury within 2 weeks prior to randomization, or will not have fully recovered from surgery, or has major surgery planned during the time the participant is expected to be treated in the study</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Anticoagulation for New-Onset Post-Operative Atrial Fibrillation After CABG [NCT04045665]</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Patients of age ≥18 years who undergo isolated CABG for coronary artery disease
+* POAF that persists for \&gt;60 minutes or is recurrent (more than one episode) within 7 days after the index CABG surgery
+Exclusion Criteria:
+* Clinical history of either permanent, persistent or paroxysmal atrial fibrillation
+* Any pre-existing clinical indication for long-term OAC
+* Any absolute contraindication to OAC
+* Planned use of post-operative dual antiplatelet therapy (DAPT)
+  a. This includes, but is not limited to, patients with recent PCI with drug-eluting or bare-metal stent.
+* Cardiogenic shock
+* Major perioperative complication\* occurring between CABG and randomization
+  a. including, but not limited to, stroke, TIA, MI, major bleeding (BARC type 4 bleeding), severe sepsis, renal failure requiring dialysis, or need for reoperation due to bleeding (e.g. pericardial tamponade).
+* Concomitant left atrial appendage closure during CABG
+* Concomitant valve surgery during CABG or prior valve surgery (including aortic, mitral, tricuspid or pulmonary)
+* Concomitant mitral valve annuloplasty during CABG
+* Concomitant carotid artery endarterectomy during CABG
+* Concomitant aortic root replacement during CABG
+* Concomitant surgery for AF during CABG
+* Liver cirrhosis or Child-Pugh Class C chronic liver disease
+* Pharmacologic therapy with an investigational drug or device within 30-days prior to randomization or plan to enroll patient in an investigational drug or device trial during participation in this trial
+* Pregnancy at the time of randomization
+* Unable or unwilling to provide inform consent
+* Unable or unwilling to comply with the study treatment and follow-up
+* Existence of underlying disease that limits life expectancy to less than one year</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Study to Evaluate the Effect of Balcinrenone/Dapagliflozin in Patients With Heart Failure and Impaired Kidney Function [NCT06307652]</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 130 Years  |  All
+Inclusion Criteria:
+* Age ≥ 18 years
+* Documented diagnosis of symptomatic HF (NYHA functional class II-IV)
+* Having had a recent HF event within 6 months (hospitalization or urgent visit)
+* Have a LVEF value from an assessment within the last 12 months
+* Managed with SoC therapy for HF and renal impairment according to local guidelines
+* NT-proBNP must be \&gt;300 pg/mL (\&gt;600 pg/mL if concomitant atrial fibrillation or atrial flutter)
+* Not taking an MRA
+* An eGFR ≥ 20 to \&lt; 60 mL/min/1.73 m2
+* Serum/plasma potassium ≤ 5.0 mmol/L
+Exclusion Criteria:
+* Acute coronary syndrome (unstable angina or myocardial infarction), stroke or transient ischaemic attack within the previous 3 months prior to enrolment or during the screening period
+* Major cardiac surgery, coronary revascularisation or valvular repair or replacement, or implantation of a Cardiac resynchronisation therapy device within 3 months prior to enrolment or during the screening period, or planned to undergo any of these operations
+* History of hypertrophic obstructive cardiomyopathy
+* Complex congenital heart disease or severe uncorrected primary valvular disease
+* Symptomatic bradycardia or second- or third-degree heart block without a pacemaker
+* Systolic BP \&lt; 90 mmHg, or symptomatic hypotension within the past 24 hours
+* Primary pulmonary hypertension, chronic pulmonary embolism, severe pulmonary disease including COPD or exacerbation of COPD requiring invasive mechanical ventilation assistance within 12 months prior to enrolment
+* Type 1 diabetes mellitus
+* Kidney replacement therapy in the past 4 weeks, currently requiring kidney replacement or imminent plan to start kidney replacement therapy
+* Acute or chronic liver disease with severe impairment of liver function, eg, ascites, oesophageal varices, coagulopathy, and encephalopathy
+* Suspected or confirmed COVID-19 infection within the last 4 weeks or hospitalisation for COVID-19 within the last 12 weeks
+* Treatment with strong or moderate CYP3A4 inhibitor or inducer</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Study of Oral Deucrictibant XR Tablet for Prophylaxis and Deucrictibant IR Capsule for On-Demand Treatment of Angioedema Attacks in Adults With Acquired Angioedema Due to C1 Inhibitor Deficiency [NCT07266805]</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Provision of written informed consent
+* Male or female (sex at birth) aged ≥18 years
+* Diagnosis of AAE-C1INH
+* History of AAE-C1INH attacks prior to the Screening Visit:
+* Participants enrolling in Part 1 must have stable underlying disease of AAE-C1INH
+  * The underlying condition can reasonably be expected to remain stable for the duration
+* Reliable access and ability to use available therapy to effectively manage AAE- C1INH attacks.
+* Female participants of childbearing potential must agree to the protocol-specified pregnancy testing and to be abstinent from heterosexual intercourse or to use an acceptable contraception method.
+Females of non-childbearing potential (prepubertal, surgically sterile, or postmenopausal with ≥ 12 months amenorrhea and postmenopausal FSH confirmation) are not required to use contraception during the study.
+• Capable of recording, without assistance, eDiary and ePRO data using an electronic device, as evidenced by the eDiary and ePRO training.
+Exclusion Criteria:
+* Participation in a clinical study with any other investigational drug within the last 30 days or within 5 half-lives of the investigational drug at the Screening Visit (whichever is longer).
+* Participants who have previously received prophylactic therapy but have stopped can participate in this study provided the last dose of the treatment was received prior to the timepoint before the Screening Visit
+* Any females who are pregnant, plan to become pregnant, or are currently breast-feeding
+* Abnormal hepatic function
+* Moderate or severe renal impairment
+* Any clinically significant comorbidity or systemic dysfunction that would interfere with the participant's safety or ability to participate in the study.
+* History of epilepsy and/or other significant neurological diseases
+* Any clinically significant and uncontrolled gastrointestinal dysfunction that may impact study drug absorption
+* Evidence of current alcohol or drug abuse
+* Use of medications that are moderate and strong inhibitors of cytochrome P450 (CYP) 3A4, or strong inducers of CYP3A4 within the last 30 days or within 5 half-lives (whichever is longer) at the time of the Screening Visit
+* Known hypersensitivity to deucrictibant or any of the excipients of the study drug
+* Use of angiotensin-converting enzyme inhibitors or any estrogen-containing medications</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Belzutifan/MK-6482 for the Treatment of Advanced Pheochromocytoma/Paraganglioma (PPGL), Pancreatic Neuroendocrine Tumor (pNET), Von Hippel-Lindau (VHL) Disease-Associated Tumors, Advanced Gastrointestinal Stromal Tumor (wt GIST), or Solid Tumors With HIF-2α Related Genetic Alterations (MK-6482-015) [NCT04924075]</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 12 Years – Not specified  |  All
+The main inclusion criteria include but are not limited to the following:
+* Male and female participants at least 12 years of age (at least 18 years of age for Cohort B1)
+* Diagnosis of one of the following: Advanced/metastatic pheochromocytoma/paraganglioma (PPGL), pancreatic neuroendocrine tumors (pNET), von Hippel-Lindau (VHL) disease associated localized tumors, or advanced wild-type gastrointestinal stromal tumor (wt GIST) or advanced solid tumors with Hypoxia Inducible Factor- 2 alpha subunit (HIF-2α) related genetic alterations
+* Cohort B1: VHL Disease-associated tumors:
+  * Have a diagnosis of VHL disease as determined by a germline test locally and/or clinical diagnosis
+  * Must be ≥18 years of age
+* Has a life expectancy of at least 3 months
+The main exclusion criteria include but are not limited to the following:
+* Unable to swallow orally administered medication or has a disorder that might affect the absorption of belzutifan
+* History of a second malignancy, unless potentially curative treatment has been completed with no evidence of malignancy for 2 years
+* Any of the following: A pulse oximeter reading \&lt;92% at rest, or requires intermittent supplemental oxygen, or requires chronic supplemental oxygen
+* Clinically significant cardiac disease, including unstable angina, acute myocardial infarction, or arterial bypass (CABG) or Percutaneous transluminal coronary angioplasty (PTCA) ≤6 months from study entry, or New York Heart Association Class III or IV congestive heart failure
+* Received prior treatment (except somatostatin analogs) with chemotherapy, targeted therapy, biologics, or other investigational therapy within the past 4 weeks of first dose of study intervention</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>A Phase III Study to Investigate the Efficacy and Safety of Baxdrostat in Combination With Dapagliflozin on CKD Progression in Participants With CKD and High Blood Pressure. [NCT06268873]</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Participants of any sex and gender must be ≥ 18 years old, or older, at the time of signing the informed consent.
+2. Participants with CKD and eGFR ≥ 30 and \&lt; 90 mL/min/1.73 m2 at screening
+3. Urine albumin creatinine ratio \&gt; 200 mg/g (22.6 mg/mmol) and \&lt; 5000 mg/g (565 mg/mmol) at screening
+4. Participants with history of HTN and a SBP ≥ 130 mmHg at screening and ≥ 120 mmHg at the randomisation visit
+5. Stable and maximum tolerated dose of an ACE inhibitor or an ARB (not both) for at least 4 weeks prior to Screening Visit
+6. Central laboratory serum potassium must meet the following criteria at the Screening Visit, based on screening eGFR:
+   * for participants with screening eGFR ≥ 45 mL/min/1.73 m2, potassium must be ≥ 3.0 and ≤ 4.8 mmol/L at the Screening Visit
+   * for participants with screening eGFR \&lt; 45 mL/min/1.73 m2, potassium must be ≥ 3.0 and ≤ 4.5 mmol/L at the Screening Visit
+Exclusion Criteria:
+1. Systolic blood pressure \&gt; 180 mmHg, or DBP \&gt; 110 mmHg at screening.
+2. Known hyperkalaemia, defined as potassium of ≥ 5.5 mmol/L within 3 months at screening.
+3. Serum sodium \&lt; 135 mmol/L at the Screening Visit, determined as per central laboratory.
+4. Diabetes mellitus:
+   (a) T1DM at Screening Visit: (i) For US only: patients with T1DM treated with SGLT2i for at least 4 months, without DKA during that period, and who have experience with ketone monitoring are eligible for inclusion.
+   (ii) For Japan only: patients with T1DM treated with dapagliflozin 10 mg for at least 4 months, without DKA during the period of dapagliflozin treatment are eligible for inclusion.
+   (b) Uncontrolled T2DM at screening: HbA1C \&gt; 10.5% (\&gt; 91 mmol/mol).
+5. New York Heart Association functional HF class IV at screening.
+6. Stroke, transient ischaemic cerebral attack, valve implantation or valve replacement, carotid surgery, or carotid angioplasty, acute coronary syndrome, or hospitalisation for worsening heart failure within previous 3 months prior to randomisation.
+7. Any dialysis (including for acute kidney injury) within 3 months prior to Screening Visit.
+8. Any acute kidney injury within 3 months prior to the Screening Visit
+9. History of organ transplant or bone marrow transplant, or planned organ transplant within 6 months following randomisation (including kidney transplant).
+10. History or ongoing allergy/hypersensitivity, as judged by the investigator, to SGLT2 inhibitor (eg, empagliflozin) or ASI.
+11. Any clinical condition requiring systemic immunosuppression therapy other than stable maintenance therapy for at least 3 months prior to Visit 1.
+12. Any use of mineralocorticoid receptor antagonists (such as spironolactone, eplerenone, or finerenone), potassium-sparing diuretics (such as triamterene or amiloride), or potassium binders (such as sodium zirconium cyclosilicate, patiromer, or sodium polystyrene sulfonate) within 4 weeks prior to screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="36" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Study of Lesion-Specific Invasive Haemodynamic Angina Thresholds [NCT07386418]</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Eligibility for PCI due to angina or angina-equivalent symptoms on exertion
+2. 2 severe epicardial stenoses in a major coronary artery, defined as:
+   1. ≥70% stenosis in a coronary artery with ≥2.5mm diameter, on invasive coronary angiography (ICA)
+   2. Severe stenosis in a vessel with ≥2.5mm diameter, on CTCA
+3. Evidence of ischaemia on an invasive or non-invasive test, including:
+   1. Physiological test during invasive coronary angiography (ICA)
+   2. Dobutamine stress echocardiography (DSE)
+   3. Stress perfusion cardiac magnetic resonance (CMR)
+   4. Myocardial perfusion scintigraphy (MPS)
+   5. Fractional flow reserve computed-tomography (FFR-CT)
+Exclusion Criteria:
+1. Age \&lt;18 years
+2. Acute coronary syndrome within 3 months
+3. Previous coronary artery bypass graft
+4. Significant left main stem disease
+5. Single lesion amenable to PCI
+6. Chronic total occlusion of the target artery
+7. Moderate to severe valve disease
+8. LVEF ≤40%, contraindication to PCI or drug-eluting stents
+9. PCI performed with drug-eluting balloons without stenting
+10. Contraindication to antiplatelet therapy
+11. Contraindication to adenosine
+12. Physical inability to exercise with an ergometer
+13. Femoral artery access
+14. Pregnancy
+15. Inability to consent</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2636,13 +3315,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B10"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -2686,6 +3367,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -2734,6 +3416,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -2776,6 +3459,114 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Efficacy of KL1333 in Adult Patients With Primary Mitochondrial Disease [NCT05650229]</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Age 18 years or older.
+* A confirmed PMD diagnosis caused by a known pathogenic gene mutation or deletion of the mitochondrial genome (category 6 of the International Classification of Inborn Metabolic Disorders \[ICIMD\])12 according to American College of Medical Genetics (ACMG)/Association of Molecular Pathology (AMP) criteria1, with multisystemic disease expressions, including:
+  1. m.3243A\&gt;G associated MELAS-MIDD spectrum disorders,
+  2. single large scale mtDNA deletion associated KSS-CPEO spectrum disorders,
+  3. other multisystemic mtDNA-related disease (including MERRF).
+* Presence of chronic mitochondrial fatigue:
+  * History of mitochondrial fatigue for at least 3 months prior to the Screening Visit AND
+  * Presence of at least moderate level of fatigue, assessed by PROMIS® Fatigue PMD Short form raw score ≥ 27 at Screening and Baseline
+* Presence of mitochondrial myopathy defined as:
+  * Myopathy (proximal muscle weakness), NMDAS Section III Clinical Assessment, item 5 score ≥ 1, which reads: "minimal reduction in hip flexion and/or shoulder abduction only (e.g. MRC 4+/5)". For the inclusion only hip flexion, but not shoulder abduction, should be taken into account. AND / OR
+  * Exercise Tolerance: NMDAS Section I, item 9 score ≥ 1, which reads: "unlimited on flat - symptomatic on inclines or stairs".
+* Patients must be able to perform at least 2 repetitions and the maximal capacity must not exceed 17 repetitions in males or 16 repetitions in females in a 30s STS test at screening.
+* Clinically stable, apart from symptoms associated with the diagnosis of mitochondrial disease, at Screening and Baseline, as determined by medical history, physical examination, 12-lead ECG, vital signs measurements, and clinical laboratory evaluations at Screening, as assessed by the investigator.
+* The patient is willing and able to attend study appointments within the specified time windows.
+* Willingness and ability to complete electronic PROs.
+* Willingness to maintain a stable diet during the Screening and study periods.
+* Patients who take any mitochondrial disease-focused vitamins or supplemental therapies, including coenzyme Q10 (CoQ10), niacin/nicotinamide (vitamin B3), and L-arginine, has been on a stable dose regimen of these for 3 months prior to randomisation and intends to stay on a stable dose for the duration of the study period.
+* Willingness to suspend treatment with idebenone during the study.
+* Female patient is not pregnant and at least one of the following conditions apply:
+  1. Not a woman of childbearing potential (WOCBP)
+  2. WOCBP must agree not to try and become pregnant and use a highly effective method of contraception from the time of informed consent through at least 36 days (\~5 half-lives of KL1333 plus 30 days) after the last dose of investigational medicinal product (IMP) administration.
+* Male patients with female partner(s) of childbearing potential must agree to use a male condom in addition to using highly effective contraception throughout the treatment period and for 96 days after the last dose of IMP administration. The requirement to use a male condom also applies to male patients with a pregnant or breastfeeding partner.
+* Female patients must agree not to breastfeed starting at Screening and throughout the study period and for 36 days after the last dose of IMP administration.
+* Female patients must agree to not donate ova throughout the study period and for 36 days after the last dose of IMP administration, and male patients must agree to not donate sperm throughout the study period and for 96 days after the last dose of IMP administration.
+Exclusion Criteria:
+* Primary mitochondrial disease with predominant neurodegenerative phenotypes, such as, but not limited to, Leigh syndrome, Leber hereditary optic neuropathy (LHON) and Neuropathy ataxia-retinitis pigmentosa syndrome (NARP).
+* Primary mitochondrial disease nuclear DNA mutations or mutations causing mtDNA destabilisation. Genetic mtDNA variants of uncertain significance, likely pathogenic, or pathogenic mutations with degrees of heteroplasmy below what can be considered to definitely cause PMD.
+* General fatigue or muscle weakness due to causes other than mitochondrial disease, in the opinion of the investigator.
+* Significant cardiovascular disease (e.g., sustained or symptomatic arrhythmia; dilated heart chambers or reduced function; Mobitz II atrioventricular block or greater) OR abnormal ECG that is clinically significant, as determined by the investigator. Any QTcF \&gt; 450 msec for male patients and \&gt; 470 msec for female patients is exclusionary. In the case of an exclusionary QTcF, the ECG can be repeated twice and the average of 3 QTcF intervals should be used to determine the QTcF eligibility.
+* Recent history of unstable disease, inadequately controlled neurological manifestations or not recovered from stroke-like episodes including but not limited to:
+  1. stroke-like episodes within the last 6 months
+  2. more than 1 seizure/month within the last 6 months
+  3. hospitalised for Status Epilepticus within the last 6 months
+  4. more than 4 days of migraine episodes/month within the last 6 months
+* History of inflammatory bowel disease, gastric erosions, peptic ulcer disease, or gastrointestinal bleeding episodes. Gastroesophageal reflux disease diagnosed by objective endoscopic or radiographic means, and clinically symptomatic at any point over the last 6 months.
+* The patient has one or more clinical laboratory test values outside the reference range, based on the blood and urine samples taken at the Screening Visit, that are of potential risk to the patient's safety, or the patient has, at the Screening Visit:
+  * estimated glomerular filtration rate (eGFR) calculated by the Chronic Kidney Disease Epidemiology Collaboration (CKD-EPI) creatinine equation \&lt;30 mL/min/1.73 m2
+  * a serum total bilirubin value \&gt; 1.5 times the upper limit of the reference range unless elevation is related to Gilbert's syndrome and the investigator can rule out any underlying liver dysfunction based on other tests, the patient has a Child-Pugh score ≤6, and after discussing the case with the medical monitor
+  * a serum alanine aminotransferase (ALT) or aspartate aminotransferase (AST) value \&gt; 2 times the upper limit of the reference range. Values between 2 and 3 times the upper limit of the reference range may be allowed if concomitant to elevation in creatine kinase as long as the investigator can rule out any underlying liver dysfunction based on other tests, the patient has a Child-Pugh score ≤6, and after discussing the case with the medical monitor
+* The patient has, in the investigator's opinion, severe ataxia, neuropathy, balance problems or other medical condition that would interfere the evaluation of the 30s STS test.
+* Untreated or undertreated sleep apnoea, in the opinion of the investigator.
+* Use of idebenone within 14 days prior to the first dose.
+* Patients have a history of unstable or severe pulmonary, immunological, oncological, hepatic disease, renal disease, or another medically significant illness other than PMD or takes medication that could, in the investigator's opinion, interfere with the assessments of safety, tolerability, or efficacy, or interfere with the conduct or interpretation of the study.
+* The patient is, in the investigator's opinion, unlikely to comply with the protocol e.g. due to cognitive impairment or is unsuitable for any reason.
+* The patient has an immediate family member (defined as family members residing at the same address) who participates in the study.
+* Female patients with a positive pregnancy result at Screening or at Baseline.
+* A patient cannot participate if they received an investigational drug 30 days or 5 half-lives prior to the Screening Visit (whichever is longer), or plans to use an investigational drug (other than the study intervention) during the study
+* Hypersensitivity to the active substance or to any of the excipients or placebo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>26-Jun 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>A Study of Baricitinib (LY3009104) for the Delay of Stage 3 Type 1 Diabetes in At-Risk Children and Adults [NCT07222137]</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 1 Year – 35 Years  |  All
+Inclusion Criteria:
+* Have a history of at least one documented occasion of at least two diabetes-related autoantibodies, AND one occasion of at least two diabetes-related autoantibodies obtained at screening or prescreening
+* Have Stage 1b or Stage 2 type 1 diabetes
+* Have a body weight of ≥8 kilograms (kg) (18 pounds) at screening
+Exclusion Criteria:
+* Have any other type of diabetes
+* Have uncontrolled high blood pressure
+* Have had a heart attack, heart disease, stroke, or heart failure
+* Have a history or high risk of venous thromboembolism, lymphoproliferative disease or malignancy
+* Have a current or recent clinically serious infection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitor update 2026-06-26 15:37 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -3315,15 +3315,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A3:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3367,7 +3365,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3416,7 +3413,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3459,7 +3455,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Monitor update 2026-06-29 16:08 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B70"/>
+  <dimension ref="A3:B94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2220,6 +2220,335 @@
         </is>
       </c>
     </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate Safety, Pharmacokinetics, and Activity of GDC-7035 as a Single Agent and in Combination in Patients With Advanced Solid Tumors [NCT06619587]</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Histologically documented advanced or metastatic solid tumor with KRAS G12D mutation
+* Agreement to adhere to the contraception requirements described in the protocol for participants of childbearing potential and participants who produce sperm
+Exclusion criteria:
+* Malabsorption or other condition that would interfere with enteral absorption
+* Active brain metastases
+* Clinically significant cardiovascular dysfunction or liver disease</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="36" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Endoscopic Submucosal Dissection for Early GI Neoplasia in the United Kingdom [NCT03039309]</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Male or Female, aged 18 years or above undergoing endoscopic submucosal dissection
+* Participant is able to give informed consent for participation in the study
+Exclusion Criteria:
+* Patients under the age of 18
+* Patients unable to give informed consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Safety, Pharmacokinetics, and Activity of RO7566802 as a Single Agent and in Combination With Atezolizumab in Participants With Locally Advanced or Metastatic Solid Tumors [NCT06031441]</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Eastern Cooperative Oncology Group (ECOG) Performance Status of 0-1
+* Life expectancy \&gt;=3 months, in the investigator's judgment
+* Adequate hematologic and end-organ function
+* Histologically confirmed locally advanced, recurrent, or metastatic incurable solid tumor malignancy that has progressed after available standard therapy; or for whom standard therapy has proven to be ineffective or intolerable or is considered inappropriate; or for whom a clinical trial of an investigational agent is a recognized standard of care
+* Measurable disease per RECIST v1.1
+* Tumor specimen availability, for certain cohorts
+Exclusion Criteria:
+* Any anti-cancer therapy, whether investigational or approved, including chemotherapy, hormonal therapy, or radiotherapy, within 3 weeks prior to Cycle 1 Day 1, with certain exceptions
+* Active hepatitis B or C
+* Active tuberculosis
+* Positive test for human immunodeficiency virus (HIV) infection
+* Administration of a live, attenuated vaccine (e.g., Flumist) within 4 weeks prior to RO7566802 infusion
+* Symptomatic, untreated, or actively progressing central nervous system (CNS) metastases
+* Active or history of autoimmune disease
+* Prior allogeneic stem cell or organ transplantation
+* Uncontrolled tumor-related pain
+* Significant cardiovascular disease
+Other protocol-defined inclusion/exclusion criteria may apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="36" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>A Phase I/II Study of AZD4512 Monotherapy or in Combination With Anticancer Agents in Participants With Relapsed/Refractory B-cell Non-Hodgkin Lymphoma [NCT07123454]</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Key Inclusion Criteria:
+* Eligible patients must be adults (≥18 years)
+* Documented histologically confirmed diagnosis of B-cell non-Hodgkin lymphoma (B-NHL) as per World Health Organization (WHO) 2022 classification. In the dose escalation phase, any B-NHL subtype is allowed (excluding some subtypes), while the backfill phase restricts inclusion to defined subtypes: large B-cell lymphomas (as defined as Diffuse large B-cell lymphoma (DLBCL), Grade 3b Follicular lymphoma (FL), high-grade B-cell lymphoma (HGBCL) NOS, DLBCL/HGBCL with MYC and BCL2 rearrangements, primary mediastinal Large B-cell lymphoma, T-cell/histiocyte-rich LBCL, and transformed indolent lymphoma) and mantle cell lymphoma.
+* Patients must have relapsed or refractory disease after at least two prior lines of systemic therapy and lack additional standard options with established benefit:
+A)LBCL patients must have progressed after both anti-CD20 and at least one systemic chemotherapy regimen, and have considered-or be ineligible for-CAR-T, T cell engager, and stem cell transplant modalities.
+B) Mantle cell lymphoma (MCL) patients must have had anti-CD20 and Bruton's Tyrosine Kinase (BTK) inhibitor.
+Additional criteria include measurable disease by Lugano 2014, Eastern Cooperative Oncology Group (ECOG) performance status ≤2, and adequate organ and bone marrow function (as specified by blood counts, cardiac ejection fraction, renal and hepatic parameters, and coagulation indices).
+Key Exclusion criteria
+* Patients are excluded if they have a diagnosis of post-transplant lymphoproliferative disease, Richter's transformation, Burkitt's lymphoma, or chronic lymphocytic leukemia (CLL)/ Small lymphocytic lymphoma (SLL), Waldenstrom Macroglobulinemia/ Lymphoplasmacytic Lymphoma, or if they have active Central nervous system (CNS) involvement from their B-NHL. Exclusion also applies to those who have received Chimeric antigen receptor-T (CAR-T) or T cell engager therapies within 90 days prior to Cycle 1 Day 1 (C1D1), any investigational drug or other systemic anticancer therapies (except low-dose corticosteroids) within 21 days or 5 half-lives, and curative radiation within 14 days (localized palliative radiotherapy is allowed).
+* Other exclusions include allogeneic Hematopoietic stem cell transplantation (HSCT) within 180 days (unless stable without active (graft-versus-host disease) GVHD for ≥2 months), autologous HSCT within 90 days (unless resolved toxicities), major surgery within 28 days, use of strong CYP3A inhibitors within 14 days or 5 half-lives before the dosing date, use of QTc-prolonging agents within 5 half-lives before the dosing date, or other malignancies within two years. Patients with unresolved ≥ Grade 2 AEs from prior therapy (except specified tolerable conditions), serious uncontrolled medical conditions, active infection within 14 days, or history/suspicion of significant interstitial lung disease/pneumonitis are also excluded.
+* Females who are pregnant or breastfeeding are not eligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="36" customHeight="1">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Study of CryptiVax-1001 in Maintenance Setting for Advanced Serous Ovarian, Fallopian Tube, or Primary Peritoneal Cancer [NCT07665515]</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  Female
+Inclusion Criteria:
+* Able to comprehend and are willing to sign the ICF and willing to follow the study procedures
+* Female, aged 18 years of age or older at the time of informed consent.
+* Histologically confirmed diagnosis of epithelial ovarian, fallopian tube, or primary peritoneal carcinoma of high-grade serous histology or other high-grade predominantly serous subtypes
+* The FIGO 2014 stage III or IV disease at initial diagnosis.
+* Underwent optimal PDS or IDS with residual disease ≤1 cm (R0 or R1 resection)
+* Completed first-line platinum-based chemotherapy (minimum 4 cycles of carboplatin and paclitaxel, or equivalent, received in either neoadjuvant or adjuvant, or both settings).
+* In the presence of measurable target lesion, achieved CR or PR per investigator assessment based on RECIST 1.1 after completion of chemotherapy. In the absence of measurable target lesion, no new lesion or overt progression per investigator assessment based on RECIST 1.1 after completion of chemotherapy.
+* A minimum of 4 weeks from screening since the last dose of first-line platinum-based chemotherapy but not more than 12 weeks from screening since the last dose of first-line platinum-based chemotherapy.
+* No evidence of radiologic or clinical progression between the end of chemotherapy and baseline screening.
+* Known BRCAwt status.
+* HRP confirmed
+* No prior, current, or planned treatment with bevacizumab or PARPi in the first-line maintenance setting.
+* ECOG performance status of 0 or 1.
+* Adequate haematologic and organ function
+* Negative pregnancy test for WOCBP.
+* HLA type matching Cryptivax-1001
+Exclusion Criteria:
+* Non-epithelial or low malignant potential ovarian tumours
+* Presence of uncontrolled ascites or pleural effusion requiring drainage within 4 weeks of screening.
+* Concurrent malignancy or history of another malignancy within the past 3 years except for malignancies with a negligible risk of metastasis or death
+* Active autoimmune disease requiring systemic immunosuppression
+* Uncontrolled intercurrent illness that, in the opinion of the investigator, would compromise participant safety or interfere with study assessments
+* History of anaphylactic reaction to mRNA-LNP therapies.
+* Previous treatment with any cancer vaccine, checkpoint inhibitor, or adoptive cellular immunotherapy.
+* Administration of any vaccine within 30 days prior to first dosing.
+* Participation in a clinical study involving administration of an IMP (new chemical entity) in the past 90 days or 5 half-lives of that drug (if known) prior to first dosing, whichever is longer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="36" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>A Clinical Study of Ifinatamab Deruxtecan (I-DXd) in People With Metastatic Prostate Cancer (MK-2400-001) [NCT06925737]</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  Male
+Inclusion Criteria:
+The main inclusion criteria include but are not limited to the following:
+* Has histologically- or cytologically-confirmed adenocarcinoma of the prostate without small cell histology
+* Has prostate cancer progression while on androgen deprivation therapy (ADT) (or post bilateral orchiectomy) within 6 months prior to Screening
+* Has current evidence of distant metastatic disease (M1 disease) documented by either bone lesions on bone scan and/or soft tissue disease by computed tomography (CT)/magnetic resonance imaging (MRI)
+* Has received prior treatment with 1 or 2 androgen receptor pathway inhibitors (ARPIs) and progressed during or after at least 8 weeks of treatment
+* Has provided tumor tissue from a core or excisional biopsy from soft tissue not previously irradiated and obtained after disease progression on the most recent prior therapy
+* Has recovered from adverse events (AEs) due to previous anticancer therapies
+Exclusion Criteria:
+The main exclusion criteria include but are not limited to the following:
+* Is unable to swallow tablets/capsules
+* Has any of the following indicators of interstitial lung disease (ILD)/pneumonitis:
+  1. Has any history of ILD/pneumonitis that required steroid use, except for a history of radiation pneumonitis that did not require steroids
+  2. Has current ILD/pneumonitis
+  3. Has a clinical or radiographic suspicion of ILD for which the diagnosis of ILD cannot be ruled out
+* Has clinically severe pulmonary compromise resulting from intercurrent pulmonary illnesses
+* Has uncontrolled or significant cardiovascular disease
+* Has received prior treatment with a taxane-based chemotherapy agent for metastatic castration-resistant prostate cancer (mCRPC)
+* Has had prior discontinuation of an antibody drug conjugate (ADC) that consists of an exatecan derivative (eg, trastuzumab deruxtecan) due to treatment-related toxicities
+* Has a "superscan" bone scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="36" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Assess the Efficacy and Safety of RO7790121 in Participants With Moderate to Severe Rheumatoid Arthritis Who Have Not Responded to or Who Cannot Tolerate Tumor Necrosis Factor (TNF) and/or Janus Kinase (JAK Inhibitors) [NCT07137598]</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Has moderate to severe active RA defined by the presence of \&gt;=6 swollen joints and \&gt;=6 tender joints at screening and baseline (based on 66/68-joint count)
+* Diagnosis of RA for \&gt;=3 months and also fulfills the 2010 American College of Rheumatology (ACR)/European Alliance of Associations for Rheumatology (EULAR) classification criteria for RA
+* Demonstrated an inadequate response or loss of response to or intolerance to \&gt;=1 conventional synthetic disease-modifying antirheumatic drug (csDMARD)
+Exclusion Criteria:
+* Have failed more than two TNF inhibitors or JAK inhibitors
+* Class IV RA according to ACR revised response criteria (Hochberg et al. 1992)
+* Past or current use of other biologic disease-modifying antirheumatic drugs (bDMARDs) (excluding TNF inhibitors) or rituximab
+* Treatment with investigational therapy within 4 weeks or within 5 half-lives of the investigational therapy, whichever is longer, prior to initiation of study treatment.
+* History of any arthritis with onset prior to age 17 years or current diagnosis of inflammatory joint disease other than RA
+* Has been treated with intra-articular, intramuscular, intravenous, trigger point or tender point, intra-bursa, or intra-tendon sheath corticosteroids in the preceding 8 weeks prior to the first dose of study drug
+* History of a severe allergic reaction or anaphylactic reaction or known hypersensitivity to any component of the study drug (or its excipients) and/or other products in the same class
+* Any major surgery within 6 weeks prior to screening or a major surgery planned during the study
+* Any serious, chronic and/or unstable pre-existing medical, psychiatric, or other- condition
+* History of malignancy, with the exception non-metastatic basal cell or cutaneous squamous cell cancer adequately treated with electrodesiccation and curettage or resection or in situ cervical cancer adequately treated and cured
+* Participants with severe chronic or recurrent viral, bacterial, parasitic, or fungal infections
+* History of active hepatitis B virus (HBV), hepatitis C virus (HCV), or human immunodeficiency virus (HIV) infection
+* History of organ transplant
+* Any identified confirmed congenital or acquired immunodeficiency
+* Abnormal laboratory values and liver function test</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="36" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Efficacy and Safety of a New Formulation of Oral Cladribine Compared With Placebo in Participants With Generalized Myasthenia Gravis (MyClad) [NCT06463587]</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Adults of ≥ 18 years of age at the time of signing the informed consent.
+* Diagnosis of Myasthenia Gravis with generalized muscle weakness, meeting clinical criteria for Myasthenia Gravis Foundation of America Class II to IVa classification.
+  * In participants positive for Acetylcholine receptor antibody (anti-AChR) or muscle-specific kinase antibody(anti-MuSK)
+  * In participants that are autoantibody seronegative i.e. not positive for anti-AChR and anti-MuSK antibodies and participants who are positive for anti-low-density lipoprotein receptor-related protein 4 antibodies (anti-LRP4)
+* Has a Screening and Baseline MG-ADL score more than or equal to (\&gt;=) 6 with \&gt;= 50 percentage (%) of the total score due to non-ocular symptoms. Screening and Baseline MG-ADL scores must be stable. The difference between the Screening and Baseline scores should not be more than 2 and there should be no reported MG exacerbation during the Screening period
+* If treated with oral corticosteroids: should be on a stable daily dose for at least 3 months prior to and during screening. In such case, the daily dose of oral steroids should not exceed 20 milligrams(mg)/day for prednisone/ prednisolone, 16 mg/day for methylprednisolone, 3 mg/day for dexamethasone, or 80 mg for hydrocortisone or equivalent doses for other corticosteroids.
+* If treated with acetylcholinesterase inhibitor should be on a stable daily dose (pyridostigmine dose ≤ 480 mg/day or neostigmine ≤ 300 mg/day) for at least 3 months prior to and during screening
+* Have a body weight \&gt;= 40 kilograms
+* Other protocol defined inclusion criteria could apply
+Exclusion Criteria:
+* Immunologic disorder other than MG or any other condition requiring chronic oral, intravenous, intramuscular, or intraarticular corticosteroid therapy. Well-controlled thyroid disease, as per the Treating Investigator or the participants regular treating physician recorded in the source documents, is not exclusionary
+* Molecularly characterized or suspected congenital myasthenic syndrome, Lambert-Eaton myasthenic syndrome, inherited myopathy, muscular dystrophy, acquired myopathy or any other neurologic or systematic disease that mimics MG muscular weakness
+* Active, clinically significant viral, bacterial, or fungal infection, including brain MRI or chest X-ray findings consistent with signs of infection such as PML or TB, or any major episode of infection requiring hospitalization or treatment with parenteral anti-infectives within 8 weeks prior or during Screening, or completion of oral anti-infectives within 8 weeks prior or during Screening. Vaginal candidiasis, onychomycosis, and genital or oral herpes simplex virus considered by the Investigator to be sufficiently controlled would not be exclusionary
+* Has a history of or current diagnosis of active tuberculosis (TB) or is currently undergoing treatment for latent TB infection or has an untreated latent TB infection as determined by documented results within 3 months of the Screening Visit of a positive TB skin test .
+* Active malignancy, or history of cancer or signs of malignancy in any Screening assessment
+* Treatment with nonsteroidal immunosuppressants, used in gMG, such as azathioprine, mycophenolate mofetil, methotrexate, cyclosporine, cyclophosphamide, tacrolimus within 4 weeks prior to randomization
+* Treatment with FcRn or complement inhibitors (such as eculizumab, rozanolixizumab efgartigimod, ravulizumab, zilucoplan or nipocalimab) within 8 weeks prior to randomization
+* History of thymectomy within 6 months prior to Screening.
+* History of generalized seizures (except for history of febrile seizures during the participant's childhood).
+* Negative or indeterminate for Varicella Zoster Virus antibodies at screening
+* History of myasthenic crisis in the last 12 months prior to and during screening
+* History of recurrent infections (that is 3 or more infections per year documented in available source data) within the last 2 years
+* Discontinuation of treatment with any non-steroidal immunosuppressants used in gMG, such as azathioprine, mycophenolate mofetil, methotrexate, cyclosporine, cyclophosphamide, tacrolimus within the last 6 months prior to Screening
+* If treated with non-steroidal immunosuppressants for gMG, the dose at Screening higher than 50 mg/day for azathioprine, 500 mg/day for mycophenolate mofetil, 1 mg/day for tacrolimus, 50 mg/day for cyclosporine, 25 mg/day for cyclophosphamide, or 7.5 mg/week for methotrexate
+* Participation in clinical study of any investigational drug within 6 months, or 5 half-lives of the investigational drug used in the previous clinical study prior to randomization, whichever is longer. However, participants with any prior exposure to cladribine may not enter the study regardless of timing of exposure
+* Other protocol defined exclusion criteria could apply</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2231,7 +2560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C67"/>
+  <dimension ref="A3:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3304,6 +3633,303 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="36" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>KHENERFIN Study: A Trial to Evaluate the Efficacy and Safety of Sonlicromanol in Primary Mitochondrial Diseases [NCT06451757]</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion criteria
+1. Signed Informed Consent
+2. Males and females aged ≥18 years with a multi-system primary mitochondrial disease.
+3. A confirmed mitochondrial DNA tRNALeu(UUR) m.3243A\&gt;G mutation (m.3243A\&gt;G PMD) plus an age adjusted heteroplasmy percentage ≥ 20% in white blood cells \[=blood heteroplasmy/0.977(age+12)\]. Or in urine (urinary epithelial cells), or buccal smear or skeletal muscle (results (obtained per local guidance) ≥ 20% must be available prior to the subject being randomized).
+4. Presence of chronic fatigue (not attributable to other etiologies than PMD):
+   1. Patient self-reported chronic fatigue for at least 3 months prior to the Screening Visit and recorded in the clinical patient files; AND
+   2. Presence of fatigue (raw total score \&gt;22), assessed by Neuro-QoL SFv1-F at Screening.
+5. Presence of mitochondrial myopathy defined as:
+5xSST at Screening and Baseline should be ≥ 11 seconds and participant must demonstrate the ability to complete the test at baseline (i.e., complete the test within 30 seconds).
+6\. Other Inclusion criteria per protocol.
+Exclusion criteria
+1. Treatment with any IMP within 3 months (or 5 times the half-life of the IMP, whichever is longer) prior to screening or plans to use an IMP (other than the study intervention) during the study.
+2. Bone deformities, motor abnormalities or chronic ulcers that in the opinion of the PI may interfere with and/or confound the interpretation of the subject's performance during the 5 times sit to stand test (5XSST).
+3. Surgery of gastrointestinal tract that might interfere with drug absorption. Or severe GI dysmotility, chronic vomiting, diarrhea, bouts of pseudo-obstruction which will impair appropriate IMP absorption in the opinion of the investigator.
+4. Clinically significant respiratory disease and/or cardiac disease (medical history or current clinical findings) in the opinion of the investigator.
+5. Prior interventional cardiac procedure (e.g., cardiac catheterization, angioplasty/percutaneous coronary intervention, balloon valvuloplasty, etc.) within 3 months prior to screening.
+6. QTcF \&gt; 450 msec (men) or QTcF \&gt; 470 msec (women).
+7. Structural heart disease based on cardiac MRI or Echocardiography (e.g., clinically significant valve disease; i.e., aortic or mitral valve stenosis or regurgitation) and/or abnormal conduction (QRS \&gt;120 msec, PR \&lt; 120 msec), and/or repolarization (QTcF \&gt; 450 msec (men) or QTcF \&gt; 470 msec (women)). Myocardial function (LVEF \&lt;52% in men and \&lt; 54% in women), symptomatic ischemic heart disease (inducible ischemia or coronary obstruction), and/or pathologic hypertrophy (e.g. \&gt; 15mm septal or posterior wall thickness), that is not well controlled under current specialized care. Subjects with congestive heart failure class II and above should also be excluded.
+8. Family history of unexplained/uninvestigated syncope or congenital long and short QT syndrome or sudden death (under the age of 60). ECG evidence of acute or recent ischemia, acute or Recent Myocardial Infraction, atrial fibrillation, high grade AV Blocks (Second Degree AV Block Type II or Third-degree AV Block), complete Heart Block or active conduction system abnormalities with the exception of any of the following:
+   1. First degree atrioventricular (AV)-block
+   2. Second degree AV-block Type 1 (Mobitz Type 1/Wenckebach type)
+   3. Right bundle branch block.
+9. History of acute heart failure (within the last 3 months).
+10. Higher degree of AV-blocks (AVB II° or III°).
+11. Other exclusion criteria per protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Learn More About How Safe Finerenone is, When it is Taken for a Longer Time With Standard Treatment, in Children and Young Adults With Heart Failure and Left Ventricular Systolic Dysfunction [NCT07192952]</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: Not specified – 18 Years  |  All
+Inclusion Criteria:
+* For participants rolling over from randomized controlled trial (RCT): Prior participation in the finerenone Phase 3 study FIORE (21466) and not permanently discontinued from the study intervention prior to the end of treatment (EoT) visit in FIORE.
+* For newly enrolled infants \&lt;6 months of age: Left ventricular systolic dysfunction (LVSD) with left ventricular ejection fraction (LVEF) ≤ 50% at screening assessed by echocardiography.
+* For newly enrolled infants \&lt;6 months of age: Elevated NT-pro BNP levels (\&gt; 500 mg/L) at screening.
+* For newly enrolled infants \&lt;6 months of age: Heart failure (HF) etiologies include congenital heart defects (CHD) with biventricular physiology and systemic LV; idiopathic cardiomyopathy (CM); familial/inherited and/or genetic CM; history of myocarditis (diagnosis of an acute episode at least 3 months prior to treatment assignment); neuromuscular disorder; inborn error of metabolism; mitochondrial disorder; acquired (chemotherapy, iatrogenic, infection, rheumatic, or nutritional); ischemic (e.g., Kawasaki disease and postoperative HF); LV noncompaction.
+* For newly enrolled infants \&lt;6 months of age: Receiving standard of care (SoC) treatment for heart failure according to local guidelines or investigator´s discretion (on a stable regimen for 30 days before baseline).
+* Newly enrolled newborns and infants \&lt; 6 months of age must have a body weight of ≥3 kg at Visit 1.
+Exclusion Criteria:
+* For participants rolling over from randomized controlled trial (RCT): To roll-over to FIORELLO, all participants: Potassium (K+) \&gt;5.5 mmol/L. After unblinding:
+  * For participants who received finerenone in FIORE: K+ \&gt;5.5 mmol/ L
+  * For participants who received placebo in FIORE: K+ \&gt;5.0 mmol/L for children ≥2 years of age, and \&gt;5.3 mmol/L for children \&lt;2 years of age (if eGFR is \&lt;60 mL/min/1.73m² for participants \&lt;2 years of age, the serum potassium threshold of \&gt;5.0 mmol/L will be used for exclusion)
+* For newly enrolled newborns and infants \&lt; 6 months of age: Potassium ≥ 5.3 mmol/l (if eGFR is \&lt;60 mL/min/1.73m², the serum potassium threshold of \&gt;5.0 mmol/L will be used for exclusion).
+* For participants rolling over from RCT: Severe renal dysfunction with estimated glomerular filtration rate (eGFR) \&lt; 30 ml/min/1.73m² at FIORE EoT or Visit 1.
+* For newly enrolled infants \&lt; 6 months of age: Severe renal dysfunction with eGFR \&lt; 30 ml/min/1.73m2 at screening or Visit 1.
+* Treatment with a mineralocorticoid receptor antagonist, other than the study intervention, (e.g., spironolactone, eplerenone) within 30 days of Visit 1.
+* Requirement of any intravenous (IV) vasoactive agents; mechanical ventilation; mechanical circulatory support; sustained or symptomatic arrhythmias not controlled by drug or device therapy within 30 days prior to study treatment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="36" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>ELEVATE-HFpEF Clinical Study [NCT06678841]</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 40 Years – Not specified  |  All
+Inclusion Criteria:
+1. Age ≥ 40 years
+2. Documented EF ≥50% within the preceding 12 months
+3. HFpEF defined as:
+   1. Documented worsening HF episode (either HF hospitalization or documented urgent clinic visit for HF with intravenous diuretics) within 12-months prior to baseline visit OR
+   2. Dyspnea on exertion and New York Heart Association (NYHA) ≥ class II symptoms AND AT LEAST ONE OF THE FOLLOWING CRITERIA:
+      * Interstitial / pulmonary edema on prior chest imaging in the last year AND current loop diuretic use for heart failure
+      * Elevated NT-proBNP in the last year defined as \&gt;400 pg/m for patients with no AF or paroxysmal AF, or \&gt;900 pg/ml for patients with ≥persistent AF
+      * Mean pulmonary capillary wedge pressure (PCWP) ≥15 mm Hg or LVEDP ≥16 mm Hg at rest on cardiac catheterization OR pulmonary artery diastolic and wedge pressure (PADP) ≥15 mm Hg at rest on implantable monitor (e.g., CardioMEMs)
+      * Echo criteria defined by ≥2 of:
+        * LV wall thickness ≥ 12 mm
+        * LV mass index (BSA indexed LVH): sex at birth male \&gt;115 g/m2, sex at birth female \&gt;95 g/m2
+        * Relative wall thickness ≥0.42
+        * E/e' ≥15 in sinus rhythm (or \&gt; 11 in the setting of atrial fibrillation) OR septal \&lt;7 cm/s or lateral e' \&lt;10cm/s
+        * Tricuspid regurgitation (TR) velocity \&gt;2.8 m/s
+        * Left atrial (LA) enlargement, defined by LA volume index \&gt;34 ml/m2
+4. Patient is on stable guideline indicated HF medical therapy (Class I recommendations) for at least 30 days
+5. Patient's average heart rate on baseline ambulatory electrocardiographic monitor is at least 5 bpm lower than their calculated personalized cardiac pacing rate (e.g. if a patient's personalized cardiac pacing rate is 70 bpm and their average heart rate on the ambulatory electrocardiographic monitor is less than or equal to 65 bpm the patient is eligible)
+6. Patient is willing and able to adhere to the protocol (e.g., patient is able to ambulate independently at baseline).
+Exclusion Criteria:
+1. Improved or recovered EF (i.e., prior LVEF\&lt;50%)
+2. Patient has a previously implanted, currently implanted, or is intended to have implanted a cardiac implantable electronic device capable of delivering pacing (e.g., pacemaker, implantable cardioverter defibrillator (ICD), cardiac resynchronization therapy (CRT))
+3. Current pregnancy (requirement for negative pregnancy test may vary by jurisdiction)
+4. Average heart rate \&lt;50 bpm or symptomatic bradycardia
+5. Acute coronary syndrome (including MI), cardiovascular surgery, or urgent percutaneous coronary intervention (PCI) within the 3 months prior to baseline visit or an elective PCI within 30 days prior to baseline visit.
+6. Current acute decompensated HF requiring intravenous diuretics, vasodilators and/or inotropic drugs.
+7. Severe obesity defined as BMI \&gt;45.
+8. Persistent, long-standing persistent, or permanent atrial fibrillation (AF) with an average heart rate \&lt;50 bpm or evidence of ventricular pauses exceeding 6 seconds
+9. Planned AF ablation
+10. Infiltrative cardiomyopathies (e.g., amyloidosis, sarcoidosis)
+11. Hypertrophic cardiomyopathies
+12. Uncontrolled hypertension as defined by BP \&gt;160/100 mmHg on two measurements ≥15 minutes apart
+13. End Stage Renal Disease (CKD 4 or greater)
+14. More than moderate valvular disease (e.g. exclude patients with moderate severe or severe valvular disease)
+15. Significant primary pulmonary disease on home oxygen
+16. Known contraindication for a pacemaker implant
+17. Advanced co-morbidity with life expectancy \&lt; 1 year
+18. Patients who are currently enrolled in a potentially confounding drug or device trial during the course of the study. Co-enrollment in concurrent trials is only allowed when documented pre-approval is obtained from the Medtronic Study Manager.
+19. Patient is a vulnerable adult (e.g. patient mentally incapable of giving consent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>A Study of VERVE-102 in Patients With Familial Hypercholesterolemia or Premature Coronary Artery Disease [NCT06164730]</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 70 Years  |  All
+Inclusion Criteria:
+* Diagnosis of HeFH or premature CAD
+Exclusion Criteria:
+* Homozygous familial hypercholesterolemia
+* Active or history of chronic liver disease
+* Current treatment with PCSK9 inhibitor or prior treatment within specified timeframe
+* Clinically significant or abnormal laboratory values as defined by the protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="36" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>A Phase 3 Study to Evaluate the Safety and Efficacy L606 in Participants With PH-ILD [NCT07285655]</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 80 Years  |  All
+Inclusion Criteria:
+* Participant is between 18 years to 80 years old.
+* Has a confirmed diagnosis of ILD based on High Resolution Computed Tomography (HRCT) chest imaging.
+* Evidence of PH as demonstrated from Right Heart Catheterization (RHC) with the following hemodynamic parameters:
+* Pulmonary vascular resistance (PVR) ≥ 320 dynes.sec/cm5 (i.e. 4 Woods Units (WU)), and
+* Mean Pulmonary Artery Pressure (mPAP) of ≥ 25 mmHg, and
+* \- Pulmonary capillary wedge pressure (PCWP) or Left-Ventricular End Diastolic Pressure (LVEDP) of ≤ 15 mmHg.
+* FEV1/FVC (ratio) \&gt; 0.70.
+* 6-minute walk distance ≥ 150 meters
+Exclusion Criteria:
+* PH in the updated WHO Classification Groups 1, 2, 4, or 5.
+* Has evidence of clinically significant left-sided heart disease as defined by echocardiography.
+* Participants with history of persistent/permanent or uncontrolled atrial fibrillation.
+* Participants with severe obstructive sleep apnea.
+* Has experienced exacerbation of underlying lung disease or active respiratory infection requiring antibiotics.
+* Initiation of pulmonary rehabilitation.
+Note: Other protocol defined inclusion/exclusion criteria may apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="36" customHeight="1">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>A Study to See if Lepodisiran Can Reduce Plaque in Coronary Arteries of Adults With Elevated Lp(a) Who Have Had Heart Events or Are at High Risk [NCT07613294]</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 45 Years – 80 Years  |  All
+Inclusion Criteria:
+* Have an Lp(a) ≥175 nmol/L
+* Have established cardiovascular (CV) disease or are at risk for a first CV event
+* Have angiographic evidence of coronary artery disease on screening CCTA
+* If taking lipid-lowering medications, inclusive of statins or prescription strength niacin and PCSK9 inhibitors, these should be stable for 8 weeks
+Exclusion Criteria:
+* Have had a major CV event less than 60 days before measurement of the Lp(a) level used for eligibility or uncontrolled high blood pressure at screening
+* Have moderate to severe renal dysfunction
+* Have severe heart failure
+* Have a history of coronary artery bypass graft surgery (CABG)
+* Have a planned coronary angiography, percutaneous coronary intervention (PCI), coronary artery bypass graft, or valvular intervention
+* Have had a procedure to remove lipoproteins from the blood or received therapy specifically targeting Lp(a)
+* Are unable to safely undergo CCTA due to medication intolerance, contrast allergies, or anatomical/technical factors</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="36" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Acoramidis Transthyretin Amyloidosis Prevention Trial in the Young (ACT-EARLY) Study in Asymptomatic Carriers of a Pathogenic TTR Variant [NCT06563895]</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 75 Years  |  All
+Key Inclusion Criteria:
+* Male or female ≥ 18 to ≤ 75 years of age inclusive.
+* Participants must have an established genotype (hetero- or homozygosity) through a medically-indicated genetic test of a TTR gene variant that is known to be pathogenic or likely pathogenic (eg, V30M/p.V50M, V122I/p.V142I, T60A/p.T80A, or all other pathogenic TTR variants).
+* Participant's age is within 10 years younger than or older than PADO.
+Key Exclusion Criteria:
+* Evidence of ATTR-CM or ATTR-PN.
+* Current or past (within last 1 to 12 months, depending on specific agent) treatment with other TTR modifying therapies.
+* Contraindication to or inability to undergo cardiac magnetic resonance testing.
+* Major organ dysfunction, including: kidney disease, liver disease, heart disease (including cardiomyopathy), neuropathy
+* Other diseases or conditions such has cancer within 5 years, untreated hyperthyroidism or hypothyroidism, type 1 diabetes, active hepatitis B or C, HIV.
+* Major surgery within the past 3 months or planned during the next 12 months.
+* Known hypersensitivity to acoramidis.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3315,13 +3941,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B16"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3365,6 +3994,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3413,6 +4043,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3424,8 +4055,13 @@
           <t>25-Jun 12:37</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>A Pan-European Post-Authorisation Safety Study: Risk of Pancreatic Cancer Among Type 2 Diabetes Patients Who Initiated Exenatide as Compared With Those Who Initiated Other Non-Glucagon-Like Peptide 1 Receptor Agonists Based Glucose Lowering Drugs [NCT05663515]</t>
@@ -3454,7 +4090,31 @@
 7. One or more prescriptions (or dispensed prescriptions) of DPP-4i (incretin mimetics) on or prior to the index date.</t>
         </is>
       </c>
-    </row>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 99 Years  |  All
+For inclusion in either exposure group, all of the following inclusion criteria must be fulfilled:
+1. Aged 18 years or older at the index date
+2. Individual level data on prescriptions, diagnoses and medical history is available for a minimum of 12 months prior to the index date
+3. A diagnosis of T2DM on index date or prior to index date
+For inclusion in the overall exenatide exposure group, the following criterion must be fulfilled:
+1. One incident prescription (or incident dispensed prescription) for exenatide (BYETTA or BYDUREON/ BYDUREON BCise) between the start and 12 months before the end of the study period. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+   For inclusion in the BYDUREON/ BYDUREON BCise exposure group, for the analyses of the secondary objective, the criterion a) is substituted with criterion b):
+2. One incident prescription (or incident dispensed prescription) for BYDUREON/ BYDUREON BCise between the start and 12 months before the end of the study period. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+   For inclusion in the comparator group, the following criterion must be fulfilled:
+3. One incident prescription (or incident dispensed prescription) of a GLD between the start and 12 months before the end of the study period. The GLD must not be a DPP-4i, a GLP-1 RA, or a combination with either a DPP-4i or a GLP-1 RA. This incident prescription must have succeeded a prescription of a GLD of another drug class during the baseline period.
+Patients are not eligible for any of the study population groups if they fulfil any of the following exclusion criteria:
+1. A diagnosis of type 1 diabetes mellitus (T1DM) on index date or a diagnosis of T1DM during the baseline period that is not succeeded by a T2DM diagnosis during the remaining part of the baseline period.
+2. A diagnosis of gestational diabetes during the baseline period or on index date.
+3. A diagnosis of polycystic ovarian syndrome during the baseline period or on index date in combination with exposure to metformin (Anatomical Therapeutic Chemical Classification System (ATC) code of the World Health Organization (WHO): A10BA02) as the only GLD on index date or during the baseline period.
+4. History of any cancer on or prior to index date. The only exception is that nonmelanoma skin cancer does not lead to exclusion.
+5. History of any acute pancreatitis, other diseases of the pancreas, or disorders of the pancreas on or prior to index date.
+6. One or more prescriptions (or dispensed prescriptions) of a GLP-1 RA (incretin mimetics) other than exenatide on or prior to index date.
+7. One or more prescriptions (or dispensed prescriptions) of DPP-4i (incretin mimetics) on or prior to the index date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -3528,6 +4188,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -3562,6 +4223,116 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>KHENERFIN Study: A Trial to Evaluate the Efficacy and Safety of Sonlicromanol in Primary Mitochondrial Diseases [NCT06451757]</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion criteria
+1. Signed Informed Consent
+2. Males and females aged ≥18 years with a multi-system primary mitochondrial disease.
+3. A confirmed mitochondrial DNA tRNALeu(UUR) m.3243A\&gt;G mutation (m.3243A\&gt;G PMD) plus an age adjusted heteroplasmy percentage ≥ 20% in white blood cells \[=blood heteroplasmy/0.977(age+12)\]. Or in urine (urinary epithelial cells), or buccal smear or skeletal muscle (results (obtained per local guidance) ≥ 20% must be available prior to the subject being randomized).
+4. Presence of chronic fatigue (not attributable to other etiologies than PMD):
+   1. Patient self-reported chronic fatigue for at least 3 months prior to the Screening Visit and recorded in the clinical patient files; AND
+   2. Presence of fatigue (raw total score \&gt;22), assessed by Neuro-QoL SFv1-F at Screening.
+5. Presence of mitochondrial myopathy defined as:
+5xSST at Screening and Baseline should be ≥ 11 seconds and participant must demonstrate the ability to complete the test at baseline (i.e., complete the test within 30 seconds).
+6\. Other Inclusion criteria per protocol.
+Exclusion criteria
+1. Treatment with any IMP within 3 months (or 5 times the half-life of the IMP, whichever is longer) prior to screening or plans to use an IMP (other than the study intervention) during the study.
+2. Bone deformities, motor abnormalities or chronic ulcers that in the opinion of the PI may interfere with and/or confound the interpretation of the subject's performance during the 5 times sit to stand test (5XSST).
+3. Surgery of gastrointestinal tract that might interfere with drug absorption. Or severe GI dysmotility, chronic vomiting, diarrhea, bouts of pseudo-obstruction which will impair appropriate IMP absorption in the opinion of the investigator.
+4. Clinically significant respiratory disease and/or cardiac disease (medical history or current clinical findings) in the opinion of the investigator.
+5. Prior interventional cardiac procedure (e.g., cardiac catheterization, angioplasty/percutaneous coronary intervention, balloon valvuloplasty, etc.) within 3 months prior to screening.
+6. QTcF \&gt; 450 msec (men) or QTcF \&gt; 470 msec (women).
+7. Structural heart disease based on cardiac MRI or Echocardiography (e.g., clinically significant valve disease; i.e., aortic or mitral valve stenosis or regurgitation) and/or abnormal conduction (QRS \&gt;120 msec, PR \&lt; 120 msec), and/or repolarization (QTcF \&gt; 450 msec (men) or QTcF \&gt; 470 msec (women)). Myocardial function (LVEF \&lt;52% in men and \&lt; 54% in women), symptomatic ischemic heart disease (inducible ischemia or coronary obstruction), and/or pathologic hypertrophy (e.g. \&gt; 15mm septal or posterior wall thickness), that is not well controlled under current specialized care. Subjects with congestive heart failure class II and above should also be excluded.
+8. Family history of unexplained/uninvestigated syncope or congenital long and short QT syndrome or sudden death (under the age of 60). ECG evidence of acute or recent ischemia, acute or Recent Myocardial Infraction, atrial fibrillation, high grade AV Blocks (Second Degree AV Block Type II or Third-degree AV Block), complete Heart Block or active conduction system abnormalities with the exception of any of the following:
+   1. First degree atrioventricular (AV)-block
+   2. Second degree AV-block Type 1 (Mobitz Type 1/Wenckebach type)
+   3. Right bundle branch block.
+9. History of acute heart failure (within the last 3 months).
+10. Higher degree of AV-blocks (AVB II° or III°).
+11. Other exclusion criteria per protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>29-Jun 16:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Frexalimab in Preservation of Endogenous Insulin Secretion Compared to Placebo in Adults, Adolescents and Children on Top of Insulin Therapy (FABULINUS) [NCT06111586]</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 6 Years – 35 Years  |  All
+Inclusion Criteria:
+* Participants who meet the criteria of T1D according to American Diabetes Association
+* Initiated exogenous insulin replacement therapy not longer than 90 days prior to screening visit at which random C-peptide will be assessed (V1).
+* Receiving at least one of the following T1D standard of care (SOC), insulin hormone replacement therapy
+  * one or multiple daily injections (MDI) of basal insulin, prandial insulin and/or premixed insulin, or
+  * continuous subcutaneous insulin infusion (CSII)
+* Participants must be positive for at least 1 of the following T1D autoantibodies confirmed by medical history and/or obtained at study screening:
+  * Glutamic acid decarboxylase (GAD-65)
+  * Insulinoma Antigen-2 (IA-2)
+  * Zinc-transporter 8 (ZnT8) or
+  * Insulin (if obtained not later than 10 days after exogenous insulin therapy initiation)
+* Have random C-peptide levels ≥ 0.2 nmol/L determined at screening visit.
+* Be vaccinated according to the local vaccination schedule. Any vaccinations should take place at least 28 days prior to randomization for non-live vaccines and at least 3 months prior to randomization for live vaccines.
+* Contraceptive use by men and women should be consistent with local regulations regarding the methods of contraception for those participating in clinical studies
+* Participants body weight at screening must be at least 20kg.
+Exclusion Criteria:
+* Serious systemic viral, bacterial or fungal infection (eg, pneumonia, pyelonephritis), infection requiring hospitalization or IV antibiotics or significant chronic viral (including history of recurrent or active herpes zoster, acute or active cytomegalovirus (CMV), Epstein-Barr Virus (EBV) as determined at screening), bacterial, or fungal infection (eg, osteomyelitis) 30 days before and during screening.
+* Participants with a history of invasive opportunistic infections, such as, but not limited to histoplasmosis, listeriosis, coccidioidomycosis, candidiasis, pneumocystis jirovecii, and aspergillosis, regardless of resolution.
+* Evidence of active or latent tuberculosis (TB) as documented by medical history and examination, chest X-rays (posterior anterior and lateral), and/or TB testing. Blood testing (eg, QuantiFERON® TB Gold test) is strongly preferred; if not available, any local approved TB test is allowed.
+* Evidence of any clinically significant, severe or unstable, acute or chronically progressive, uncontrolled infection, medical or surgical condition (eg, but not limited to, cerebral, cardiac, pulmonary, renal, hepatic, gastrointestinal, neurologic, acquired or inherited bone/skeletal disorders including repeated bone fractures for unknown reason, juvenile osteoporosis, osteogenesis imperfecta, osteochondropathies, or any known immune deficiency), or any condition that may affect participant safety in the judgment of the Investigator (including vaccinations which are not updated based on local regulation).
+* History or current hypogammaglobulinemia.
+* History of a systemic hypersensitivity reaction or significant allergies, other than localized injection site reaction, to any humanized mAb. Clinically significant multiple or severe drug allergies, intolerance to topical corticosteroids, or severe post-treatment hypersensitivity reactions (including, but not limited to, erythema multiforme major, linear IgA dermatosis, toxic epidermal necrolysis, and exfoliative dermatitis).
+* Has other autoimmune diseases (eg, rheumatoid arthritis \[RA\], polyarticular juvenile idiopathic arthritis \[pJIA\], psoriatic arthritis \[PsA\], ankylosing spondylitis \[AS\], MS, SLE), that require treatment with biologic drugs (mono or polyclonal antibodies) or systemic corticosteroid therapy (at discretion of investigator).
+* History, clinical evidence, suspicion or significant risk for thromboembolic events, as well as myocardial infarction, stroke, antiphospholipid syndrome, other prothrombotic disorders and/or participants requiring antithrombotic treatment.
+* Diabetes of forms other than autoimmune T1D that include but is not limited to genetic forms of diabetes, maturity-onset diabetes of the young (MODY), latent autoimmune diabetes of the adult (LADA), secondary to medications or surgery, type 2 diabetes by judgement of the investigator.
+* History of malignancy of any organ system, treated or untreated, within 5 years of screening, regardless of whether there is evidence of local recurrence or metastases.
+* Systemic corticosteroids (duration \&gt; 7 days), adrenocorticotropic hormone 1 month prior to screening.
+* Any IV, IM or SC administered biologic treatments, \&lt; 3 months or \&lt; than 5 half-lives (whichever is longer), prior to randomization.
+* Any live (attenuated or viral-vector) vaccine (including but not limited to varicella zoster, oral polio, nasal influenza, rabies) within 3 months prior to randomization.
+* Any non-live (inactivated, mRNA, recombinant, conjugate, toxoid) vaccine administered less than 28 days prior to randomization.
+* Other medications not compatible or interfering with IMP at discretion of investigator.
+* Any immunosuppressive therapy within 12 weeks prior to randomization.
+* Course of Thymoglobulin®, teplizumab or other immunomodulatory treatments at any time.
+* Any drugs that may be used for treatment of T1D and type 2 diabetes other than insulin including but not limited to metformin, glucagon-like peptide 1 (GLP-1) agonists and sodium-glucose co-transporter-2 and 1 (SGLT2/1) inhibitor and verapamil within 2 weeks prior to screening.
+* Abnormal laboratory test(s) at screening.
+The above information is not intended to contain all considerations relevant to a patient's potential participation in a clinical trial.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitor update 2026-06-29 18:21 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -3941,7 +3941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A3:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3949,8 +3949,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3994,7 +3992,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -4043,7 +4040,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -4114,7 +4110,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -4188,7 +4183,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -4223,7 +4217,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Monitor update 2026-06-30 12:28 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B94"/>
+  <dimension ref="A3:B118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2549,6 +2549,334 @@
         </is>
       </c>
     </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="36" customHeight="1">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Efficacy and Safety of Standard-of-Care Chemotherapy and Bevacizumab With or Without INCA33890 in the First-Line Treatment of Metastatic Microsatellite Stable Colorectal Cancer [NCT07284849]</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Stage IV colorectal adenocarcinoma not amenable to curative resection.
+* No prior systemic treatment for unresectable or metastatic disease. Participants who received adjuvant or neoadjuvant therapy may enroll if there was no recurrence within 12 months of the end of treatment.
+* Measurable disease per RECIST v1.1.
+* ECOG performance status of 0 or 1.
+* Adequate organ function determined by laboratory results.
+Exclusion Criteria:
+* MSI-H/dMMR per historical data in the medical record.
+* BRAF V600E mutation per historical data in the medical record.
+* Untreated and/or progressing CNS metastases.
+* History of other malignancy within 2 years.
+* Treatment with an anti-PD-(L)1 or other immune checkpoint inhibitor for any indication within the last 3 years.
+* Active autoimmune disease that has required systemic treatment in the past 2 years.
+* Significant concurrent and/or uncontrolled medical condition.
+* History of organ transplant, including allogeneic stem cell transplantation.
+Other protocol-defined inclusion/exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="36" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Phase Ib/II Platform Study of Multiple Anti-Cancer Agents in Participants With Metastatic Prostate Cancer [NCT07590934]</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 99 Years  |  Male
+Inclusion Criteria:
+1. Participants with a diagnosis of histologically confirmed adenocarcinoma of the prostate (no small cell, neuroendocrine, sarcomatoid, spindle or signet cell).
+2. Minimum life expectancy of 3 months or more.
+3. Eastern Cooperative Oncology Group (ECOG) performance status of O or 1 at screening, with no deterioration.
+4. PCWG3 (Prostate Cancer Working Group 3) modified RECIST Version 1.1 evaluable disease.
+5. Must have received at least one novel androgen receptor pathway inhibitor (ARPI), such as enzalutamide or darolutamide or apalutamide or abiraterone acetate.
+6. Must have one or more unresectable metastatic lesions.
+7. Must have had prior orchiectomy and/or ongoing androgen deprivation therapy, and a castrate level of serum testosterone (\&lt;50ng/dL or \&lt;l.7nmol/L).
+8. Progressive metastatic castration-resistant prostate cancer (mCRPC) following the most recent treatment at time of study entry.
+9. Adequate organ and marrow function.
+10. Non sterilised participants who are sexually active with a partner of childbearing potential must use a condom (plus spermicide, if available), must refrain from fathering a child, freezing or donating sperm, and it is recommended for the partner to also use a highly effective contraceptive method.
+Inclusion Criteria for Sub study 1:
+1. Must have received a single line of ARPI, such as enzalutamide, darolutamide, apalutamide or abiraterone acetate.
+2. PSMA positive mCRPC by computed tomography positron emission tomography, obtained with PSMA ligand defined as at least 1 PSMA positive metastatic lesion with tracer uptake greater than liver, and no PSMA negative lesions. All measurable or intraprostatic lesions must be PSMA positive.
+3. Capable of self-administering oral formulations.
+Exclusion Criteria:
+1. Any evidence of non adenocarcinomatous forms of prostate cancer (including small cell, spindle cell, signet cell, neuroendocrine, sarcomatous).
+2. Known, unresolved urinary tract obstruction.
+3. Participants with a history of central nervous system metastases.
+4. Symptomatic malignant spinal cord compression or findings indicative of impending cord compression.
+5. Participants with a history of leptomeningeal carcinomatosis.
+6. Previous or concurrent cancer distinct from the cancer under investigation in primary site or histology .
+7. Concurrent serious medical conditions.
+8. Previous history of interstitial lung disease or non-infectious pneumonitis.
+9. Participants with a history or clinical/laboratory features suggestive of myelodysplastic syndrome or acute myeloid leukaemia.
+10. Persistent toxicities caused by previous therapy.
+11. Participants unable to swallow orally administered medications or with gastrointestinal disorders likely to interfere with absorption.
+12. Active infection, including tuberculosis, hepatitis C virus, and hepatitis B virus infection.
+13. Known hypersensitivity to study intervention or any of their excipients.
+Exclusion Criteria for Sub study 1:
+1. History of uncontrolled seizures or requirement for \&gt;2 antiepileptic drugs.
+2. History of severe brain injury or stroke.
+3. Skeletal metastases demonstrating a superscan appearance on bone scan.
+4. Participants have received prior therapy with AZD9574 or more than 1 prior line of any other Poly-ADP-ribose polymerase inhibitor (PARPi)-based regimen (either as a treatment or as maintenance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="36" customHeight="1">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>A Study of SNDX-5613 in Combination With Intensive Chemotherapy in Participants With Acute Myeloid Leukemias [NCT06226571]</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 75 Years  |  All
+Inclusion Criteria:
+* Established, pathologically confirmed diagnosis of AML by World Health Organization 2022 criteria.
+* Previously untreated AML and eligible to receive intensive chemotherapy.
+* KMT2Ar, NPM1c, or NUP98r mutations identified by local laboratory prior to the first dose of SNDX-5613.
+* Eastern Cooperative Oncology Group performance status ≤2 and ≤1 if \&gt;65 years old .
+* Adequate liver, kidney, and cardiac function.
+Exclusion Criteria:
+* Diagnosis of acute promyelocytic leukemia.
+* Clinically active central nervous system leukemia (blasts detected in cerebrospinal fluid, radiographic or clinical signs and symptoms).
+* Fridericia's corrected QT interval (QTcF) \&gt;450 milliseconds (average of triplicate), diagnosis or suspicion of Long QT syndrome or family history of Long QT syndrome.
+* Any gastrointestinal issue of the upper gastrointestinal tract that might affect oral drug absorption or ingestion.
+* Cirrhosis with a Child-Pugh score of B or C.
+* Any of the following within the 6 months prior to study entry: myocardial infarction, uncontrolled/unstable angina, congestive heart failure (New York Heart Association Classification Class ≥II), life-threatening, uncontrolled arrhythmia, cerebrovascular accident, or transient ischemic attack.
+* Hepatitis B, Hepatitis C, or HIV-positive with detectable viral load.
+* Documented active, uncontrolled infection.
+* Uncontrolled disseminated intravascular coagulation.
+* Lactating/breast feeding or pregnant.
+* Use of prohibited concomitant chemotherapy, radiation therapy, or immunotherapy.
+* Use of strong CYP3A4 inducers or inhibitors (except for Itraconazole, Ketoconazole, Posaconazole, or Voriconazole).</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="36" customHeight="1">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>Study to Evaluate Adverse Events and Efficacy of Intravenous (IV) Telisotuzumab Adizutecan in Combination With a PD-1 Immune Checkpoint Inhibitor in Adult Participants With Advanced or Metastatic Non-Squamous NSCLC With No Prior Treatment for Advanced Disease, and No Actionable Genomic Alterations [NCT06772623]</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Must have histologically documented non-squamous (NSq) non small cell lung carcinoma (NSCLC) that is locally advanced or metastatic will be enrolled into the study.
+* Must have measurable disease per response evaluation criteria in solid tumors (RECIST) v1.1.
+* For Part 1, participants must have had no more than 1 systemic therapy for advanced disease including platinum-based chemotherapy or an immune checkpoint inhibitor (as monotherapy or in combination with chemotherapy), or appropriate targeted therapy for an actionable gene alteration, if applicable, for epidermal growth factor receptor (EGFR) wild-type (WT) NSq NSCLC.
+* For Part 2, participants must have no prior systemic therapy for advanced disease, no known actionable genomic alteration.
+* Must have documented programmed death ligand 1 (PD-L1) status.
+* For Part 2, participant must have evaluable c-Met immunohistochemistry (IHC) result per central testing prior to randomization.
+* Must have adequate organ function.
+Exclusion Criteria:
+* Known uncontrolled metastases to the central nervous system.
+* History of interstitial lung disease (ILD) or pneumonitis that required treatment with systemic steroids, or any evidence of active ILD or pneumonitis on screening chest computed tomography (CT) scan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="36" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>A Clinical Study of the Anti-cancer Effects of an Investigational Therapy or Chemotherapy in Patients With Recurring Uterine Cancer [NCT06340568]</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  Female
+Key Inclusion Criteria:
+* Are female adults (defined as ≥18 years of age or acceptable age according to local regulations at the time of voluntarily giving informed consent).
+* Have histologically confirmed endometrial cancer that:
+  * Is recurrent,
+  * Has a HER2 IHC score of 1+, 2+ (Cohort 1), or 3+ (Cohort 2) as determined by central laboratory testing for HER2 expression, and
+  * Is not defined as a true sarcoma (i.e., leiomyosarcoma or endometrial stromal sarcoma). Note: Uterine carcinosarcoma is allowed.
+* Have measurable disease defined by RECIST v1.1.
+* Have Eastern Cooperative Oncology Group (ECOG) Performance Status of 0, 1 or 2.
+* Have recurrent endometrial cancer and meet any of the following:
+  * developed recurrence \&lt;12 months from completing platinum-based chemotherapy given as adjuvant therapy for Stage I to III disease, or
+  * developed recurrence after platinum-based chemotherapy in the recurrent/metastatic setting.
+* Have received prior ICI treatment (i.e., anti-programmed death 1/anti-programmed death-ligand 1)
+* Have a life expectancy of ≥12 weeks at screening.
+Key Exclusion Criteria:
+* Are ineligible for all options in the investigator's choice of chemotherapy arm, per local prescribing information and institutional guidelines (applicable to Cohort 1 only).
+* Have a history of small bowel obstruction requiring hospitalization within the past 3 months prior the first dose of study treatment.
+* Have an uncontrolled intercurrent illness that would limit compliance with study requirement or substantially increase risk of incurring adverse events.
+* Have clinically uncontrolled pleural effusion, ascites or pericardial effusion requiring drainage, or peritoneal shunt within 2 weeks prior to the first dose of study treatment.
+* Have a history of (non-infectious) interstitial lung disease (ILD)/pneumonitis that required steroids, have current ILD/pneumonitis, or where suspected ILD/pneumonitis cannot be ruled out by imaging at screening.
+* Participants with prior use of immunosuppressive medication within 14 days prior to the first dose of study treatment, except for intranasal and inhaled corticosteroids or systemic corticosteroids at doses of less than 10 mg/day of prednisone or equivalent, and topical corticosteroids. Participants receiving corticosteroids may continue if the dose is stable upon giving main informed consent.
+* Have a lung-specific intercurrent clinically significant illness including, but not limited to, any underlying pulmonary disorder (e.g., pulmonary emboli within 3 months prior to the first dose of study treatment, severe asthma, chronic obstructive pulmonary disorder with moderate acute exacerbations, restrictive lung disease, pulmonary fibrosis, radiation pneumonitis, significant pleural effusion etc.), or any autoimmune, connective tissue or inflammatory disorder with pulmonary involvement (i.e., rheumatoid arthritis, Sjogren's syndrome, sarcoidosis etc.), and/or prior pneumonectomy (complete).
+* Have uncontrolled infection requiring systemic antibiotics, antivirals, or antifungals within 2 weeks prior to the first dose of study treatment.
+* Have unresolved toxicities from previous anti-cancer therapy, defined as toxicities (other than alopecia, fatigue, or endocrinopathies that are well controlled) not yet resolved to Grade ≤1 or baseline.
+* Are pregnant or breastfeeding or are planning pregnancy during the study or within 7 months after the last dose of study treatment.
+* Have a history of allergies, hypersensitivities, or intolerance to study treatments (investigational medicinal products and auxiliary medicinal product) including any excipients thereof or to other monoclonal antibodies. Participants who have successfully undergone a desensitization process and are able to tolerate the drug are eligible.
+* Had prior treatment with topoisomerase I inhibitors, including ADCs.
+* Have left ventricular ejection fraction \&lt;55% by either echocardiography or multiple-gated acquisition within 28 days prior to the first dose of study treatment. This includes participants with tissue doppler E/e' ratio \&gt;15.
+NOTE: Other protocol defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="36" customHeight="1">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>The Ailliance Post-Market Clinical Study [NCT05856370]</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Subject provides written informed consent per institution and/or geographical requirements.
+2. Subject is intended to receive or be treated with an eligible Medtronic Cranial and Spinal Technology (CST) device(s) (see product appendices), used alone or in combination, for a cranial and/or spinal indication(s).
+3. Subject is at least 18 years of age or minimum legal age as required by local regulations.
+4. Subject agrees to complete all required assessments per the Schedule of Events.
+Exclusion Criteria:
+1. Subject is currently enrolled or plans to enroll in concurrent drug/device/biologic trial(s) that may confound this trial's results per investigator assessment (i.e. no required intervention that could affect interpretation of all-around device safety and or performance).
+2. Subject who is, or is expected to be, inaccessible for all required follow-up visits.
+3. Subject with exclusion criteria required by local law.
+4. Subject is considered vulnerable at the time of obtaining consent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="36" customHeight="1">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>European Real-World Registry for Use of the Ion Endoluminal System [NCT06923774]</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Patient is aged 18 years or older at time of consent.
+* Patient is planned to undergo a lung lesion biopsy(s) and/or localization procedure(s) utilizing the Ion endoluminal system.
+* Patient is willing and able to give written informed consent for clinical study participation.
+Exclusion Criteria:
+* Patient is participating in an interventional research study or research study with investigational agents with an unknown safety profile that would interfere with participation in this study or study results.
+* Female patient that is pregnant or breast feeding as determined by standard site practices.
+* Patient is legally incapacitated or in a legal/court ordered institution or is part of a known vulnerable population, including but not limited to dependency on the sponsor, hospital or study doctor.
+* Patient is not willing to comply with post-procedure study participation requirements.
+* Investigator, in their professional opinion, has decided that it is in the patient's best interest to not participate in the clinical study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="36" customHeight="1">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Compare the Efficacy and Safety of BMS-986489 (BMS-986012+ Nivolumab Fixed Dose Combination) in Combination With Carboplatin Plus Etoposide to That of Atezolizumab With Carboplatin Plus Etoposide as First-Line Therapy in Participants With Extensive-Stage Small Cell Lung Cancer (TIGOS). [NCT06646276]</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Participants must have diagnosis of Extensive-Stage Small Cell Lung Cancer (ES-SCLC).
+* Participants must be Healthy enough to do their normal activities with little or no help based on the ECOG performance scale.
+* Participants must have at least one tumor that can be measured using special imaging techniques like a CT scan or MRI at a site other than the brain and nervous system
+Exclusion Criteria
+* Participants have already received certain types of treatment for extensive stage small cell lung cancer
+* Participants have certain health conditions, like spread of small cell lung cancer to the brain that are causing symptoms, certain lung diseases, heart diseases, infections, autoimmune diseases, other cancers, or a type of nerve damage called peripheral sensory neuropathy
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2560,7 +2888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C88"/>
+  <dimension ref="A3:C112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3930,6 +4258,361 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="36" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>A Study of Navenibart in Participants With Hereditary Angioedema [NCT06842823]</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 12 Years – Not specified  |  All
+Inclusion Criteria:
+* Documented diagnosis of HAE (Type 1 or 2). The following must be met:
+  1. Documented clinical history consistent with HAE
+  2. Lab findings consistent with HAE Type 1 or 2
+* Experienced at least 2 HAE attacks during the Run-In period, as confirmed by an investigator based on meeting the protocol-specified definition of an HAE attack.
+Exclusion Criteria:
+* Any concomitant diagnosis of another form of chronic angioedema, such as acquired C1 inhibitor deficiency, HAE with normal C1-INH (also known as HAE type 3), idiopathic angioedema, or angioedema associated with urticaria.
+* Use of therapies prescribed for the prevention of HAE attacks may not be used during the trial or within the below time frames prior to the Run-In Period (adult participants may be on these medications at the time of the Screening Visit, but will need to washout prior to entering the Run-In Period).
+  1. Tranexamic acid, oral danazol, oral stanazolol, and oral oxandrolone within 3 days prior to Run-In
+  2. Plasma-derived C1INH for LTP within 14 days prior to Run-In
+  3. Berotralstat within 21 days prior to Run-In
+  4. Lanadelumab within 70 days prior to Run-In
+  5. Garadacimab within 90 days prior to Run-In</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="36" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>A Research Study to Look at How Well NNC0487-0111 Works Compared to Placebo in People With Heart Failure and Obesity [NCT07567001]</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Body Mass Index (BMI) greater than or equal to (\&gt;=) 30 kilograms per square metre (kg/m\^2) at screening.
+* Diagnosis of HF with New York Heart Association (NYHA) class II-IV and in stable condition at screening, at the discretion of the investigator.
+For participants with Type 2 Diabetes (T2D) at screening:
+\- Diagnosed with T2D \&gt;= 30 days before screening.
+Exclusion Criteria:
+* MI, stroke, unstable angina pectoris or worsening HF leading to either hospitalization or intravenous loop diuretics within 30 days prior to the day of screening and until randomization.
+* HF due to infiltrative cardiomyopathy (e.g., sarcoid, amyloid), arrhythmogenic right ventricular cardiomyopathy, Takutsubo cardiomyopathy, Chagas cardiomyopathy, genetic hypertrophic cardiomyopathy or obstructive cardiomyopathy, active myocarditis, constrictive pericarditis, cardiac tamponade, or uncorrected primary valve disease of moderate or severe degree.
+* Severe pulmonary disease including primary pulmonary hypertension, chronic pulmonary embolism, or severe chronic obstructive pulmonary disease (COPD) defined as:
+* requiring home oxygen; or - ongoing oral corticosteroid therapy; or - hospital for COPD Exacerbation within 12 months prior to screening.
+* Any other condition judged by the investigator to be the cause of HF symptoms (e.g., anaemia, hypothyroidism).
+Glycaemia-related:
+* History of type 1 diabetes.
+* Participant with diabetic retinopathy or maculopathy who received treatment with retinal photocoagulation, vitrectomy or anti-Vascular Endothelial Growth Factor (anti-VEGF) within 180 days before screening or who, at the time of screening, are expected to require treatment within 180 days after screening. Diabetic retinopathy or maculopathy must be verified by an eye examination performed within 90 days before screening or in the period between screening and randomization. Pharmacological pupil-dilation is a requirement unless using a digital fundus photography camera specified for non-dilated examination.
+* Glycated haemoglobin (HbA1c) greater than (\&gt;) 10 percent (%) (86 \[millimoles per mole\] mmol/mol) as measured by local or central laboratory at screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="36" customHeight="1">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Streamlined Denervation With spYral For an Optimized Treatment (SPYRAL SWYFT) in Subjects With Uncontrolled Hypertension [NCT07115953]</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Individual is diagnosed with hypertension and has a baseline office systolic blood pressure ≥140 mmHg
+2. Individual has a baseline office diastolic blood pressure ≥ 90 mmHg
+3. Individual has an average systolic baseline home blood pressure ≥135 mmHg (with ≥7 days of valid pre-procedure measurements)
+4. Individual has a valid 24-hour Ambulatory Blood Pressure Measurement at baseline
+Exclusion Criteria:
+1. Individual lacks appropriate renal artery anatomy
+2. Individual has undergone prior renal denervation
+3. Individual has a documented condition that would prohibit or interfere with ability to obtain an accurate blood pressure measurement
+4. Individual requires chronic oxygen support or mechanical ventilation other than nocturnal respiratory support for sleep apnea
+5. Individual has an estimated glomerular filtration rate (eGFR) of \&lt;45 mL/min/1.73m2
+6. Individual has one or more episode(s) of orthostatic hypotension
+7. Individual is pregnant, nursing or planning to become pregnant
+8. Individual has documented primary pulmonary hypertension
+9. Individual has documented type 1 diabetes mellitus or poorly-controlled type 2 diabetes mellitus with glycosylated hemoglobin greater than 8.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="36" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Low-carbohydrate Diet and Low-Density Lipoprotein - Cholesterol (LDL-c) Interindividual Variability [NCT07675603]</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Age: \&gt;18 years
+* Body mass index: 18.5-35 kg·m-2
+* Low-Density Lipoprotein-cholesterol \&lt;4.9 mmol/L
+* Non-fasting triglycerides \&lt;2.3 mmol/L
+Exclusion Criteria:
+* weight instability (\&gt;5% change in body mass within last 3 months)
+* smoker
+* diagnosis of hypercholesterolaemia or any other lipid-related disease
+* diagnosis of diabetes
+* diagnosis of atherosclerotic cardiovascular disease
+* elevated fasting glucose (\&gt;5.4 mmol/L)
+* dietary intolerances or allergies or to other study procedures
+* diagnosis of gastrointestinal disorders
+* any other condition/medication that could introduce bias to the study
+* already following a ketogenic diet
+* not willing to follow a ketogenic diet
+* unable to understand English language</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="36" customHeight="1">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>A Study Comparing AZD0120, a Dual-targeted CAR-T Against B-cell Maturation Antigen (BCMA) and CD19, Versus Standard Regimens in Participants With Relapsed Refractory Multiple Myeloma (DURGA-4) [NCT07391657]</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Age ≥ 18 years
+* Documented diagnosis of multiple myeloma according to the IMWG diagnostic criteria
+* Documented evidence of measurable disease:
+  1. Serum M-protein level ≥ 1 g/dL
+  2. Urine M-protein level ≥ 200 mg/24h
+  3. Serum immunoglobulin free light chain ≥ 10 mg/dL (100 mg/L) and abnormal serum immunoglobulin kappa lambda free light chain ratio
+* Documented evidence of PD by IMWG 2016 criteria based on investigator's determination during or after the most recent line of therapy. Participants with only 1 prior line of therapy must have progressed within 47 months of a stem cell transplant, or if not transplanted, then within 42 months of starting initial therapy
+* Received 1 to 3 lines of prior therapy including an IMiD and either a PI or a CD38 antibody. Participant must have undergone at least 2 complete cycles of treatment for each line of therapy, unless PD was the best response to the line of therapy
+* Eligible to receive at least one of the standard regimens (DKd, PVd, DPd, or Kd) as determined by the Investigator.
+* ECOG performance status score of 0 to 1
+* Adequate hematology and chemistry laboratory values:
+  1. Haemoglobin ≥ 8.0 g/dL
+  2. Absolute neutrophil count ≥ 1 × 10\^9/L (1000 per mm3)
+  3. Platelet count ≥ 75 × 10\^9/L (75000 per mm3) in participants with \&lt; 50% of bone marrow nucleated cells are plasma cells or ≥ 50 × 10\^9/L (50000 per mm3) in participants with ≥ 50% of bone marrow nucleated cells are plasma cells
+  4. Absolute lymphocyte count ≥ 300/µL (0.3 × 109/L)
+  5. Total bilirubin ≤ 1.5 × ULN in the absence of Gilbert's syndrome or ≤ 3 × ULN if the participant has Gilbert's syndrome. AST and ALT≤ 3.0 × ULN. CrCl by Cockcroft and Gault method ≥ 30 mL/minute
+Exclusion Criteria:
+* Known active, or prior history of CNS involvement or exhibits clinical signs of meningeal involvement of MM.
+* Primary amyloidosis, active plasma cell leukaemia, Waldenstrom macroglobulinemia or Polyneuropathy Organomegaly Endocrinopathy M-protein and Skin (POEMS) syndrome.
+* Participants with primary refractory MM (failed to generate at least a minimal response to any prior therapy)
+* Significant neurological or psychiatric condition
+* Significant medical condition that places the participant at an unacceptable risk for treatment-related complications
+* Previously received any prior BCMA-targeted treatment
+* Previously received CAR-T or CAR-NK therapy directed at any target
+* Previously received T-cell engager therapy directed at any target
+* Previously received allogeneic stem cell transplantation at any time during prior therapy or received autologous stem cell transplantation within 12 weeks of randomization</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="36" customHeight="1">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Test Whether BI 764524 Helps People With an Eye Condition Called Diabetic Retinopathy [NCT06321302]</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+General inclusion criteria
+* Diagnosis of diabetes mellitus (DM) under regular treatment with Haemoglobin A1c (HbA1c) (glycated haemoglobin) (HbA1c) \&lt;12%; DM should be under regular investigation by a trained specialist as per local standard of care prior to and during the trial
+* Age ≥18 years at time of signing Informed Consent Form (ICF)
+Ocular inclusion criteria: study eye
+* Moderate to severe non-proliferative diabetic retinopathy (NPDR) (Diabetic Retinopathy Severity Scale (DRSS) level 43 to 53) as assessed by Ultra-widefield colour fundus photography (UWF-CFP) images (within the 7-field grid) and confirmed by the central reading centre (CRC) at screening. Patient staged at DRSS level of 43 based on UWF-CFP images can be included only if:
+  * They are participating in the standard 7-field CFP sub-study of the trial, and
+  * They are staged as DRSS level of 47 to 53 on standard 7-field CFP imaging, as confirmed by the CRC at screening.
+* Ultra-widefield fluorescein angiography (UWF-FA) image gradable for presence of retinal non-perfusion (RNP) as confirmed by the CRC at screening
+* Visual acuity: best corrected visual acuity (BCVA) letter score of ≥49 letters (approximate Snellen equivalent of 20/100 or better) using ETDRS chart at starting distance of 4 meter (m) at screening and reconfirmed at baseline
+* Sufficiently clear ocular media, adequate pupillary dilation, and fixation to permit quality fundus imaging
+Main exclusion criteria in study eye:
+\- Evidence of active retinal neovascularisation (NV) on clinical exam and/or UWF-CFP images within the 7-field grid, confirmed by the CRC grading.
+The following are permitted if, based on the assessment of the investigator, do not require acute treatment:
+* Small neovascular lesions within the ETDRS 7-field that are detected only on UWF-FA, but not on clinical exam or UWF-CFP
+* Neovascularisations outside of the ETDRS 7-field on ultra-widefield imaging
+  * Evidence of active NV of the iris (small iris tufts are not an exclusion) or in the anterior chamber angle
+  * Prior pan-retinal photocoagulation (PRP). Peripheral scatter or targeted laser treatment in up to 1 quadrant outside the ETDRS 7-field area is permitted if it was performed at least 6 months prior to Day 1
+  * CI-DME, defined as central subfield thickness (CST) ≥320 micrometer (μm) as measured by Heidelberg Spectralis optical coherence tomography (OCT) and confirmed by central reading centre (CRC) at screening (equivalent measurements from other OCT machines may be accepted); participants with a CST of 320-330 μm can be included if, in the opinion of the investigator, the participant is not expected to require treatment for CI-DME during the duration of the study (e.g. no profound impact on BCVA, stable CST, etc.). CST must be re-confirmed at baseline. A CRC confirmation of the baseline CST is not required.
+  * Previous treatment in the study eye for NPDR and/or diabetic macular edema (DME) with intravitreal (IVT) anti-vascular endothelial growth factor (VEGF) (including anti-VEGF/Ang2) or short acting corticosteroid drugs (e.g. triamcinolone) within 6 months prior to Day 1 or \&gt;4 treatments within the last 18 months (referred to elsewhere as 'previous IVT treatment').
+  * Any previous IVT treatment other than anti-VEGF and short-acting steroids. Previous dexamethasone IVT drug delivery system (Ozurdex) or fluocinolone acetonide intravitreal implant (Iluvien) is not allowed
+  * Refractive error of more than -8 dioptres of myopia (spherical equivalent) in the study eye. For patients having undergone refractive or cataract surgery in the study eye, either the pre-operative refractive error or the axial length measurement should be used, at the investigator's discretion. Axial length should be less than 26 mm
+  * Any concurrent or past ocular condition in the study eye which, in the judgement of the investigator, could:
+* Require medical or surgical intervention during the study period to prevent or treat vision loss (e.g. advanced cataract, history of retinal detachment or macular hole (Stage 3 or 4) in the study eye)
+* Could likely contribute to a significant loss of BCVA during the study period if left untreated (e.g. advanced epiretinal membrane and/or vitreomacular traction, active or history of optic neuritis in either eye)
+* Contraindicate the use of the investigational drug, or may render the patient at high risk for treatment complications (e.g. active infectious or non-infectious conjunctivitis/keratitis in either eye; history of recurrent infectious or inflammatory ocular disease in either eye (e.g. uveitis)
+* May affect interpretation of the study results (e.g. central atrophy of the retinal pigment epithelium or photoreceptors; age-related macular degeneration, hereditary retinal degenerative diseases, myopic macular degeneration, past, current or planned use of medications known to be toxic to the retina, lens or optic nerve (e.g. deferoxamine, chloroquine/hydroxychloroquine, chlorpromazine, phenothiazines, tamoxifen, nicotinic acid, and ethambutol); history of central serous chorioretinopathy, ischemic optic neuropathy or retinal vascular occlusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="36" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>Neural Cardiac Therapy for Heart Failure Study (NECTAR-HF) [NCT01385176]</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Age 18 or above, and of legal age to give informed consent specific to national laws
+* Willing and capable of providing informed consent
+* Capable of participating in all testing associated with this clinical investigation
+* Stable symptomatic heart failure NYHA class II-III
+* Left ventricular (LV) ejection fraction equal or smaller than 35 %
+* Left ventricular end diastolic diameter (LVEDD) of 5.5 cm or greater
+* Prescribed to optimal pharmacologic therapy
+Exclusion Criteria:
+* QRS larger than 130 ms
+* Patients who have been hospitalized for heart failure and who required the use of HF IV therapy within 30 days before enrollment
+* Patients unable to tolerate anesthesia required for implant
+* Patients with unstable angina, myocardial infarction, PTCA, coronary artery bypass graft, cerebral vascular accident, or transient ischemic attack within previous 90 days before enrollment
+* Patients whose primary cause of heart failure is mitral or aortic valve disease, with a severe classification
+* Patients with persistent or permanent atrial fibrillation within 90 days prior to enrollment
+* Pacemaker indicated patients
+* Patients whose heart failure is due to congenital heart disease
+* Patients who have started treatment for sleep apnea or sleep disordered breathing with therapies to maintain airway patency (e.g., CPAP, Bi-PAP,APAP) with or without oxygen supplementation within the previous 6 months prior to enrollment
+* Patients with hypertrophic obstructive cardiomyopathy or infiltrative cardiomyopathy (e.g. amyloidosis, sarcoidosis)
+* Patients with documented chronic obstructive lung disease
+* Patients on or indicated for renal dialysis
+* Type 1 diabetic patients
+* Type 2 diabetic patients that have been treated with insulin for more than 5 years prior to enrollment
+* Patients with a life expectancy of less than 12 months per physician judgment
+* Patients involved in any concurrent clinical investigation
+* Women of childbearing potential who are or might be pregnant at the time of the study or breastfeeding
+* Patients with a prior cardiac transplant or expecting a heart transplant operation within the next 12 months
+* Patients with a prior vagotomy
+* Patients with prior or existing vagal nerve stimulation treatment
+* Patients implanted with any active implantable medical device other than a left sided single or dual chamber implantable cardioverter defibrillator (ICD) with bipolar sensing, or a left sided CRT device with each sensing channel programmed to either bipolar sensing or no sensing. All CRT patients must have had CRT for at least 1 year prior to enrollment. The total number of CRT patients will not exceed 30
+* Patients with locally implanted semi-/permanent devices such as vascular catheters, etc. that would interfere with the NECTAR-HF study system
+* Patients with previously implanted devices on the right side that became infected before removal
+* Patients with previous neck surgery and resultant scar formation that interferes with the ability to implant the study system on the right side of the neck (Thyroid/parathyroid, carotid artery etc)
+* Patients with known recurrent nerve paralysis
+* Patients who have undergone radiotherapy for thyroid disease/cancer
+* Patients who have existing or prior tracheotomy
+* Patients with severe vertebral cervical disease and limited mobility in the neck; includes those that frequently wear a brace
+* Patients with carotid murmur/vascular bruit/carotid artery lesion
+* Patients with known/suspected vascular malformation in carotid/vertebral circulatory bed
+* Patients who are likely to need an MRI of the neck area because of previous medical conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="36" customHeight="1">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>Impact of Personalised Cardiac Anaesthesia and Cerebral Autoregulation on Neurological Outcomes in Patients Undergoing Cardiac Surgery [NCT05595954]</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 65 Years – Not specified  |  All
+Inclusion Criteria:
+* Elective primary or reoperative coronary artery bypass graft and/or valvular and/or ascending aorta surgery requiring cardiopulmonary bypass.
+Exclusion Criteria:
+* Surgery requiring moderate (28-31.9ºC) or deep (\&lt;28ºC) hypothermic circulatory arrest;
+* Heart and/or lung transplantation;
+* Urgent (within 24 hours) and emergency surgery;
+* Inability to follow procedures or insufficient knowledge in English, German or French;
+* Inability to give consent.
+Participants who undergo cardiac surgery under minimal extracorporeal circulation will also be excluded.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3941,7 +4624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C22"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3949,6 +4632,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3992,6 +4677,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -4040,6 +4726,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -4110,6 +4797,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -4183,6 +4871,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -4217,6 +4906,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -4266,6 +4956,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -4326,6 +5017,129 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Streamlined Denervation With spYral For an Optimized Treatment (SPYRAL SWYFT) in Subjects With Uncontrolled Hypertension [NCT07115953]</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Individual is diagnosed with hypertension and has a baseline office systolic blood pressure ≥140 mmHg
+2. Individual has a baseline office diastolic blood pressure ≥ 90 mmHg
+3. Individual has an average systolic baseline home blood pressure ≥135 mmHg (with ≥7 days of valid pre-procedure measurements)
+4. Individual has a valid 24-hour Ambulatory Blood Pressure Measurement at baseline
+Exclusion Criteria:
+1. Individual lacks appropriate renal artery anatomy
+2. Individual has undergone prior renal denervation
+3. Individual has a documented condition that would prohibit or interfere with ability to obtain an accurate blood pressure measurement
+4. Individual requires chronic oxygen support or mechanical ventilation other than nocturnal respiratory support for sleep apnea
+5. Individual has an estimated glomerular filtration rate (eGFR) of \&lt;45 mL/min/1.73m2
+6. Individual has one or more episode(s) of orthostatic hypotension
+7. Individual is pregnant, nursing or planning to become pregnant
+8. Individual has documented primary pulmonary hypertension
+9. Individual has documented type 1 diabetes mellitus or poorly-controlled type 2 diabetes mellitus with glycosylated hemoglobin greater than 8.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Test Whether BI 764524 Helps People With an Eye Condition Called Diabetic Retinopathy [NCT06321302]</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+General inclusion criteria
+* Diagnosis of diabetes mellitus (DM) under regular treatment with Haemoglobin A1c (HbA1c) (glycated haemoglobin) (HbA1c) \&lt;12%; DM should be under regular investigation by a trained specialist as per local standard of care prior to and during the trial
+* Age ≥18 years at time of signing Informed Consent Form (ICF)
+Ocular inclusion criteria: study eye
+* Moderate to severe non-proliferative diabetic retinopathy (NPDR) (Diabetic Retinopathy Severity Scale (DRSS) level 43 to 53) as assessed by Ultra-widefield colour fundus photography (UWF-CFP) images (within the 7-field grid) and confirmed by the central reading centre (CRC) at screening. Patient staged at DRSS level of 43 based on UWF-CFP images can be included only if:
+  * They are participating in the standard 7-field CFP sub-study of the trial, and
+  * They are staged as DRSS level of 47 to 53 on standard 7-field CFP imaging, as confirmed by the CRC at screening.
+* Ultra-widefield fluorescein angiography (UWF-FA) image gradable for presence of retinal non-perfusion (RNP) as confirmed by the CRC at screening
+* Visual acuity: best corrected visual acuity (BCVA) letter score of ≥49 letters (approximate Snellen equivalent of 20/100 or better) using ETDRS chart at starting distance of 4 meter (m) at screening and reconfirmed at baseline
+* Sufficiently clear ocular media, adequate pupillary dilation, and fixation to permit quality fundus imaging
+Main exclusion criteria in study eye:
+\- Evidence of active retinal neovascularisation (NV) on clinical exam and/or UWF-CFP images within the 7-field grid, confirmed by the CRC grading.
+The following are permitted if, based on the assessment of the investigator, do not require acute treatment:
+* Small neovascular lesions within the ETDRS 7-field that are detected only on UWF-FA, but not on clinical exam or UWF-CFP
+* Neovascularisations outside of the ETDRS 7-field on ultra-widefield imaging
+  * Evidence of active NV of the iris (small iris tufts are not an exclusion) or in the anterior chamber angle
+  * Prior pan-retinal photocoagulation (PRP). Peripheral scatter or targeted laser treatment in up to 1 quadrant outside the ETDRS 7-field area is permitted if it was performed at least 6 months prior to Day 1
+  * CI-DME, defined as central subfield thickness (CST) ≥320 micrometer (μm) as measured by Heidelberg Spectralis optical coherence tomography (OCT) and confirmed by central reading centre (CRC) at screening (equivalent measurements from other OCT machines may be accepted); participants with a CST of 320-330 μm can be included if, in the opinion of the investigator, the participant is not expected to require treatment for CI-DME during the duration of the study (e.g. no profound impact on BCVA, stable CST, etc.). CST must be re-confirmed at baseline. A CRC confirmation of the baseline CST is not required.
+  * Previous treatment in the study eye for NPDR and/or diabetic macular edema (DME) with intravitreal (IVT) anti-vascular endothelial growth factor (VEGF) (including anti-VEGF/Ang2) or short acting corticosteroid drugs (e.g. triamcinolone) within 6 months prior to Day 1 or \&gt;4 treatments within the last 18 months (referred to elsewhere as 'previous IVT treatment').
+  * Any previous IVT treatment other than anti-VEGF and short-acting steroids. Previous dexamethasone IVT drug delivery system (Ozurdex) or fluocinolone acetonide intravitreal implant (Iluvien) is not allowed
+  * Refractive error of more than -8 dioptres of myopia (spherical equivalent) in the study eye. For patients having undergone refractive or cataract surgery in the study eye, either the pre-operative refractive error or the axial length measurement should be used, at the investigator's discretion. Axial length should be less than 26 mm
+  * Any concurrent or past ocular condition in the study eye which, in the judgement of the investigator, could:
+* Require medical or surgical intervention during the study period to prevent or treat vision loss (e.g. advanced cataract, history of retinal detachment or macular hole (Stage 3 or 4) in the study eye)
+* Could likely contribute to a significant loss of BCVA during the study period if left untreated (e.g. advanced epiretinal membrane and/or vitreomacular traction, active or history of optic neuritis in either eye)
+* Contraindicate the use of the investigational drug, or may render the patient at high risk for treatment complications (e.g. active infectious or non-infectious conjunctivitis/keratitis in either eye; history of recurrent infectious or inflammatory ocular disease in either eye (e.g. uveitis)
+* May affect interpretation of the study results (e.g. central atrophy of the retinal pigment epithelium or photoreceptors; age-related macular degeneration, hereditary retinal degenerative diseases, myopic macular degeneration, past, current or planned use of medications known to be toxic to the retina, lens or optic nerve (e.g. deferoxamine, chloroquine/hydroxychloroquine, chlorpromazine, phenothiazines, tamoxifen, nicotinic acid, and ethambutol); history of central serous chorioretinopathy, ischemic optic neuropathy or retinal vascular occlusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun 12:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>A Safety, Tolerability, and Efficacy Study of VX-880 in Participants With Type 1 Diabetes [NCT04786262]</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 65 Years  |  All
+Key Inclusion Criteria:
+* Clinical history of T1D with \&gt; 5 years of duration of insulin dependence
+* At least two episodes of documented severe hypoglycemia in the 12 months prior to enrollment
+* Stable diabetic treatment
+* Consistent use of continuous glucose monitor (CGM) for at least 3 months before Screening and willingness to use CGM for the duration of the study
+Key Exclusion Criteria:
+-Prior islet cell transplant, organ transplant, or cell therapy
+Other protocol defined Inclusion/Exclusion criteria may apply</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitor update 2026-06-30 15:10 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -4624,7 +4624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A3:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4632,8 +4632,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -4677,7 +4675,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -4726,7 +4723,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -4797,7 +4793,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -4871,7 +4866,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -4906,7 +4900,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -4956,7 +4949,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -5017,7 +5009,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -5057,7 +5048,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Monitor update 2026-07-01 13:27 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B118"/>
+  <dimension ref="A3:B142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2877,6 +2877,425 @@
         </is>
       </c>
     </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="36" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>A Clinical Study of MK-2870 Alone or With Other Treatments to Treat Gastrointestinal Cancers (MK-9999-02A) [NCT06428409]</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+The main inclusion criteria include but are not limited to the following:
+* Has one of the following cancers:
+  * Unresectable or metastatic colorectal cancer and has received prior therapy for the cancer
+  * Advanced or metastatic pancreatic ductal adenocarcinoma (PDAC) and has received prior therapy for the cancer
+  * Advanced and/or unresectable biliary tract cancer (BTC) and has received prior therapy for the cancer
+  * Advanced and/or unresectable BTC and has not received prior therapy for the cancer
+* For participants who have received prior therapy for cancer: Has recovered from any side effects due to previous cancer treatment
+Exclusion Criteria:
+The main exclusion criteria include but are not limited to the following:
+* History of severe eye disease
+* For participants who have received prior therapy for cancer: Received prior systemic anticancer therapy including investigational agents within 4 weeks before starting study intervention
+* History of (noninfectious) pneumonitis/interstitial lung disease (ILD) that required steroids, has current pneumonitis/ILD, or has suspected ILD or pneumonitis that cannot be ruled out by standard diagnostic assessments at Screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="36" customHeight="1">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Assess the Efficacy, Safety, Pharmacodynamics, and Pharmacokinetics of Tazemetostat in Combination With Lenalidomide Plus Rituximab Versus Placebo in Combination With Lenalidomide Plus Rituximab in Adult Patients at Least 18 Years of Age With Relapsed/Refractory Follicular Lymphoma. [NCT04224493]</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+1. Have voluntarily agreed to provide written informed consent and demonstrated willingness and ability to comply with all aspects of the protocol.
+2. Males or females are ≥18 years of age, or per country adult legal age regulations, at the time of providing voluntary written informed consent.
+3. Life expectancy ≥3 months before enrollment.
+4. Meet requirement for hepatitis and human immunodeficiency virus (HIV) infection as follows
+   * Negative serologic or polymerase chain reaction (PCR) test results for acute or chronic hepatitis B virus (HBV) infection Note: Participants whose HBV infection status could not be determined by serologic test results have to be negative for HBV-DNA by PCR to be eligible for study participation. Participants seropositive for HBV with undetectable HBV DNA by PCR are permitted with appropriate antiviral prophylaxis.
+   * Negative test results for hepatitis C virus (HCV) Note: Participants who are positive for HCV antibody must be negative for HCV RNA by PCR to be eligible for study participation
+   * If HIV positive, HIV infection is controlled. Based on Cancer Clinical Trial Eligibility Criteria: Patients with HIV, Hepatitis B Virus, or Hepatitis C Virus Infections - Guidance for Industry (https://www.fda.gov/media/121319/download), patients with HIV should be considered eligible if they have CD4+ T-cell counts ≥ 350 cells/uL and in general, if they have not had an opportunistic infection within the past 12 months. Other exclusion criteria should be considered regarding the drug-drug interaction if antiviral drugs are used. Therefore, in case of controlled HIV infection, since antiviral drugs are used, trial patients should be on established ART for at least 4 weeks and have an HIV viral load less than 400 copies/mL prior to enrolment.
+5. Have histologically confirmed FL, Grades 1 to 3A.
+6. Must have been previously treated with at least 1 prior systemic chemotherapy, immunotherapy, or chemoimmunotherapy:
+   a. Systemic therapy includes treatments such as:
+   i. Rituximab monotherapy
+   ii. Chemotherapy given with or without rituximab
+   iii. Radioimmunoconjugates such as 90Y-ibritumomab tiuxetan and 131I-tositumomab.
+   b. Systemic therapy does not include, for example:
+   i. Local involved field radiotherapy for limited-stage disease
+   ii. Helicobacter pylori eradication
+   c. Prior investigational therapies will be allowed provided the subject has received at least 1 prior systemic therapy as discussed in Inclusion Criterion #6a.
+   d. Prior autologous/allogeneic hematopoietic stem cell transplant (HSCT) will be allowed.
+   e. Prior chimeric antigen receptor T-cell therapy (CAR T) will be allowed.
+7. Must have documented relapsed, refractory, or PD after treatment with systemic therapy (refractory defined as less than PR or disease progression \&lt;6 months after last dose).
+8. Have measurable disease as defined by the Lugano Classification (Cheson, 2014; Appendix 5).
+9. Eastern Cooperative Oncology Group (ECOG) performance status of 0, 1, or 2.
+10. Within 7 days prior to randomization, all clinically significant toxicity related to a prior anticancer treatment (ie, chemotherapy, immunotherapy, and/or radiotherapy must have either resolved to Grade 1 per NCI CTCAE Version 5.0 OR are clinically stable and no longer clinically significant.
+11. Have provided sufficient tumor tissue block or unstained slides for EZH2 mutation testing in all subjects to allow for stratification
+    a. If EZH2 mutation status is known from site-specific testing, subjects can be enrolled. Tumor tissue will be required for confirmatory testing of EZH2 status at study-specific laboratories. If the archival tumor sample was collected more than 24 months prior to the anticipated administration of the first dose (cycle 1 day 1), then a fresh biopsy must be provided. Fresh tumor biopsy is appropriate except for procedures deemed to result in unacceptable risk because of the anatomical location including brain, lung/mediastinum, pancreas, or endoscopic procedures extending beyond the esophagus, stomach, or bowel. Archival tumor biopsy sections mounted on slides are also acceptable.
+    NOTE: Confirmatory testing will also be performed for Stage 1, if local EZH2 testing is conducted, unless there is insufficient tumor tissue to perform testing after discussion with the Sponsor's or Designee Medical Monitor.
+12. Time between prior anticancer therapy and first dose of tazemetostat as follows:
+    1. Cytotoxic chemotherapy - At least 21 days.
+    2. Noncytotoxic chemotherapy (eg, small molecule inhibitor) - At least 14 days.
+    3. Nitrosoureas - At least 6 weeks.
+    4. Monoclonal and/or bispecific antibodies or CAR T - At least 28 days.
+    5. Radiotherapy - At least 6 weeks from prior radioisotope therapy; at least 12 weeks from 50% pelvic or total body irradiation.
+13. Adequate renal function defined as calculated creatinine clearance ≥30 mL/minute per the Cockcroft and Gault formula.
+14. Adequate bone marrow function:
+    a. Absolute neutrophil count (ANC) ≥1000/mm3 (≥1.0 × 10\^9/L) if no lymphoma infiltration of bone marrow OR ANC ≥750/mm3 (≥75 × 10\^9/L) with bone marrow infiltration
+    * Without growth factor support (filgrastim or pegfilgrastim) for at least 14 days.
+      b. Platelets ≥75,000/mm3 (≥75 × 10\^9/L)
+    * Evaluated at least 7 days after last platelet transfusion.
+      c. Hemoglobin ≥9.0 g/dL
+    * May receive transfusion
+15. Adequate liver function:
+    1. Total bilirubin ≤1.5 × the upper limit of normal (ULN) except for unconjugated hyperbilirubinemia of Gilbert's syndrome.
+    2. Alkaline phosphatase (ALP) (in the absence of bone disease), alanine aminotransferase (ALT), and aspartate aminotransferase (AST) ≤3 × ULN (≤5 × ULN if subject has liver infilration).
+16. International normalized ratio (INR) ≤1.5 × ULN and activated partial thromboplastin time (aPTT) ≤1.5 × ULN (unless on warfarin, then INR ≤3.0). In subjects with thromboembolism risk, prophylactic anticoagulation, or antiplatelet therapy at investigator discretion is recommended.
+17. Females of childbearing potential (FCBP) must have a negative urine or serum pregnancy tests (beta-human chorionic gonadotropin \[β-hCG\] tests with a minimum sensitivity of 25 mIU/mL or equivalent units of β-hCG) at screening within 10 to 14 days prior to first dose of study drug. The subject may not receive study drug until the study doctor has verified that the results of pregnancy tests are negative. All females will be considered to be of childbearing potential unless they are naturally postmenopausal (at least 24 months consecutively amenorrhoeic \[amenorrhea following cancer therapy does not rule out childbearing potential\] and without other known or suspected cause) or have been sterilized surgically (ie, total hysterectomy and/or bilateral oophorectomy, with surgery completed at least 1 month before dosing).
+18. Females of childbearing potential (FCBP) enrolled must either practice complete abstinence or agree to use two reliable methods of contraception simultaneously. This includes ONE highly effective method of contraception and ONE additional effective contraceptive method. Contraception must begin at least 28 days prior to first dose of study drug, continue during study treatment (including during dose interruptions), and for 12 months after study drug discontinuation. Female subjects must also refrain from breastfeeding for 12 months following last dose of study drug. If the below contraception methods are not appropriate for the FCBP, she must be referred to a qualified contraception provider to determine the medically effective contraception method appropriate for the subject. The following are examples of highly effective and additional effective methods of contraception:
+    Examples of highly effective methods:
+    * Intrauterine device (IUD)
+    * Hormonal (ovulation inhibitory combined \[estrogen and progesterone\] birth control pills or intravaginal/transdermal system, injections, implants, levonorgestrel-releasing intrauterine system \[IUS\], medroxyprogesterone acetate depot injections, ovulation inhibitory progesterone-only pills \[e.g. desogestrel\]) NOTE: There is a potential for tazemetostat interference with hormonal contraception methods due to enzymatic induction.
+    * Bilateral tubal ligation
+    * Partner's vasectomy (if medically confirmed \[azoospermia\] and sole sexual partner).
+    Examples of additional effective methods:
+    * Male latex or synthetic condom,
+    * Diaphragm,
+    * Cervical Cap
+    NOTE: Female subjects of childbearing potential exempt from these contraception requirements are subjects who practice complete abstinence from heterosexual sexual contact. True abstinence is acceptable when this is in line with the preferred and usual lifestyle of the subject. Periodic abstinence (eg, calendar, ovulation, symptothermal, or post ovulation methods) and withdrawal are not acceptable methods of contraception.
+19. All study participants enrolled must be registered into the applicable pregnancy prevention program (e.g. REVLIMID REMS in the US, Pregnancy Prevention Programme \[PPP\] in Europe) for lenalidomide to be administered and be willing and able to comply with the requirements of the applicable program as appropriate for the country in which the drug is being used.
+    a. Female subjects of childbearing potential (FCBP) must adhere to the scheduled pregnancy testing as required in theapplicable pregnancy prevention program. During study treatment, FCBP must agree to have pregnancy testing weekly for the first 28 days of study participation and then every 28 days for FCBP with regular or no menstrual cycles OR every 14 days for FCBP with irregular menstrual cycles. FCBP must also have a pregnancy test at end of lenalidomide treatment, at day 14 (for FCBP with irregular menstrual cycles) and day 28 following the last dose of lenalidomide and at overall treatment discontinuation (at the End-of-Treatment/30-day safety Follow-up visit). Female subjects exempt from this requirement are subjects who have been naturally postmenopausal for at least 24 consecutive months OR are surgically sterilized (ie, total hysterectomy or bilateral oophorectomy) with surgery at least 1 month before the first dose of study treatment.
+20. Male subjects must either practice complete abstinence or agree to use a latex or synthetic condom, even with a successful vasectomy (medically confirmed azoospermia), during sexual contact with a pregnant female or FCBP from first dose of study drug, during study treatment (including during dose interruptions), and for 3 months after study drug discontinuation.
+NOTE: Male subjects must not donate semen or sperm from first dose of study drug, during study treatment (including during dose interruptions), and for 3 months after study drug discontinuation.
+Exclusion Criteria:
+All Subjects
+1. Prior exposure to tazemetostat or other inhibitor(s) of EZH2.
+2. Prior exposure to lenalidomide or drugs of the same class.
+3. Grade 3b, mixed histology, or FL that has histologically transformed to diffuse large B-cell lymphoma (DLBCL) (subjects transformed from DLBCL to FL may be enrolled).
+4. Has thrombocytopenia, neutropenia, or anemia of Grade ≥3 (per CTCAE Version 5.0 criteria) or any prior history of myeloid malignancies, including myelodysplastic syndrome (MDS)/acute myeloid leukemia (AML) or myeloproliferative neoplasm (MPN).
+5. Has a prior history of T-cell lymphoblastic lymphoma (T-LBL)/T-cell acute lymphoblastic leukemia (T-ALL) or B-cell acute lymphoblastic leukemia (B-ALL).
+6. Subjects with uncontrolled leptomeningeal metastases or brain metastases or history of previously treated brain metastases.
+7. Subjects taking medications that are known strong CYP3A inhibitors and strong or moderate CYP3A inducers (including St. John's wort).
+8. Are unwilling to exclude grapefruit juice, Seville oranges, and grapefruits from the diet and/or consumed within 1 week of the first dose of study drug and for the duration of the study.
+9. Major surgery within 4 weeks before the first dose of study drug.
+   a. Note: Minor surgery (eg, minor biopsy of extracranial site, central venous catheter placement, shunt revision) is permitted within 3 weeks prior to enrollment.
+10. Are unable to take oral medication OR have malabsorption syndrome or any other uncontrolled gastrointestinal condition (eg, nausea, diarrhea, vomiting) that might impair the bioavailability of tazemetostat.
+11. Significant cardiovascular impairment: history of congestive heart failure greater than New York Heart Association (NYHA) Class II, uncontrolled arterial hypertension, unstable angina, myocardial infarction, or stroke within 6 months of the first dose of study drug; or cardiac ventricular arrhythmia.
+12. Prolongation of corrected QT interval using Fridericia's formula (QTcF) to ≥480 msec at screening or history of long QT syndrome.
+13. Venous thrombosis or pulmonary embolism within the last 3 months before starting tazemetostat.
+    a. Note: Participants who have experienced deep vein thrombosis/pulmonary embolism more than 3 months before enrollment are eligible but are recommended to receive prophylaxis.
+14. Have an active infection requiring systemic therapy.
+15. Known hypersensitivity to any component of tazemetostat or lenalidomide; known severe hypersensitivity to any component of rituximab requiring hospitalization or resuscitation.
+16. Active viral infection with or seropositive for HBV: HBV surface antigen (HBsAg) positive OR HBsAg negative, anti-HBs positive and/or anti-HBc positive with detectable HBV DNA.
+    NOTE: Subjects who are HBsAg negative, anti-HBs positive and/or anti-HBc positive, but with undetectable viral DNA and normal ALT are eligible. Subjects who are seropositive due to HBV vaccination (HBsAg negative, HBV surface antibody \[anti-HBs\] positive, and HBV core antibody \[anti-HBc\] negative) are eligible.
+17. Active viral infection with hepatitis C virus (as measured by positive HCV antibody and detectable viral RNA, HIV), or known active infection with human T-cell lymphotropic virus.
+    NOTE: Subjects with a history of hepatitis C infection (HCV antibody reactive) who have normal ALT and undetectable HCV RNA are eligible.
+18. Any other medical or social condition that, in the Investigator's judgment, will interfere with a participant's ability to provide informed consent, to receive study drugs, or meet study demands, or that substantially increases the risk associated with the subject's participation in the study, or that may interfere with interpretation of results.
+19. Female subjects who are pregnant or lactating/breastfeeding.
+20. Subjects who have undergone a solid organ transplant.
+21. Subjects with malignancies other than FL. a. Exception: Subjects with another malignancy who have been disease-free for 3 years, or subjects with a history of a completely resected non-melanoma skin cancer or successfully treated in situ carcinoma are eligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="36" customHeight="1">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>A Study of Abemaciclib (LY2835219) With Abiraterone in Men With Prostate Cancer That Has Spread to Other Parts of the Body and is Expected to Respond to Hormonal Treatment (Metastatic Hormone-Sensitive Prostate Cancer) [NCT05288166]</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  Male
+Inclusion Criteria:
+* Adenocarcinoma of the prostate (as the predominant histology)
+* High-risk metastatic hormone-sensitive prostate cancer. High risk is defined as:
+  * Greater than or equal to (≥)4 bone metastases by bone scan and/or
+  * ≥1 visceral metastases by computed tomography or magnetic resonance imaging
+* Must have initiated androgen deprivation therapy (ADT) with luteinizing hormone-releasing hormone (LHRH) agonist/antagonist or bilateral orchiectomy prior to randomization. Up to 3 months of ADT prior to randomization is permitted with or without first-generation anti-androgen.
+* Adequate organ function
+* Eastern Cooperative Oncology Group (ECOG) performance status of 0 or 1
+Exclusion Criteria:
+* Prior treatment with abemaciclib or any other cyclin dependent kinase 4 and 6 (CDK4 \&amp; 6) inhibitor
+* Development of metastatic prostate cancer in the context of castrate levels of testosterone
+* Received any prior systemic therapy for metastatic prostate cancer (including investigational agents), except for ADT and first-generation anti-androgen
+* Clinically significant cardiovascular disease as evidenced by myocardial infarction, arterial thrombotic events, or severe/unstable angina in the past 6 months, or New York Heart Association Class II to IV heart failure
+* History of syncope of cardiovascular etiology, ventricular arrhythmia of pathological origin, or sudden cardiac arrest. Chronic and hemodynamically stable atrial arrhythmia well-controlled on medical therapy is permitted
+* Uncontrolled hypertension
+* Clinically active or chronic liver disease, moderate/severe hepatic impairment
+* Known untreated central nervous system (CNS) metastasis. Participants with a history of treated brain metastases are eligible if stable for at least 8 weeks prior to randomization and off corticosteroid for at least 2 weeks prior to randomization</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="36" customHeight="1">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Effect of Proactive Therapeutic Drug Monitoring on Maintenance of Sustained Disease Control in Adults With Rheumatoid Arthritis on a Subcutaneous TNF Inhibitor: The Rheumatoid Arthritis Therapeutic DRUg Monitoring Trial (RA-DRUM) [NCT06440629]</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 74 Years  |  All
+Inclusion Criteria:
+1. A clinical diagnosis of RA
+2. ≥ 18 and under 75 years of age at screening
+3. On stable therapy with standard dose of a SC TNFi (adalimumab) for a minimum of 3 months and a maximum of 24 months
+4. In low disease activity or remission (DAS28-CRP under 3.2) and indication for continuation of treatment according to the treating physician
+5. Subject capable of understanding and signing an informed consent form
+Exclusion Criteria:
+1. Major comorbidities, such as previous malignancies within the last 5 years, uncontrolled diabetes mellitus, severe infections (including HIV), uncontrollable hypertension, severe cardiovascular disease (NYHA class 3 or 4), severe respiratory diseases, demyelinating disease, significant chronic widespread pain syndrome, significant renal or hepatic disease, and/or other diseases or conditions which either contraindicate treatment with SC TNFi or make adherence to the protocol difficult
+2. Hypersensitivity to sc TNFi (adalimumab).
+3. Pregnancy, or subject considering becoming pregnant during the study period
+4. Psychiatric or mental disorders, alcohol abuse or other substance abuse, language barriers, or other factors that makes adherence to the study protocol difficult
+5. Changes in csDMARD co-medication, including dose changes of csDMARD or changes in the dose of corticosteroids within the last 2 months
+6. Co-medication with bDMARD, tsDMARD, or other immunosuppressive drugs (excluding csDMARD and corticosteroids ≤ 7.5 mg prednisolone (or equivalent) once daily).
+7. Active participation in any other interventional study.
+8. In need of live vaccines during the study period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="36" customHeight="1">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Safety, Efficacy, and Pharmacokinetics of BNT327 in Combination With Chemotherapy and Other Investigational Agents for Lung Cancer [NCT06712316]</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Key Inclusion Criteria:
+* Have systemic treatment naive, histologically or cytologically confirmed diagnosis of Stage IIIB or IIIC (who are not amenable to curative surgery or radiotherapy) or Stage IV NSCLC per the Union Internationale contre le Cancer/American Joint Committee on Cancer staging system, 9th edition.
+* Have at least one measurable lesion as the targeted lesion based on RECIST v1.1. Lesions treated after prior local treatment (radiotherapy, ablation, interventional procedures, etc.) are generally not considered as target lesions. If the lesion with prior local treatment is the only targeted lesion, evidence-based radiology must be provided to demonstrate disease progression (the single bone metastasis or the single central nervous system metastasis should not be considered as a measurable lesion).
+* Eastern Cooperative Oncology Group Performance Status of 0 or 1.
+* Adequate organ function.
+Key Exclusion Criteria:
+* Have histologically or cytologically confirmed NSCLC with small-cell lung cancer histologic or neuroendocrine component.
+* Have received any of the following therapies or drugs within the noted time intervals prior to study treatment:
+  * Previous chemotherapy (platinum-based) or PD(L)-1 for treating NSCLC in either neo-adjuvant/adjuvant or locally advanced/metastatic setting.
+  * Participants who received prior treatment with anti-VEGF monoclonal antibody, or PD(L)-1/VEGF bispecific antibody
+  * Have received systemic corticosteroids (at a dosage greater than 10 mg/day of prednisone or an equivalent dose of other corticosteroids) within 7 days prior to the initiation of study treatment. Note: local, intranasal, intraocular, intra-articular or inhaled corticosteroids, short-term use (\&lt;=7 days) of corticosteroids for prophylaxis (e.g., prevention of contrast agent allergy) or treatment of non-autoimmune conditions (e.g., delayed hypersensitivity reactions caused by exposure to allergens) are allowed.
+* Have uncontrolled hypertension or poorly controlled diabetic conditions prior to study treatment.
+* Have a serious or non-healing wound, or (incompletely healed) bone fracture. This includes history (within 6 months prior to study entry) or risk of abdominal fistula, tracheoesophageal fistula, gastrointestinal perforation, or intra-abdominal abscess or esophageal and gastric varices. In addition, the participant must have undergone correction (or spontaneous healing) of the perforation/fistula and/or the underlying process causing fistula/perforation.
+* Participants with significant risk of hemorrhage (per investigator clinical judgment).
+* Have superior vena cava syndrome or symptoms of spinal cord compression.
+NOTE: Other protocol defined Inclusion/Exclusion criteria may apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="36" customHeight="1">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Phase III Study of Datopotamab Deruxtecan Versus Docetaxel in Previously Treated TROP2-positive Advanced or Metastatic Non-squamous NSCLC Without Actionable Genomic Alterations [NCT07291037]</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Pathologically documented Stage IIIB, IIIC, or Stage IV non-squamous non-small cell lung cancer (NSCLC) without actionable genomic alterations (AGA) at the time of randomisation and meets the criteria for NSCLC:
+  * Participants must have documented negative test results for epidermal growth factor receptor (EGFR), anaplastic lymphoma kinase (ALK), and ROS proto-oncogene 1 (ROS1) genomic alterations.
+  * Has no known tumour genomic alterations in neurotrophic tyrosine receptor kinase (NTRK), proto-oncogene B-raf (BRAF), rearranged during transfection (RET), mesenchymal-epithelial transition (MET) exon 14 skipping, Kirsten rat sarcoma viral oncogene homolog (KRAS) G12C, human epidermal growth factor receptor 2 (HER2) or any other actionable driver oncogenes for which there are locally approved and available targeted first-line therapies.
+  * Prospectively assessed trophoblast cell surface protein 2 (TROP2) normalised membrane ratio (NMR) positive.
+* Documentation of radiographic disease progression while on or after receiving the most recent treatment regimen for advanced or metastatic NSCLC.
+* Participants must have received platinum based chemotherapy (PBC) in combination with anti-programmed death-protein 1 (anti-PD-1)/anti-programmed death-ligand 1 (anti-PD-L1) monoclonal antibody (mAb) as the only prior line of therapy or received PBC and anti-PD-1/anti-PD-L1 monoclonal antibody (in either order) sequentially as the only 2 prior lines of therapy.
+* Provision of acceptable formalin fixed and paraffin embedded (FFPE) tumour sample for assessment of TROP2.
+* At least one lesion not previously irradiated that qualifies as a Response Evaluation Criteria in Solid Tumours, Version 1.1 (RECIST 1.1) target lesion (TL) at baseline and can be accurately measured at baseline as ≥ 10 mm in the longest diameter (except lymph nodes, which must have short axis ≥ 15 mm) with computed tomography (CT) or magnetic resonance imaging (MRI) and is suitable for accurate repeated measurements.
+* Eastern Cooperative Oncology Group (ECOG) Performance Status (PS) of 0 or 1.
+* Adequate bone marrow reserve and organ function within 7 days before randomisation.
+Exclusion Criteria:
+* Squamous, mixed NSCLC, or small cell lung cancer (SCLC) histology.
+* NSCLC disease that is eligible for definitive local therapy alone.
+* History of another primary malignancy other than NSCLC, except for malignancy treated with curative intent with no known active disease within 3 years before randomisation and of low potential risk for recurrence.
+* Spinal cord compression or brain metastases, unless asymptomatic, stable, and not requiring treatment with corticosteroids or anticonvulsants for at least 7 days prior to randomisation.
+* Clinically significant corneal disease.
+* Has active or uncontrolled hepatitis B or C virus infection.
+* Known human immunodeficiency virus (HIV) infection that is not well controlled.
+* Uncontrolled infection requiring intravenous (IV) antibiotics, antivirals, or antifungals.
+* History of non-infectious interstitial lung disease (ILD)/pneumonitis including radiation pneumonitis that required steroids, has current ILD/pneumonitis, or has suspected ILD/pneumonitis that cannot be ruled out by imaging at screening.
+* Severe pulmonary function compromise per Investigator discretion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="36" customHeight="1">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>Study of TDXd, Chemotherapy, Pembrolizumab, and Trastuzumab in First-Line Metastatic HER2-Positive Gastric or Gastroesophageal Junction Cancer [NCT06731478]</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+1. Sign and date the Tissue Prescreening ICF, prior to central HER2 and PD-L1 CPS testing. Sign and date the Main Screening ICF, prior to the start of any trial-specific qualification procedures. Sign and date the Optional PGx ICF (included in the Main Screening ICF) prior to any PGx procedure.
+2. Adults ≥18 years of age on the day of signing the ICF. Follow local regulatory requirements if the legal age of consent for trial participation is \&gt;18 years old.
+3. Previously untreated, unresectable, locally advanced or metastatic gastric or GEJ adenocarcinoma histologically confirmed by pathology report. Prior treatment in the perioperative and/or adjuvant setting is permissible, provided there is \&gt;6 months between the end of perioperative or neoadjuvant treatment and the diagnosis of recurrent disease.
+   Note: Prior use of IO (ie, anti-PD-1/PD-L1) therapy in the (neo)adjuvant setting is allowed as long as there is \&gt;6 months between the end of IO therapy and the diagnosis of recurrent disease.
+4. Centrally determined HER2-positive (IHC 3+ or IHC 2+/ISH-positive) gastric or GEJ cancer as classified by the American Society of Clinical Oncology-College of American Pathologists for GC on a tumor biopsy as detected by prospective central test on new (core, incisional, excisional biopsy) or existing tumor tissue taken at the time of diagnosis of locally advanced or metastatic disease.
+   Note: Archival samples taken from a previous diagnostic or surgical biopsy not previously irradiated can be accepted. Details pertaining to tumor tissue submission can be found in the Study Laboratory Manual.
+5. Centrally determined tumor PD-L1 CPS using the PD-L1 assay:
+   * For the Main Cohort: PD-L1 CPS ≥1
+   * For the Exploratory Cohort: PD-L1 CPS \&lt;1
+6. All participants must provide a tumor sample for tissue-based IHC staining to centrally determine HER2 expression, PD-L1 CPS, and other correlatives. The mandatory FFPE or new biopsy tumor sample can be from either the primary tumor or metastatic biopsy. Specimens with limited tumor content (as centrally determined) and cytology samples are inadequate for defining tumor HER2 and PD-L1 status.
+7. At least 1 target measurable lesion on CT or MRI, assessed by the investigator based on RECIST v1.1. Lesions situated in a previously irradiated area are considered measurable if progression has been shown in such lesions.
+8. LVEF ≥50% within 28 days before randomization.
+Exclusion Criteria
+1. Prior exposure to other HER2-targeting therapies (including ADCs).
+2. Lack of physiological integrity of the upper gastrointestinal tract (ie, severe Crohn disease that results in malabsorption) or malabsorption syndrome that would preclude feasibility of oral chemotherapy for participants planned to be offered capecitabine as part of the study treatment.
+3. Known total or partial DPD enzyme deficiency. Note: Screening for DPD enzyme deficiency is required only in regions/countries where DPD testing is SoC and with unknown DPD status. For regions/countries where DPD testing is not SoC, local practice should be followed. In Spain and Italy, screening for DPD enzyme deficiency is mandatory for all participants with unknown DPD status.
+4. Contraindications to trastuzumab, 5-FU, capecitabine, cisplatin, or oxaliplatin treatment as per local label.
+5. Medical history of myocardial infarction within 6 months before randomization or symptomatic CHF (New York Heart Association Class II to IV). Participants with troponin levels above ULN at Screening (as defined by the manufacturer) and without any myocardial infarction -related symptoms should have a cardiologic consultation during the Screening Period to rule out myocardial infarction.
+6. Has a corrected QT interval (QTcF) prolongation to \&gt;470 ms (females) or \&gt;450 ms (males) based on the average of the screening triplicate 12-lead ECG.
+7. Has a history of (non-infectious) ILD/pneumonitis that required steroids, has current ILD/pneumonitis, or where suspected ILD/pneumonitis cannot be ruled out by imaging at Screening
+8. Lung-specific intercurrent clinically significant illnesses including, but not limited to, any underlying pulmonary disorder (eg, pulmonary emboli within 3 months of the trial randomization, severe asthma, severe chronic obstructive pulmonary disease, restrictive lung disease, pleural effusion, etc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="36" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>A Clinical Study to Test if an Investigational Treatment Called BNT314 When Used in Combination With Another Investigational Treatment Pumitamig (BNT327) and Chemotherapy, is Beneficial and Safe for Patients With Advanced Colorectal Cancer [NCT07079631]</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Key Inclusion Criteria:
+* Have unresectable histologically confirmed adenocarcinoma of the colon or rectum.
+* Have confirmed non-microsatellite instability-high (non-MSI-H)/pMMR mCRC per Food and Drug Administration (FDA)/European Commission (EC) approved test or based on local testing.
+* Have measurable disease defined by RECIST v1.1.
+* Must provide a tumor tissue sample (formalin-fixed, paraffin-embedded or tissue slides) collected before C1D1 for enrollment. A newly obtained tumor sample is preferred. If it is not feasible to obtain a recent tumor sample, participants can provide archival tumor tissue (less than 2 years prior treatment).
+* Have Eastern Cooperative Oncology Group Performance Status of 0 or 1.
+* Have a life expectancy of ≥12 weeks.
+* Have an adequate organ and bone marrow function within ≤7 days of Day 1 as defined in the protocol.
+* Have had an adequate previous treatment washout period before randomization/enrollment as defined in the protocol.
+Inclusion criteria applicable to only protocol-specific cohorts:
+* Have histologically confirmed metastatic colorectal cancer and radiographically documented disease progression after ≥2 prior lines of systemic therapy for metastatic disease as defined in the protocol.
+* Have progressed following first-line chemotherapy as specified in the protocol.
+* Have not received prior systemic therapy for MSS/pMMR mCRC. Participants who received chemotherapy, radiotherapy, or chemoradiotherapy with curative intent for non-metastatic disease in the neoadjuvant or adjuvant setting are eligible for the study if therapy was completed at least 6 months prior to initiation of study treatment.
+Other cohort-specific inclusion criteria apply.
+Key Exclusion Criteria:
+* Confirmed MSI-H/deficient mismatch repair mCRC (per FDA/CE approved test or based on local testing).
+* Prior treatment with epithelial cell-adhesion molecule or 4-1BB targeted or immunotherapy.
+* Prior treatment with immune checkpoint inhibitors or programmed death-ligand 1 (PD\[L\]-1)/vascular endothelial growth factor bispecific antibody.
+* Is a candidate to locoregional treatment (including surgical resection, stereotactic radiation therapy or tumor ablation) with potential to induce complete or near complete response and prolonged tumor control (sometimes described as "radical" intent), per investigator's assessment.
+* Have uncontrolled or significant cardiovascular disease as specified in the protocol.
+* Have left ventricular ejection fraction \&lt;50% by echocardiogram or multigated acquisition within 28 days before randomization/enrollment.
+* Have clinically uncontrolled pleural effusion, ascites or pericardial effusion requiring drainage, peritoneal shunt, or cell-free concentrated ascites reinfusion therapy within 2 weeks prior to randomization/enrollment.
+* Have clinically active central nervous system metastases, defined as untreated and symptomatic, or requiring therapy with corticosteroids or anticonvulsants to control associated symptoms. Participants with treated brain metastases that are no longer symptomatic and who require no treatment with corticosteroids or anticonvulsants may be included in the study if they have recovered from the acute toxic effect of radiotherapy. Participants with untreated, asymptomatic brain metastases for whom local therapy is not indicated per SoC may be eligible if neurologically stable and (if deemed necessary by the investigator). Except for brain metastases history, any participants at imminent risk for spinal cord compression or leptomeningeal disease are not eligible.
+* Have unresolved toxicities from previous anticancer therapy, defined as toxicities (other than alopecia) not yet resolved to Grade ≤1 or baseline toxicities that have resolved with sequelae (e.g., tracheostomy, chronic use of feeding tube, replacement hormones) are allowed, if not associated with increased risk of complications per investigator's assessment.
+* Participants in Part B or C who fulfill one of the conditions:
+  * Prior treatment with anticancer therapies (as defined in the protocol) with unusual toxicity, or
+  * Known dihydropyrimidine dehydrogenase (DPD) deficiency, testing performed according to the local guidelines. If not tested, lack of DPD activity must be tested for the participants who have not received anticancer therapies (as defined in the protocol) in the prior lines of treatment; testing should be performed according to the local guidelines.
+* Have a history of another primary malignancy within 2 years, except adequately resected non-melanoma skin cancer, curatively treated in-situ disease, or other solid tumors curatively treated (adjuvant hormone therapy for malignancies at low risk of relapse is allowed) or have a known additional malignancy that is progressing or requires treatment.
+* Have a history of small bowel obstruction requiring hospitalization within the past 3 months prior to the first dose of IMP.
+* Have 24-h urine protein excretion ≥1 g. If qualitative urine protein is ≤1+, a 24-h urine protein quantitative test is not required.
+* Have active autoimmune disease or a history of autoimmune disease (myasthenia gravis, myositis, autoimmune hepatitis, systemic lupus erythematosus, rheumatoid arthritis, psoriatic arthritis, inflammatory bowel disease, vasculitis, antiphospholipid antibody syndrome, Wegener granulomatosis, Sjögren's syndrome, Guillain-Barré syndrome, or multiple sclerosis) with a risk of exacerbation following PD-L1 inhibition or have an immune deficiency (allogeneic hematopoietic stem cell transplantation or organ transplantation). Participants with protocol-specified conditions may be eligible.
+* Have serious non-healing wounds, ulcers, or bone fractures. This includes history of abdominal fistula, gastrointestinal perforation, or intra abdominal abscess or esophageal and gastric varices, acute gastrointestinal bleeding for which an interval of 6 months must pass before enrollment into this study. In addition, the participant must have undergone correction (or spontaneous healing) of the perforation/fistula and/or the underlying process causing the fistula/perforation.
+* Have evidence of major coagulation disorders or other significant risks of hemorrhage as specified in the protocol.
+NOTE: Other protocol defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2888,7 +3307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C112"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2896,6 +3315,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -2944,6 +3365,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -2985,6 +3407,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3042,6 +3465,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -3095,6 +3519,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -3173,6 +3598,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -3247,6 +3673,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -3297,6 +3724,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -3332,6 +3760,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -3370,6 +3799,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -3403,6 +3833,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
@@ -3451,6 +3882,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
@@ -3512,6 +3944,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
@@ -3556,6 +3989,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
@@ -3597,6 +4031,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
@@ -3645,6 +4080,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
@@ -3681,6 +4117,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
@@ -3729,6 +4166,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -3776,6 +4214,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
@@ -3824,6 +4263,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
@@ -3861,6 +4301,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
@@ -3910,6 +4351,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
@@ -3961,6 +4403,7 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
@@ -4010,6 +4453,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
@@ -4050,6 +4494,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -4113,6 +4558,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
@@ -4144,6 +4590,7 @@
         </is>
       </c>
     </row>
+    <row r="80"/>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
@@ -4185,6 +4632,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
@@ -4222,6 +4670,7 @@
         </is>
       </c>
     </row>
+    <row r="86"/>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
@@ -4258,6 +4707,7 @@
         </is>
       </c>
     </row>
+    <row r="89"/>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
@@ -4295,6 +4745,7 @@
         </is>
       </c>
     </row>
+    <row r="92"/>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
@@ -4334,6 +4785,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
@@ -4373,6 +4825,7 @@
         </is>
       </c>
     </row>
+    <row r="98"/>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
@@ -4415,6 +4868,7 @@
         </is>
       </c>
     </row>
+    <row r="101"/>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -4466,6 +4920,7 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
@@ -4516,6 +4971,7 @@
         </is>
       </c>
     </row>
+    <row r="107"/>
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
@@ -4580,6 +5036,7 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
@@ -4610,6 +5067,205 @@
 * Inability to follow procedures or insufficient knowledge in English, German or French;
 * Inability to give consent.
 Participants who undergo cardiac surgery under minimal extracorporeal circulation will also be excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113"/>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="36" customHeight="1">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>MagnetisMM-32: A Study to Learn About the Study Medicine Called Elranatamab in People With Multiple Myeloma (MM) That Has Come Back After Taking Other Treatments (Including Prior Treatment With an Anti-CD38 Antibody and Lenalidomide) [NCT06152575]</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Prior diagnosis of multiple myeloma as defined by International Myeloma Working Group (IMWG) criteria and previously received 1 to 4 prior lines of therapy including prior anti-cluster of differentiation 38 (CD38) antibody and prior lenalidomide.
+* Documented evidence of progressive disease or failure to achieve a response to last line of therapy per IMWG criteria.
+* Measurable disease defined as at least 1 of the following: (a) Serum M-protein ≥0.5 g/dL; (b) Urinary M-protein excretion ≥200 mg/24 hours; (c) Serum involved immunoglobulin FLC ≥10 mg/dL AND abnormal serum immunoglobulin kappa to lambda FLC ratio (\&lt;0.26 or \&gt;1.65).
+* Have clinical laboratory values within the specified range.
+* ECOG (Eastern Cooperative Oncology Group) performance status ≤2.
+* Not pregnant or breastfeeding and willing to use contraception.
+Exclusion Criteria:
+* Smoldering multiple myeloma.
+* Plasma cell leukemia.
+* Amyloidosis.
+* Polyneuropathy, organomegaly, endocrinopathy, monoclonal gammopathy and skin abnormalities (POEMS) syndrome.
+* Known central nervous system (CNS) involvement or clinical signs of myelomatous meningeal involvement.
+* Stem cell transplant within 12 weeks prior to enrolment, or active graft versus host disease.
+* Any active, uncontrolled bacterial, fungal, or viral infection.
+* Any other active malignancy within 3 years prior to enrolment (exceptions include, adequately treated basal cell or squamous cell skin cancer, carcinoma in situ)
+* Previous treatment with a B cell maturation antigen (BCMA)-directed therapy or CD3-redirecting therapy.
+* Unable to receive investigator's choice therapy.
+* Live attenuated vaccine within 4 weeks of the first dose of study intervention.
+* Administration with an investigational product (e.g. drug or vaccine) within 30 days preceding the first dose of study intervention used in this study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116"/>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="36" customHeight="1">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Study of Single Agent Belantamab Mafodotin Versus Pomalidomide Plus Low-dose Dexamethasone (Pom/Dex) in Participants With Relapsed/Refractory Multiple Myeloma (RRMM) [NCT04162210]</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Capable of giving signed informed consent.
+* Participants must be 18 or older, at the time of signing the informed consent. In Republic of Korea, participants must be over 19 years of age inclusive, at the time of signing informed consent.
+* Eastern Cooperative Oncology Group (ECOG) performance status of 0 to 2.
+* Histologically or cytologically confirmed diagnosis of Multiple myeloma (MM) as defined according to IMWG, and : Has undergone autologous stem cell transplant (SCT), or is considered transplant ineligible; Has received at least 2 prior lines of anti-myeloma treatments, including at least 2 consecutive cycles of both lenalidomide and a proteasome inhibitor (given separately or in combination), and must have documented disease progression on, or within 60 days of, completion of the last treatment or must be non-responsive while on last treatment, where non-responsive is defined as not achieving at least Minimal Response (MR) after 2 complete treatment cycles. In such cases lack of achieving of at least MR must be determined no earlier than at least 4 weeks after the last treatment.
+* Has measurable disease with at least one of the following: Serum M-protein \&gt;=0.5 gram per deciliter (g/dL) (\&gt;=5 gram per Liter); Urine M-protein \&gt;=200 mg/24 hours; Serum free light chain (FLC) assay: Involved FLC level \&gt;=10 milligram per deciliter (mg/dL) (\&gt;=100 mg/L) and an abnormal serum FLC ratio (\&lt;0.26 or \&gt;1.65).
+* Participants with a history of autologous SCT are eligible for study participation provided the following eligibility criteria are met: Transplant was \&gt;100 days prior to initiating study treatment; No active infection(s).
+* Adequate organ system functions as defined: Absolute neutrophil count (ANC) \&gt;=1.0\*10\^9/L; Hemoglobin \&gt;= 8.0 g/dL; Platelets \&gt;= 50x10\^9/L; Total bilirubin \&lt;=1.5\* Upper limit of normal (ULN) (isolated bilirubin \&gt;1.5\*ULN is acceptable if bilirubin is fractionated and direct bilirubin \&lt;35 percent); ALT \&lt;=2.5\*ULN; Estimated glomerular filtration rate (eGFR) \&gt;=30 milliliter per minute per 1.73 square meter (mL/min/1.73 m\^2); Spot urine (albumin/creatinine ratios) \&lt;=500 milligram per gram (mg/g) (56 milligram per millimoles \[mg/mmol\]).
+* Contraceptive use by men or women should be consistent with local regulations regarding the methods of contraception for those participating in clinical studies. Male participants are eligible to participate if they agree to the following during the intervention period and until 6 months after the last dose of study intervention to allow for clearance of any altered sperm: Refrain from donating sperm PLUS, either: Be abstinent from heterosexual intercourse as their preferred and usual lifestyle (abstinent on a long term and persistent basis) and agree to remain abstinent OR Must agree to use contraception/barrier as detailed below depending on whether they are randomised to Arm 1 (belantamab mafodotin) or Arm 2 (pom/dex), even if they have undergone a successful vasectomy: Agree to use a male condom throughout study treatment including the 6 month follow-up period even if they have undergone a successful vasectomy and a female partner to use an additional highly effective contraceptive method with a failure rate of \&lt;1 percent per year when having sexual intercourse with a pregnant woman or a woman of childbearing potential who is not currently pregnant. Four weeks for male participants on Treatment Arm 2 (pom/dex).
+* A female participant is eligible to participate if she is not pregnant or breastfeeding, and at least one of the following conditions applies: Is not a woman of childbearing potential (WOCBP) OR Is a WOCBP and agrees to abide by the following: Arm 1 (belantamab mafodotin): Use a contraceptive method that is highly effective (with a failure rate of \&lt;1 percent per year) which includes abstinence, preferably with low user dependency during the intervention period and for 4 months after the last dose of study treatment. Arm 2 (pom/dex): Due to pomalidomide being a thalidomide analogue with risk for embryofetal toxicity and prescribed under a pregnancy prevention/controlled distribution program, WOCBP participants will be eligible if they commit either to abstain continuously from heterosexual sexual intercourse or to use two methods of reliable birth control (one method that is highly effective), beginning 4 weeks prior to initiating treatment with pomalidomide, during therapy, during dose interruptions and continuing for at least 4 weeks following discontinuation of pomalidomide treatment. Two negative pregnancy tests must be obtained prior to initiating therapy. The first test should be performed within 10-14 days and the second test within 24 hours prior to prescribing pomalidomide therapy. And agrees not to donate eggs (ova, oocytes) for the purpose of reproduction during this period. The investigator should confirm the effectiveness of the contraceptive method(s) ahead of the first dose of study intervention.
+* All prior treatment-related toxicities (defined by National Cancer Institute- Common Toxicity Criteria for Adverse Events \[NCI-CTCAE\], version 5.0, 2017) must be \&lt;=Grade 1 at the time of enrollment, except for alopecia and Grade 2 peripheral neuropathy.
+Exclusion Criteria:
+* Symptomatic amyloidosis, active POEMS syndrome (polyneuropathy, organomegaly, endocrinopathy, myeloma protein, and skin changes); active plasma cell leukemia at the time of screening.
+* Systemic anti-myeloma therapy or use of an investigational drug within \&lt;14 days or 5 half-lives, whichever is shorter, before the first dose of study intervention.
+* Prior treatment with an anti-MM monoclonal antibody within 30 days prior to receiving the first dose of study intervention.
+* Prior B cell maturation antigen (BCMA)-targeted therapy or prior pomalidomide treatment.
+* Plasmapheresis within 7 days prior to the first dose of study intervention.
+* Prior allogeneic stem cell transplant. (Participants who have undergone syngeneic transplant will be allowed only if no history of, or currently active, Graft-Versus-Host Disease \[GvHD\]).
+* Any major surgery within the last 4 weeks.
+* Presence of active renal condition (infection, requirement for dialysis or any other condition that could affect participant's safety). Participants with isolated proteinuria resulting from MM are eligible, provided they fulfil criteria as described in inclusion criteria.
+* Any serious and/or unstable pre-existing medical, psychiatric disorder, or other conditions (including lab abnormalities) that could interfere with participant's safety, obtaining informed consent, or compliance with study procedures.
+* History of (non-infectious) pneumonitis that required steroids, or current pneumonitis.
+* Evidence of active mucosal or internal bleeding.
+* Current unstable liver or biliary disease per investigator assessment defined by the presence of ascites, encephalopathy, coagulopathy, hypoalbuminaemia, esophageal or gastric varices, persistent jaundice, or cirrhosis. (Stable chronic liver disease \[including Gilbert's syndrome or asymptomatic gallstones\] or hepatobiliary involvement of malignancy is acceptable if participant otherwise meets entry criteria)
+* Participants with previous or concurrent malignancies other than multiple myeloma are excluded, unless the second malignancy has been considered medically stable for at least 2 years. The participant must not be receiving active therapy, other than hormonal therapy for this disease. (Participants with curatively treated non-melanoma skin cancer are allowed without a 2-year restriction).
+* Evidence of cardiovascular risk including any of the following: Evidence of current clinically significant uncontrolled arrhythmias including clinically significant electrocardiogram (ECG) abnormalities including 2nd degree (Mobitz Type II) or 3rd degree atrioventricular block; History of myocardial infarction, acute coronary syndromes (including unstable angina), coronary angioplasty, or stenting or bypass grafting within 3 months of Screening; Class III or IV heart failure as defined by the New York Heart Association (NYHA) functional classification system; Uncontrolled hypertension.
+* Known immediate or delayed hypersensitivity reaction or idiosyncrasy to drugs chemically related to belantamab mafodotin, pomalidomide, dexamethasone or any of the components of the study intervention.
+* Pregnant or lactating female.
+* Active infection requiring treatment.
+* Known human immunodeficiency virus (HIV), unless the participant can meet all of the following criteria: Established anti-retroviral therapy (ART) for at least 4 weeks and HIV viral load \&lt;400 copies/mL; CD4+ T-cell (CD4+) counts ≥350 cells/uL; No history of AIDS-defining opportunistic infections within the last 12 months.(Consideration must be given to ART and prophylactic antimicrobials that may have a drug-drug interaction and/or overlapping toxicities with belantamab mafodotin or other combination products as relevant)
+* Participants with Hepatitis B will be excluded unless the following criteria can be met: If the participant is hepatitis B core antibody (HbcAb) positive or hepatitis B surface antigen (HbsAg) negative, then hepatitis B virus (HBV) deoxyribonucleic acid (DNA) should be undectectable at the time of screening; If HbsAg+ at screening or \&lt;=3 months prior to first dose of study treatment, then HBV DNA should be undetectable, highly effective antiviral treatment should be started ≥4 weeks prior to first dose of study treatment, exclusion of participants with cirrhosis and participants in Japan must test hepatitis B e antigen (HBeAg) and hepatitis B e antibody (HBeAb ).
+* Positive hepatitis C antibody test result or positive hepatitis C Ribonucleic acid (RNA) test result at screening or within 3 months prior to first dose of study treatment unless the participant can meet the following criteria: Hepatitis C RNA test negative at Screening and successful anti-viral treatment (usually 8 weeks duration) is required, followed by a negative HCV RNA test after a washout period of at least 4 weeks (Hepatitis RNA is optional and participants with negative Hepatitis C antibody test are not required to also undergo Hepatitis C RNA testing).
+* Participants unable to tolerate thromboembolic prophylaxis.
+* Current corneal epithelial disease except for mild punctate keratopathy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119"/>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="36" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Improving Pulmonary Hypertension Screening by Echocardiography [NCT06038149]</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Unexplained breathlessness
+* Risk factors for Pulmonary arterial hypertension (PAH), chronic thromboembolic pulmonary hypertension (CTEPH)
+* Unexplained elevation of B-type natriuretic peptide (BNP/proBNP)
+* Referred for catheterisation.
+Exclusion Criteria:
+* ESC / BSE echo high probability of PH
+* Known or suspected congenital heart disease
+* Patients unlikely to benefit from management of PH or its underlying causes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>01-Jul 13:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="36" customHeight="1">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>Ultrasound-facilitated, Catheter-directed, Thrombolysis in Intermediate-high Risk Pulmonary Embolism [NCT04790370]</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 80 Years  |  All
+Inclusion Criteria:
+* Age 18-80 years, inclusive
+* Objectively confirmed acute PE, based on computed tomography pulmonary angiography (CTPA) showing a filling defect in at least one main or proximal lobar pulmonary artery
+* Elevated risk of early death/hemodynamic collapse, indicated by at least two of the following new-onset clinical criteria:
+  1. ECG-documented tachycardia with heart rate ≥100 beats per minute, not due to hypovolemia, arrhythmia, or sepsis;
+  2. SBP ≤ 110 mm Hg for at least 15 minutes;
+  3. respiratory rate \&gt; 20 x min\^-1 or oxygen saturation on pulse oximetry (SpO2) \&lt; 90% (or partial arterial oxygen pressure \&lt; 60 mmHg) at rest while breathing room air;
+* Right-to-left ventricular (RV/LV) diameter ratio ≥ 1.0 on CTPA
+* Serum troponin I or T levels above the upper limit of normal
+* Signed informed consent
+Exclusion Criteria:
+* Hemodynamic instability\*, i.e. at least one of the following present:
+  1. cardiac arrest or need for cardiopulmonary resuscitation;
+  2. need for ECMO, or ECMO initiated before randomization
+  3. PE-related shock, defined as: (i) SBP \&lt; 90 mmHg, or vasopressors required to achieve SBP ≥ 90 mmHg, despite an adequate volume status; and (ii) end-organ hypoperfusion (altered mental status; oliguria/anuria; increased serum lactate);
+  4. isolated persistent hypotension (SBP \&lt; 90 mmHg, or a systolic pressure drop by at least 40 mmHg for at least 15 minutes), not caused by new-onset arrhythmia, hypovolemia, or sepsis \* Patients who presented with temporary need for fluid resuscitation and/or low-dose catecholamines may be included, provided that they could be stabilized within 2 hours of admission and maintain SBP of ≥ 90 mmHg and adequate organ perfusion without catecholamine infusion.
+* Need for admission to an intensive care unit for a reason other than the index PE episode. NB: Patients who test positive for SARS-CoV-2 can be enrolled where the investigator believes that the pulmonary embolism is the dominant pathology in the patient's clinical presentation and qualifying cardiorespiratory parameters.
+* Temperature above 39 degrees C / 102.2 degrees F
+* Logistical reasons limiting the rapid availability of interventional procedures to treat acute PE (e.g., during the outbreak of an epidemic)
+* Index PE symptom duration \&gt; 14 days
+* Active bleeding
+* History of intracranial or intraocular bleeding at any time
+* Stroke or transient ischemic attack within the past 6 months, or previous stroke at any time if associated with permanent disability
+* Central nervous system neoplasm, or metastatic cancer
+* Major neurologic, ophthalmologic, abdominal, cardiac, thoracic, vascular or orthopedic surgery or trauma (including syncope-associated with head strike or skeletal fracture) within the past 3 weeks
+* Platelet count \&lt; 100 x 10\^9 x L\^-1
+* Patients who have received a once-daily therapeutic dose of LMWH or a therapeutic dose of fondaparinux within 24 hours prior to randomization
+* Patients who have received one of the direct oral anticoagulants apixaban or rivaroxaban within 12 hours prior to randomization
+* Patients who have received one of the direct oral anticoagulants dabigatran or edoxaban for the index PE episode, as these drugs are not approved for patients who have not received heparin for at least 5 days
+* Administration of a thrombolytic agent or a glycoprotein IIb/IIIa receptor antagonist during the current hospital stay and/or within 30 days, for any reason
+* Chronic treatment with antiplatelet agents other than low-dose acetylsalicylic acid or clopidogrel 75 mg once daily (but not both). Dual antiplatelet therapy is excluded.
+* Chronic treatment with a direct oral anticoagulant (apixaban, dabigatran, edoxaban or rivaroxaban)
+* Chronic treatment with a vitamin K antagonist, or known coagulopathy including severe hepatic dysfunction, with an International Normalized Ratio (INR) \&gt; 1.5
+* Pregnancy or lactation
+* Previous inclusion in the study
+* Known hypersensitivity to alteplase, LMWH or UFH, or to any of the excipients
+* Life expectancy less than 6 months</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor update 2026-07-01 16:05 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -3307,7 +3307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C124"/>
+  <dimension ref="A3:C124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3315,8 +3315,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3365,7 +3363,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3407,7 +3404,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3465,7 +3461,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -3519,7 +3514,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -3598,7 +3592,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -3673,7 +3666,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -3724,7 +3716,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -3760,7 +3751,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -3799,7 +3789,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -3833,7 +3822,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
@@ -3882,7 +3870,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
@@ -3944,7 +3931,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
@@ -3989,7 +3975,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
@@ -4031,7 +4016,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
@@ -4080,7 +4064,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
@@ -4117,7 +4100,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
@@ -4166,7 +4148,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -4214,7 +4195,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
@@ -4263,7 +4243,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
@@ -4301,7 +4280,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
@@ -4351,7 +4329,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
@@ -4403,7 +4380,6 @@
         </is>
       </c>
     </row>
-    <row r="68"/>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
@@ -4453,7 +4429,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
@@ -4494,7 +4469,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -4558,7 +4532,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
@@ -4590,7 +4563,6 @@
         </is>
       </c>
     </row>
-    <row r="80"/>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
@@ -4632,7 +4604,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
@@ -4670,7 +4641,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
@@ -4707,7 +4677,6 @@
         </is>
       </c>
     </row>
-    <row r="89"/>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
@@ -4745,7 +4714,6 @@
         </is>
       </c>
     </row>
-    <row r="92"/>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
@@ -4785,7 +4753,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
@@ -4825,7 +4792,6 @@
         </is>
       </c>
     </row>
-    <row r="98"/>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
@@ -4868,7 +4834,6 @@
         </is>
       </c>
     </row>
-    <row r="101"/>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -4920,7 +4885,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
@@ -4971,7 +4935,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
@@ -5036,7 +4999,6 @@
         </is>
       </c>
     </row>
-    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
@@ -5070,7 +5032,6 @@
         </is>
       </c>
     </row>
-    <row r="113"/>
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
         <is>
@@ -5115,7 +5076,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
@@ -5174,7 +5134,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Monitor update 2026-07-02 12:29 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -1146,7 +1146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B142"/>
+  <dimension ref="A3:B166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3296,6 +3296,318 @@
         </is>
       </c>
     </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="36" customHeight="1">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>A Study of NX-5948 in Adults With CLL/SLL Previously Treated With a Bruton's Tyrosine Kinase Inhibitor and a B-cell Lymphoma-2 Inhibitor (DAYBreak CLL-201) [NCT07221500]</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Age: ≥ 18 years
+* Confirmed relapsed/refractory CLL/SLL that meets iwCLL criteria for diagnosis and systemic treatment
+* Eastern Cooperative Oncology Group (ECOG) performance status of 0-2
+* Must have received a covalent BTK inhibitor (BTKi), a non-covalent BTKi, and a BCL-2 inhibitor either in separate lines of therapy or in combination; a line of therapy is considered 2 or more consecutive cycles of a systemic anti-CLL/SLL regimen
+* Participants with SLL must have measurable disease by radiographic assessment
+* Adequate organ and bone marrow function
+* Must sign an informed consent form indicating that he or she understands the purpose of the procedures required for the study and is willing to participate
+Exclusion Criteria:
+* Known or suspected prolymphocytic leukemia or Richter's transformation before entering study
+* Investigational agent or anticancer therapy within 5 half-lives or 14 days (whichever is shorter) before planned start of study drug
+  * Antibody therapy must stop at least 4 weeks before the first dose of study drug
+  * No other systemic anticancer therapy is allowed at the same time as this study; exception: continuation of hormonal therapy for breast and prostate cancer is allowed, if they are not on the list of prohibited concomitant medications in this study
+* Palliative limited-field radiotherapy within 7 days of the first dose of study or broad field radiotherapy within 28 days of first dose of study drug
+* Use of systemic corticosteroids \&gt;20 mg/day prednisone or equivalent within the 7 days before start of study drug except for those used as premedication for radio diagnostic contrast
+* Use of systemic immunosuppressive drugs other than systemic corticosteroids within 60 days before the first dose of study drug
+* Previously treated with a BTK degrader
+* Previous chimeric antigen receptor (CAR) T-cell therapy or allogeneic or autologous hematopoietic cell transplant within the past 90 days prior to enrollment
+* Thromboembolic events (eg, deep vein thrombosis, pulmonary embolism, or symptomatic cerebrovascular events), stroke, or intracranial hemorrhage within 6 months of planned start of study drug
+Note: Other Inclusion/Exclusion criteria may apply as defined in the protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="36" customHeight="1">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>Sacituzumab Tirumotecan (MK-2870) in Combination With Pembrolizumab Versus Pembrolizumab Alone in Metastatic Non-small Cell Lung Cancer (NSCLC) With Programmed Cell Death Ligand 1 (PD-L1) Tumor Proportion Score (TPS) ≥ 50% (MK-2870-007) [NCT06170788]</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Histologically or cytologically confirmed diagnosis of squamous or nonsquamous NSCLC
+  * Confirmation that epidermal growth factor receptor- (EGFR-), anaplastic lymphoma kinase- (ALK-), or proto-oncogene tyrosine-protein kinase ROS (ROS1-) directed therapy is not indicated as primary therapy
+  * Provided tumor tissue that demonstrates programmed cell death ligand 1 (PD-L1) expression in ≥50% of tumor cells as assessed by an immunohistochemistry (IHC) central laboratory
+  * An Eastern Cooperative Oncology Group (ECOG) performance status of 0 to 1 assessed within 7 days before randomization.
+  * A life expectancy of at least 3 months.
+  * Human immunodeficiency virus (HIV)-infected participants must have well controlled HIV on antiretroviral therapy (ART)
+Exclusion Criteria:
+* Diagnosis of small cell lung cancer or, for mixed tumors, presence of small cell elements.
+* Has Grade ≥2 peripheral neuropathy.
+* History of documented severe dry eye syndrome, severe Meibomian gland disease and/or blepharitis, or severe corneal disease that prevents/delays corneal healing.
+* Has active inflammatory bowel disease requiring immunosuppressive medication or previous clear history of inflammatory bowel disease (eg, Crohn's disease, ulcerative colitis, or chronic diarrhea).
+* Has uncontrolled, significant cardiovascular disease or cerebrovascular disease within the 6 months preceding study intervention.
+* Received prior systemic anticancer therapy for their metastatic NSCLC.
+* Received prior therapy with an anti-PD-1, anti-PD-L1, or anti-PD-L2 agent, or with an agent directed to another stimulatory or coinhibitory T-cell receptor Note: Prior treatment with an anti-PD-1, anti-PD- L1, or anti-PD-L2 agent in the neoadjuvant or adjuvant setting for nonmetastatic resectable NSCLC is allowed as long as therapy was completed at least 12 months before diagnosis of metastatic NSCLC.
+* Received prior systemic anticancer therapy including investigational agents within 4 weeks before randomization.
+* Received radiation therapy to the lung that is \&gt;30 Gy within 6 months of start of study intervention.
+* Received prior radiotherapy within 2 weeks of start of study intervention, or radiation-related toxicities, requiring corticosteroids.
+* Received a live or live-attenuated vaccine within 30 days before the first dose of study intervention. Administration of killed vaccines are allowed.
+* Diagnosis of immunodeficiency or is receiving chronic systemic steroid therapy
+* Known additional malignancy that is progressing or has required active treatment within the past 3 years.
+* Known active central nervous system (CNS) metastases and/or carcinomatous meningitis.
+* Known intolerance to sacituzumab tirumotecan or pembrolizumab and/or any of their excipients; for pembrolizumab, severe hypersensitivity (≥Grade 3) is exclusionary.
+* Known hypersensitivity to sacituzumab tirumotecan or other biologic therapy.
+* Active autoimmune disease that has required systemic treatment in the past 2 years.
+* History of (noninfectious) pneumonitis/interstitial lung disease (ILD) that required steroids or has current pneumonitis/ILD.
+* Active infection requiring systemic therapy
+* Concurrent active Hepatitis B and Hepatitis C virus infection.
+* Human immunodeficiency virus (HIV)-infected participants with a history of Kaposi's sarcoma and/or Multicentric Castleman's Disease.
+* History of allogeneic tissue/solid organ transplant.
+* Requires treatment with a strong inhibitor or inducer of Cytochrome P450 3A4 (CYP3A4) at least 14 days before the first dose of study intervention and throughout the study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="22" customHeight="1">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="36" customHeight="1">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Compare Iberdomide Maintenance Versus Lenalidomide Maintenance Therapy Following Autologous Stem Cell Transplant in Participants With Newly Diagnosed Multiple Myeloma [NCT05827016]</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Confirmed diagnosis of symptomatic multiple myeloma (MM).
+* Eastern Cooperative Oncology Group performance status (ECOG) score of 0, 1, or 2.
+* Received 3 to 6 cycles of an induction therapy that includes a proteasome inhibitor (PI) and immunomodulatory (IMiD) \[eg, bortezomib thalidomide and dexamethasone (VTd), lenalidomide, bortezomib and dexamethasone (RVd)\] with or without a CD38 monoclonal antibody, daratumumab + bortezomib/thalidomide/dexamethasone \[D-VTd\] and daratumumab + bortezomib/ lenalidomide/dexamethasone \[D-VRd\]), or VCd / daratumumab + bortezomib/cyclophosphamide/dexamethasone \[D-VCd\], and followed by a single or tandem autologous stem cell transplantation (ASCT). Post-stem cell transplant consolidation is permitted.
+* Participants within 12 months (single transplant) or 15 months (tandem transplant) from initiation of induction therapy who achieved at least a partial response (PR) after autologous stem cell transplantation (ASCT) with or without consolidation, according to International Myeloma Working Group (IMWG 2016) criteria.
+Exclusion Criteria
+* Progressive disease or clinical relapse (as defined by IMWG response criteria) following ASCT with or without consolidation or is not responsive to primary therapy.
+* Smoldering myeloma, solitary plasmacytoma or nonsecretory myeloma.
+* Known central nervous system/meningeal involvement of MM.
+* Prior history of malignancies, other than MM, unless the participant has been free of the disease for ≥ 5 years.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="36" customHeight="1">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>Study of Efficacy and Safety of JDQ443 Single-agent as First-line Treatment for Patients With Locally Advanced or Metastatic KRAS G12C- Mutated Non-small Cell Lung Cancer With a PD-L1 Expression &lt; 1% or a PD-L1 Expression ≥ 1% and an STK11 Co-mutation. [NCT05445843]</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 100 Years  |  All
+Key Inclusion criteria
+* Histologically confirmed locally advanced (stage IIIb/IIIc not eligible for definitive chemoradiation or surgical resection with curative intent) or metastatic (stage IV) NSCLC without previous systemic treatment for metastatic disease. Prior (neo)adjuvant treatment with chemotherapy and/or immunotherapy, or prior radiotherapy administered sequentially or concomitantly with chemotherapy and/or immunotherapy for localized or locally advanced disease are accepted if the time between therapy completion and enrollment is \&gt; 12 months.
+* Presence of a KRAS G12C mutation (all participants) and:
+  * Cohort A: PD-L1 expression \&lt; 1%, regardless of STK11 mutation status
+  * Cohort B: PD-L1 expression ≥ 1% and an STK11 co-mutation
+* At least one measurable lesion per RECIST 1.1.
+* ECOG performance status ≤ 1.
+* Participants capable of swallowing study medication.
+Key Exclusion criteria
+* Participants whose tumors harbor an EGFR-sensitizing mutation and/or ALK rearrangement by local laboratory testing. Participants with other known druggable alterations will be excluded, if required by local guidelines
+* Previous use of a KRAS G12C inhibitor or previous systemic treatment for metastatic NSCLC.
+* A medical condition that results in increased photosensitivity (i.e., solar urticaria, lupus erythematosus, etc.).
+* Known active central nervous system (CNS) metastases and/or carcinomatous meningitis
+* Participants who are taking a prohibited medication (strong CYP3A inducers) that cannot be discontinued at least seven days prior to the first dose of study treatment and for the duration of the study.
+Other inclusion/exclusion criteria may apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="22" customHeight="1">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="36" customHeight="1">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Study to Evaluate Efficacy and Safety of Firmonertinib Compared With Investigator's Choice of EGFR Inhibitor as First-Line Treatment in Participants Who Have Locally Advanced or Metastatic NSCLC With EGFR P-Loop and Alpha C-Helix Compressing (PACC) Uncommon Mutations [NCT07185997]</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Key Eligibility Criteria:
+* Histologically or cytologically documented, locally advanced or metastatic Non-Small Cell Lung Cancer (NSCLC) not amenable to curative surgery or radiotherapy.
+* Documented results of the presence of an Epidermal Growth Factor Receptor (EGFR) PACC mutation in tumor tissue or blood from local testing.
+* No prior systemic anticancer therapy regimens received for locally advanced or metastatic Non-Small Cell Lung Cancer (NSCLC) including prior treatment with any Epidermal Growth Factor Receptor (EGFR)-targeting agents (e.g., previous (EGFR) TKIs, monoclonal antibodies, or bispecific antibodies).
+* Patients who have received prior neo-adjuvant and/or adjuvant chemotherapy, immunotherapy, or chemo radiotherapy for non-metastatic disease must have experienced a treatment free interval of at least 12 months.
+* Patients with asymptomatic CNS metastases are eligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="22" customHeight="1">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="36" customHeight="1">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>Study of Sotorasib, Panitumumab and FOLFIRI Versus FOLFIRI With or Without Bevacizumab-awwb in Treatment-naïve Participants With Metastatic Colorectal Cancer With KRAS p.G12C Mutation [NCT06252649]</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Pathologically documented metastatic colorectal adenocarcinoma with KRAS p.G12C mutation by a locally validated assay.
+* Central laboratory detection of KRAS p.G12C mutation.
+* Measurable metastatic disease per RECIST v1.1 criteria.
+* Eastern Cooperative Oncology Group (ECOG) Performance Status of ≤ 1.
+* Adequate organ function.
+Exclusion Criteria:
+* Active, untreated brain metastases.
+* Leptomeningeal disease
+* Previous treatment with a KRAS p.G12C inhibitor
+* History of interstitial pneumonitis or pulmonary fibrosis or evidence of interstitial pneumonitis or pulmonary fibrosis on baseline CT scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="22" customHeight="1">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="36" customHeight="1">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Quizartinib or Placebo Plus Chemotherapy in Newly Diagnosed Patients With FLT3-ITD Negative AML [NCT06578247]</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – 70 Years  |  All
+Key Inclusion Criteria:
+1. Must be competent and able to comprehend, sign, and date an Ethics Committee (EC)- or Institutional Review Board (IRB)-approved ICF before performance of any trial-specific procedures or tests.
+2. ≥18 years or the minimum legal adult age (whichever is greater) and ≤70 years (at Screening).
+3. Newly diagnosed, morphologically documented primary AML based on the World Health Organization (WHO) 2016 classification (at Screening)
+4. Eastern Cooperative Oncology Group (ECOG) performance status (at the time the participant signs their ICF) of 0-2.
+5. Participant is a candidate for standard "7+3" induction chemotherapy regimen as specified in the protocol per investigator assessment
+Key Exclusion Criteria:
+1. Diagnosis of acute promyelocytic leukemia (APL), French-American-British classification M3 or WHO classification of APL with translocation, t(15;17)(q22;q12), or BCR-ABL positive leukemia (ie, chronic myelogenous leukemia in blast crisis); participants who undergo diagnostic workup for APL and treatment with all-trans retinoic acid (ATRA), but who are found not to have APL, are eligible (treatment with ATRA must be discontinued before starting induction chemotherapy).
+2. Diagnosis of AML secondary to prior chemotherapy or radiotherapy.
+3. Diagnosis of AML with known antecedent myelodysplastic syndrome (MDS) or a myeloproliferative neoplasm (MPN) or MDS/MPNs including chronic myelomonocytic leukemia (CMML), atypical chronic myeloid leukemia (aCML), juvenile myelomonocytic leukemia (JMML) and others.
+4. Participants with newly diagnosed AML with FLT3-ITD mutations (FLT3-ITD \[+\]) present at ≥5% VAF (or ≥0.05 SR) based on a validated FLT3 mutation assay.
+5. Prior treatment for AML, except for the following allowances prior to Day 1 of chemotherapy:
+   1. Leukapheresis;
+   2. Treatment for hyperleukocytosis with hydroxyurea;
+   3. Cranial radiotherapy for central nervous system (CNS) leukostasis;
+   4. Prophylactic intrathecal chemotherapy</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="22" customHeight="1">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="36" customHeight="1">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>Pan Tumor Rollover Study [NCT03899155]</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Signed Written Informed Consent.
+* Eligible to receive continued study treatment per the Parent Study, including treatment beyond progression per investigator assessment in the Parent Study.
+* On treatment hold in the Parent Study following long-lasting response or are eligible for treatment rechallenge as defined in the Parent Study.
+* WOCBP and male participants who are sexually active must agree to follow instructions for method(s) of contraception as described below and included in the ICF.
+Exclusion Criteria
+* Participant is not eligible for study treatment per the Parent Study eligibility criteria.
+* Participants not receiving clinical benefit as assessed by the Investigator.
+* Any clinical adverse event (AE), laboratory abnormality, or intercurrent illness which, in the opinion of the Investigator, indicates that participation in the study is not in the best interest of the participant.
+* Other protocol-defined Inclusion/Exclusion Criteria apply</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3307,7 +3619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:C124"/>
+  <dimension ref="A1:C148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3315,6 +3627,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3363,6 +3677,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3404,6 +3719,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3461,6 +3777,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -3514,6 +3831,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -3592,6 +3910,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -3666,6 +3985,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -3716,6 +4036,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -3751,6 +4072,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -3789,6 +4111,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -3822,6 +4145,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
@@ -3870,6 +4194,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
@@ -3931,6 +4256,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
@@ -3975,6 +4301,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
@@ -4016,6 +4343,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
@@ -4064,6 +4392,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
@@ -4100,6 +4429,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
@@ -4148,6 +4478,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -4195,6 +4526,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
@@ -4243,6 +4575,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
@@ -4280,6 +4613,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
@@ -4329,6 +4663,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
@@ -4380,6 +4715,7 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
@@ -4429,6 +4765,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
@@ -4469,6 +4806,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -4532,6 +4870,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
@@ -4563,6 +4902,7 @@
         </is>
       </c>
     </row>
+    <row r="80"/>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
@@ -4604,6 +4944,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
@@ -4641,6 +4982,7 @@
         </is>
       </c>
     </row>
+    <row r="86"/>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
@@ -4677,6 +5019,7 @@
         </is>
       </c>
     </row>
+    <row r="89"/>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
@@ -4714,6 +5057,7 @@
         </is>
       </c>
     </row>
+    <row r="92"/>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
@@ -4753,6 +5097,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
@@ -4792,6 +5137,7 @@
         </is>
       </c>
     </row>
+    <row r="98"/>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
@@ -4834,6 +5180,7 @@
         </is>
       </c>
     </row>
+    <row r="101"/>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -4885,6 +5232,7 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
@@ -4935,6 +5283,7 @@
         </is>
       </c>
     </row>
+    <row r="107"/>
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
@@ -4999,6 +5348,7 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
@@ -5032,6 +5382,7 @@
         </is>
       </c>
     </row>
+    <row r="113"/>
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
         <is>
@@ -5076,6 +5427,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
@@ -5134,6 +5486,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
         <is>
@@ -5167,6 +5520,7 @@
         </is>
       </c>
     </row>
+    <row r="122"/>
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
         <is>
@@ -5225,6 +5579,395 @@
 * Previous inclusion in the study
 * Known hypersensitivity to alteplase, LMWH or UFH, or to any of the excipients
 * Life expectancy less than 6 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="125"/>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="36" customHeight="1">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Compare Iberdomide Maintenance Versus Lenalidomide Maintenance Therapy Following Autologous Stem Cell Transplant in Participants With Newly Diagnosed Multiple Myeloma [NCT05827016]</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Status: ACTIVE_NOT_RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Confirmed diagnosis of symptomatic multiple myeloma (MM).
+* Eastern Cooperative Oncology Group performance status (ECOG) score of 0, 1, or 2.
+* Received 3 to 6 cycles of an induction therapy that includes a proteasome inhibitor (PI) and immunomodulatory (IMiD) \[eg, bortezomib thalidomide and dexamethasone (VTd), lenalidomide, bortezomib and dexamethasone (RVd)\] with or without a CD38 monoclonal antibody, daratumumab + bortezomib/thalidomide/dexamethasone \[D-VTd\] and daratumumab + bortezomib/ lenalidomide/dexamethasone \[D-VRd\]), or VCd / daratumumab + bortezomib/cyclophosphamide/dexamethasone \[D-VCd\], and followed by a single or tandem autologous stem cell transplantation (ASCT). Post-stem cell transplant consolidation is permitted.
+* Participants within 12 months (single transplant) or 15 months (tandem transplant) from initiation of induction therapy who achieved at least a partial response (PR) after autologous stem cell transplantation (ASCT) with or without consolidation, according to International Myeloma Working Group (IMWG 2016) criteria.
+Exclusion Criteria
+* Progressive disease or clinical relapse (as defined by IMWG response criteria) following ASCT with or without consolidation or is not responsive to primary therapy.
+* Smoldering myeloma, solitary plasmacytoma or nonsecretory myeloma.
+* Known central nervous system/meningeal involvement of MM.
+* Prior history of malignancies, other than MM, unless the participant has been free of the disease for ≥ 5 years.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128"/>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="36" customHeight="1">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate the Safety and Effectiveness of the Rapidlink Device When Used in Patients Undergoing an Open Surgical Procedure to Repair the Aorta [NCT07078383]</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Patient is aged 18 years or over on date of consent
+* Written informed consent (from patient or a legally authorized representative) to participate in study, documenting willingness and ability to comply with all study procedures and study visits (unless an exemption for emergency cases has been IRB / EC approved)
+* Patient's need for open surgical repair of the thoracic aorta using a Gelweave graft or a Thoraflex Hybrid device (AnteFlo or Plexus) in line with the applicable IFU
+* Anticipated need to use Rapidlink for the repair or replacement of the LSA, LCCA and/or IA during the open surgical repair
+* Patient has an 8-15 mm inner diameter (target SAV)
+* The diameters of the patient's target supra-aortic vessel(s), fall within the ranges specified in the IFU
+Exclusion Criteria:
+* Patient does not have a clear landing zone equal to the implantable stent length which is free from stenosis, calcification or thrombus.
+* Patient does not have a sealing zone free from tortuosity.
+* Patient has significant angulation (\&gt;79° with an internal radius of less than 6mm) for the full implantable stent length
+* Patient cannot receive anticoagulation / antiplatelet therapy during or after the index procedure as per the protocol
+* Patient has uncontrolled hypercoagulation
+* Patient has a condition which may compromise or prevent the necessary imaging requirements
+* Patient has anatomic variants which would compromise circulation to the first branch off the target artery after placement of the Rapidlink device (unless planned and/or otherwise revascularized)
+* Patient is unfit for open surgical repair involving circulatory arrest per the study investigator
+* Patient has known sensitivity to polyester, nitinol, tantalum, or materials of bovine origin
+* Patient has a ruptured aorta
+* Patient has active endocarditis or an active infective disorder of the aorta
+* Patient has an active systemic infection that, in the opinion of the investigator, would compromise the outcome of the surgical procedure
+* Patient is enrolled in another active study and has received an investigational product (device, pharmaceutical or biologic) within 6 months prior to the date of the implant or has not reached the primary endpoint of the study
+* Patient is female and is pregnant or planning to become pregnant during the course of the study. Females of childbearing potential must use acceptable methods of contraception during the course of the study.
+* Patient has an uncorrectable bleeding anomaly
+* Patient has renal failure (defined as dialysis dependent or serum creatinine ≥2.5mg/dL)
+* Patient has known sensitivity to radiopaque contrast agents that cannot be adequately pre-treated
+* Patient has a co-morbidity causing expected survival to be less than 1 year
+* Patient has any other medical, social or psychological problems that in the opinion of the investigator preclude them from receiving this treatment and the procedures and evaluations pre and post procedure
+* Patient has a known chronic aortic dissection involving the intended landing zone of the target supra-aortic vessel(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131"/>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="36" customHeight="1">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>DEFIANCE: RCT of ClotTriever System Versus Anticoagulation In Deep Vein Thrombosis [NCT05701917]</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+* Age ≥ 18 years
+* Proximal lower extremity unilateral DVT involving at least the common femoral, external iliac, or common iliac veins, alone or in combination
+* Symptom onset within 12 weeks of enrollment in the study
+* Significant symptoms, as defined by a Villalta score \&gt; 9
+* Willing and able to provide informed consent
+Exclusion Criteria
+* Bilateral iliofemoral DVT
+* Prior venous stent in the target venous segment
+* IVC aplasia/hypoplasia or other congenital anatomic anomalies of the IVC or iliac veins
+* IVC filter in place at the time of enrollment
+* Limb-threatening circulatory compromise (e.g., phlegmasia)
+* Clot in transit including IVC thrombus presenting as extension of \&gt;2cm into the IVC from the CIV
+* Symptomatic PE with right heart strain where the physician judges that a DVT intervention is inappropriate at this time.
+* Inability to be a candidate for intervention due to medical or technical reasons based on physician judgement
+* Severe allergy, hypersensitivity to, or thrombocytopenia from heparin
+* Severe allergy to iodinated contrast agents that cannot be mitigated
+* Hemoglobin \&lt; 8.0 g/dL, INR \&gt; 1.7 before warfarin was started, or platelets \&lt; 50,000/µl which cannot be corrected prior to enrollment
+* Severe renal impairment (estimated GFR \&lt; 30 ml/min) in patients who are not yet on dialysis
+* Inability to provide therapeutic anticoagulation per Investigator discretion
+* Uncontrolled severe hypertension on repeated readings (systolic \&gt; 180mmHg or diastolic \&gt; 105mmHg)
+* Recently (\&lt; 30 days) had DVT interventional procedure
+* Subject is participating in another study that may interfere with this study
+* Life expectancy \&lt; 6 months or chronic non-ambulatory status
+* Known hypercoagulable states that, in the opinion of the Investigator, cannot be medically managed throughout the study period
+* Subject has any condition for which, in the opinion of the Investigator, participation would not be in the best interest of the subject (e.g., contraindication to use of ClotTriever per local approved labeling, compromise the well-being or that could prevent, limit, or confound the protocol-specified assessments)
+* Subject has previously completed or withdrawn from this study
+* Patient unwilling or unable to conduct the follow up visits per protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="134"/>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="36" customHeight="1">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Maridebart Cafraglutide in Heart Failure With Preserved or Mildly Reduced Ejection Fraction and Obesity [NCT07037459]</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – 99 Years  |  All
+Inclusion Criteria:
+* Age ≥ 18 years at the time of informed consent.
+* BMI ≥ 30.0 kg/m\^2 at randomization.
+* HF diagnosed for at least 30 days with New York Heart Association (NYHA) Class II-IV at the time of informed consent.
+* Managed with HF standard of care therapies.
+* Left ventricular ejection fraction (LVEF) of \&gt; 40% within 12 months before randomization.
+Exclusion Criteria:
+* History of any of the following within 60 days prior to or during screening: Type I (spontaneous) MI, valvular replacement or repair, coronary revascularization, coronary artery bypass graft surgery or other major cardiovascular surgery, stroke.
+* HF due to: hypertrophic cardiomyopathy, infiltrative cardiomyopathy, active or chronic myocarditis, constrictive pericarditis, cardiac tamponade, arrhythmogenic right ventricular or left ventricular cardiomyopathy/dysplasia, uncorrected primary valvular heart disease, clinically significant congenital heart disease.
+* Hospitalized with acute decompensated HF at the time of or during the screening period.
+* Type 1 diabetes mellitus, or any type of diabetes with the exception of T2DM or history of gestational diabetes.
+* For participants with a prior diagnosis of T2DM (including those diagnosed during screening):
+  1. HbA1c \&gt; 10.0% (86 mmol/mol) at screening
+  2. Uncontrolled diabetes requiring immediate therapy
+  3. History of diabetic ketoacidosis or hyperosmolar state/coma within 12 months before randomization
+  4. One or more episodes of severe hypoglycemia within 6 months before randomization and/or history of hypoglycemia unawareness
+  5. History or presence of either proliferative diabetic retinopathy, or diabetic maculopathy, or severe non-proliferative diabetic retinopathy; or currently receiving or planning to receive treatment for diabetic retinopathy and/or macular edema.
+* SBP ≥ 180 mmHg during the screening period, or on three or more blood pressure-lowering drugs with a SBP \&gt; 160 mmHg during the screening period (including day 1 prior to randomization).
+* History of chronic pancreatitis or acute pancreatitis in the 180 days before screening or during the screening period.
+* Any personal lifetime history of, or family history(first-degree relative\[s\]) of medullary thyroid carcinoma or MEN-2.
+* eGFR \&lt; 20 mL/min/1.73 m\^2 (CKD-EPI creatinine (Cr)-cystatin C equation) or receiving dialysis at screening.
+* Calcitonin ≥ 50 ng/L (pg/mL) at screening.
+* Acute or chronic hepatitis.
+* Any of the following psychiatric history:
+  1. History of unstable major depressive disorder or other severe psychiatric disorder within 2 years prior to screening or during the screening period
+  2. Lifetime history of suicide attempt
+  3. History of non-suicidal self-injury within 5 years prior to screening or during the screening period.
+* History of any other condition that, in the opinion of the investigator, may preclude the participant from following the protocol and completing the trial.
+* Use of any glucagon-like peptide 1 receptor agonist (GLP-1 RA), glucose-dependent insulinotropic polypeptide (GIP) agonists or antagonists, or amylin analogs within 90 days prior to or during the screening period or planned use during the conduct of the trial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137"/>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="36" customHeight="1">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>A Study of NX-5948 in Adults With Relapsed/Refractory B-cell Malignancies [NCT05131022]</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Key Inclusion Criteria:
+* Age ≥18 years
+* Patients in Phase 1a (Dose Escalation) must have histologically confirmed R/R CLL, SLL, DLBCL (subgroups include Richter-transformed DLBCL, germinal center B-cell type, activated B-cell type, high-grade B-cell lymphoma with MYC and BCL-2 and/or BCL-6 rearrangements, high-grade B-cell lymphomas NOS), FL, MCL, MZL (subtypes include EMZL, MALT, NMZL, SMZL), WM, or PCNSL.
+* Patients in Phase 1a must meet the following:
+  o For non-PCNSL indications, received at least 2 prior lines of therapy and have no other available therapies known to provide clinical benefit. For PCNSL, received at least 1 prior line of therapy
+* Patients in Phase 1b (Safety and Cohort Expansion) must have 1 of the following histologically documented B-cell malignancies, must meet criteria for systemic treatment, and must have received prior therapies and/or molecular features based on details described for each cohort: CLL or SLL, DLBCL, MCL, FL, MZL, WM, or PCNSL/SCNSL.
+* Measurable disease per response criteria specific to the malignancy.
+* Eastern Cooperative Oncology Group (ECOG) performance status of 0 or 1 (0-2 for patients with PCNSL and secondary CNS involvement).
+* Adequate organ and bone marrow function
+Key Exclusion Criteria:
+* Known or suspected active prolymphocytic leukemia or Richter's transformation to Hodgkin's lymphoma prior to study enrollment
+* Prior treatment for the indication under study for anti-cancer intent that includes:
+  1. Radiotherapy within 2 weeks of planned start of study drug (excluding limited palliative radiation).
+  2. Prior systemic chemotherapy within 2 weeks of planned start of study drug.
+  3. Prior monoclonal antibody therapy within 4 weeks of planned start of study drug, except for patients enrolling in Cohort 16 (CLL with secondary wAIHA) where a 16-week washout period is required.
+  4. Prior small molecule therapy within 2 weeks or 5 half-lives (whichever is shorter) of planned start of study drug.
+  5. Autologous or allogeneic stem cell transplant within 100 days prior to planned start of study drug.
+  6. Chimeric antigen receptor (CAR) T-cell therapy within 100 days prior to start of study drug (within 60 days prior to start of study drug for Phase 1b).
+  7. Use of systemic corticosteroids outside of dosing limits described below and within 7 days prior to initiation of study treatment excepting those used as prophylaxis for radio diagnostic contrast. Patients with PCNSL/SCNSL: no greater than 40 mg/day prednisone, or equivalent. Patients with PCNSL/SCNSL using greater than 20 mg/day prednisone, or equivalent, must be clinically stable at that dose for 7 days. All other diagnoses: no greater than 20 mg/day prednisone or equivalent.
+  8. Use of systemic immunosuppressive drugs other than systemic corticosteroids for any medical condition within 60 days prior to first dose of study drug
+  9. Previously treated with a BTK degrader
+* Active, uncontrolled autoimmune hemolytic anemia (except for patients enrolling in Cohort 16) or active, uncontrolled autoimmune thrombocytopenia.
+* Patient has any of the following within 6 months of planned start of study drug:
+  1. Myocardial infarction, unstable angina, unstable symptomatic ischemic heart disease, or placement of a coronary arterial stent
+  2. Uncontrolled atrial fibrillation or other clinically significant arrhythmias, conduction abnormalities, or New York Heart Association (NYHA) class III or IV heart failure
+  3. Thromboembolic events (e.g., deep vein thrombosis, pulmonary embolism, or symptomatic cerebrovascular events), stroke, or intracranial hemorrhage
+  4. Any other significant cardiac condition (e.g., pericardial effusion, restrictive cardiomyopathy, severe untreated valvular stenosis, severe congenital heart disease, or persistent uncontrolled hypertension defined as systolic blood pressure \&gt; 160 mmHg or diastolic blood pressure \&gt; 100 mmHg despite optimal medical management)
+* Bleeding diathesis, or other known risk for acute blood loss.
+* History of Grade ≥ 2 hemorrhage within 28 days of planned start of study drug.
+* Active known concurrent malignancy or malignancy other than the one under study within the past 3 years. (Exceptions include, but are not limited to, patients with more recent history of basal or squamous cell skin cancer, superficial bladder cancer, or carcinoma in situ of the cervix or breast may enroll if they have undergone curative therapy and have no evidence of disease).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140"/>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="36" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>Thromboprophylaxis in Lower Limb Immobilisation [NCT06370273]</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 16 Years – Not specified  |  All
+Inclusion Criteria:
+* Age \&gt;/= 16 years
+* Placed in temporary lower limb immobilisation (rigid cast or brace) as a result an injury that occurred within the last 7 calendar days
+Exclusion Criteria:
+* Hospital admission is required direct from the emergency department, minor injuries unit, or fracture clinic setting with an expected length of stay \&gt;2 calendar days.
+* Absolute contraindication or known hypersensitivity to anticoagulants, including history of end stage renal failure (eGFR \&lt;20ml/min/1.73m2), hepatic failure or use of concomitant systemic treatment with azole-antimycotics (such as ketoconazole, itraconazole, voriconazole and posaconazole), HIV protease inhibitors (e.g. ritonavir) or active substances strongly inhibiting elimination pathways such as CYP3A4 or P-gp (such as clarithromycin, erythromycin or dronaderone) or a history of heparin induced thrombocytopenia.
+* Pregnancy, actively seeking conception, or active breastfeeding.
+* Preceding use of anticoagulant treatment for \&gt;3 calendar days at prophylactic or therapeutic dose.
+* Prior enrolment in the TiLLI study.
+* Non-rigid immobilisation (crepe bandage, tubigrip support, strapping).
+* Time since prescription of rigid immobilisation \&gt;3 calendar days
+* Co-enrolment onto a CTIMP where an anticoagulant is administered
+* People lacking the capacity to consent
+* Inability or refusal to use acceptable contraception up until after the last administration of IMP. Only applicable for women of childbearing potential who have been randomised to receive apixaban or rivaroxaban</t>
+        </is>
+      </c>
+    </row>
+    <row r="143"/>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="36" customHeight="1">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>A Study to Evaluate Mezigdomide, Bortezomib and Dexamethasone (MEZIVd) Versus Pomalidomide, Bortezomib and Dexamethasone (PVd) in Participants With Relapsed or Refractory Multiple Myeloma (RRMM) [NCT05519085]</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria
+\- Participant has documented diagnosis of MM and measurable disease, defined as any of the following:.
+i) M-protein ≥ 0.5 grams per deciliter (g/dL) by serum protein electrophoresis (sPEP) or.
+ii) M-protein ≥ 200 milligrams (mg) per 24-hour urine collection by urine protein electrophoresis (uPEP).
+iii) For participants without measurable disease in sPEP or uPEP: serum free light chain (sFLC) levels \&gt; 100 mg/L (10 mg/dL) involved light chain and an abnormal kappa/lambda FLC ratio.
+* Participants received 1 to 3 prior lines of antimyeloma therapy.
+* Participants achieved minimal response \[MR\] or better to at least 1 prior antimyeloma therapy.
+Exclusion Criteria
+\- Participant has had progression during treatment or within 60 days of the last dose of a proteasome inhibitor, except as noted below:.
+i) Subjects who progressed while being treated with, or within 60 days of last dose of bortezomib maintenance given once every 2 weeks (or less frequently) are not excluded.
+ii) Participants who progressed while being treated with ixazomib monotherapy maintenance ≥ 6 months prior to the time of starting study treatment are not excluded.
+* For participants with prior treatment of a bortezomib containing regimen, the best response achieved was not a minimal response (MR) or better, or participant discontinued bortezomib due to toxicity.
+* Participant has had prior treatment with mezigdomide or pomalidomide.
+* Other protocol-defined Inclusion/Exclusion criteria apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>Course Name</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>02-Jul 12:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="36" customHeight="1">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>A Phase III Study of AZD0780 on Major Adverse CV Events in Patients With a History of ASCVD Events or at High Risk for a First Event [NCT07000357]</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Status: RECRUITING  |  Age: 18 Years – Not specified  |  All
+Inclusion Criteria:
+* Meets one of the following:
+  1. Participants with history of an ASCVD event: Participants ≥ 18 years of age at the time of signing the ICF with a history of MI or ischaemic stroke suspected to be due to atherosclerotic vascular disease ≥ 1 month prior to randomisation (presumed lacunar or cardioembolic strokes are not qualifying events), or revascularisation for symptomatic lower limb PAD any time prior to screening
+     Additional risk factors based on the level of the LDL-C and timing of MI or stroke:
+     o Participants with an LDL-C ≥ 75 mg/dL (≥ 1.9 mmol/L) need to have at least one of the other additional risk factors (i to viii) below.
+     ii) T2DM requiring ongoing medical therapy iii) Age ≥ 65 years v) Previous above ankle amputation due to PAD vi) Previous diagnosis of non-end stage CKD
+  2. Participants at increased risk of a first ASCVD event: Male participant ≥ 50 years of age or female participant ≥ 55 years of age at the time of signing the ICF with LDL-C ≥ 100 mg/dL (≥ 2.6 mmol/L), with no prior history of MI, ischaemic stroke due to atherosclerotic disease, or leg revascularisation for symptomatic lower limb PAD, and with diagnostic evidence of at least one of the following disease categories (i, ii, or iii):
+  (i) Significant atherosclerotic artery disease (ii) High-risk Type 1 or Type 2 diabetes mellitus with manifestation of at least one of the following end-organ diseases:
+  1. Nephropathy - Persistent (≥ 2 readings) microalbuminuria (urine albumin/creatinine ratio ≥ 30 mg/g) and/or persistent eGFR \&lt; 60 mL/min/1.73 m2. At least one reading must come from the medical record within the last 12 months in addition to the reading from screening
+  2. Retinopathy - Treated diabetic retinopathy (surgical intervention or injectable therapy) or prior diagnosis made by a relevant healthcare specialist
+  3. Neuropathy - Treated neuropathy (medical therapy for pain relief or symptom alleviation) or prior diagnosis made by a relevant healthcare specialist
+  4. ABI \&lt; 0.9 or \&gt; 1.4 - confirmed either in study during screening or randomisation, or from the medical record within the last 5 years (iii) Documented atherosclerosis of less significance
+     For (ii) and (iii), participants need to have at least one of the additional risk factors below:
+  &lt;!-- --&gt;
+  1. CKD with eGFR x mL/min/1.73 m2
+  2. Current tobacco use
+  3. Age ≥ 65
+  4. T2DM (if included on the less significant atherosclerosis criterion iii)
+* Participants should receive a background lipid lowering regimen anticipated to achieve at least a \~50% reduction in LDL-C. Except in cases of intolerance, the regimen should include a high intensity statin therapy or lower intensity statin therapy in combination with an oral agent with proven outcome benefit (eg, ezetimibe and/or bempedoic acid).
+Participants must achieve a stable background lipid lowering therapy \&gt; 28 days before screening.
+Exclusion criteria:
+* Any underlying known disease, or condition including homozygous familial hypercholesterolaemia, or LDL or plasma apheresis within 12 months prior to randomisation, that, in the opinion of the investigator, might interfere with the interpretation of the clinical study results.
+* Any revascularisation procedure planned within the next 3 months.
+* Available imaging assessment within the last 3 years showing either coronary calcium score of zero, or a coronary computed tomography angiography with no atherosclerosis.
+* Calculated eGFR \&lt; 15 mL /min/1.73 m2 at screening.
+* Any laboratory values with the following deviations at screening:
+  * AST or ALT \&gt; 3 × ULN
+  * TBL \&gt; 2 × ULN (except for participants with Gilbert's syndrome where TBL 3 × ULN is acceptable provided direct bilirubin \&lt; 1.5 × ULN)
+  * Fasting triglycerides ≥ 400 mg/dL (≥ 4.52 mmol/L).
+  * Creatine kinase \&gt; 5 × ULN
+  * Urine albumin/creatinine ratio ≥ 500 mg/g
+* Uncontrolled T2DM defined as HbA1c ≥ 9.5% at screening.
+* Inadequately treated hypothyroidism defined as TSH \&gt; 1.5 × ULN at screening or participants whose thyroid replacement therapy was initiated or modified within the last 3 months prior to screening.
+* Use of mipomersen or lomitapide (cholesterol-lowering medications) within 12 months of screening or planned use during the study.
+* Use of gemfibrozil within one week prior to the Screening Visit or planned use during the study.
+* Use of PCSK9 inhibitors: evolocumab/alirocumab within 12 weeks of the Screening Visit or planned use during the study, or inclisiran within 18 months of the Screening Visit or planned use during the study, or any other approved PCSK9 inhibitor use within 5 half lives prior to the Screening Visit or planned use during the study.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor update 2026-07-02 14:39 UTC
</commit_message>
<xml_diff>
--- a/clearing_data.xlsx
+++ b/clearing_data.xlsx
@@ -3619,7 +3619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C148"/>
+  <dimension ref="A3:C148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3627,8 +3627,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3677,7 +3675,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3719,7 +3716,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3777,7 +3773,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -3831,7 +3826,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -3910,7 +3904,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -3985,7 +3978,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
@@ -4036,7 +4028,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -4072,7 +4063,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
@@ -4111,7 +4101,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -4145,7 +4134,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
@@ -4194,7 +4182,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
@@ -4256,7 +4243,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
@@ -4301,7 +4287,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
@@ -4343,7 +4328,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
@@ -4392,7 +4376,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
@@ -4429,7 +4412,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
@@ -4478,7 +4460,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -4526,7 +4507,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
@@ -4575,7 +4555,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
@@ -4613,7 +4592,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
@@ -4663,7 +4641,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
@@ -4715,7 +4692,6 @@
         </is>
       </c>
     </row>
-    <row r="68"/>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
@@ -4765,7 +4741,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
@@ -4806,7 +4781,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -4870,7 +4844,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
@@ -4902,7 +4875,6 @@
         </is>
       </c>
     </row>
-    <row r="80"/>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
@@ -4944,7 +4916,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
@@ -4982,7 +4953,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
@@ -5019,7 +4989,6 @@
         </is>
       </c>
     </row>
-    <row r="89"/>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
@@ -5057,7 +5026,6 @@
         </is>
       </c>
     </row>
-    <row r="92"/>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="1" t="inlineStr">
         <is>
@@ -5097,7 +5065,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
@@ -5137,7 +5104,6 @@
         </is>
       </c>
     </row>
-    <row r="98"/>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="1" t="inlineStr">
         <is>
@@ -5180,7 +5146,6 @@
         </is>
       </c>
     </row>
-    <row r="101"/>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -5232,7 +5197,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
         <is>
@@ -5283,7 +5247,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="1" t="inlineStr">
         <is>
@@ -5348,7 +5311,6 @@
         </is>
       </c>
     </row>
-    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
         <is>
@@ -5382,7 +5344,6 @@
         </is>
       </c>
     </row>
-    <row r="113"/>
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
         <is>
@@ -5427,7 +5388,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
@@ -5486,7 +5446,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="1" t="inlineStr">
         <is>
@@ -5520,7 +5479,6 @@
         </is>
       </c>
     </row>
-    <row r="122"/>
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
         <is>
@@ -5582,7 +5540,6 @@
         </is>
       </c>
     </row>
-    <row r="125"/>
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="1" t="inlineStr">
         <is>
@@ -5618,7 +5575,6 @@
         </is>
       </c>
     </row>
-    <row r="128"/>
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
         <is>
@@ -5671,7 +5627,6 @@
         </is>
       </c>
     </row>
-    <row r="131"/>
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="1" t="inlineStr">
         <is>
@@ -5724,7 +5679,6 @@
         </is>
       </c>
     </row>
-    <row r="134"/>
     <row r="135" ht="22" customHeight="1">
       <c r="A135" s="1" t="inlineStr">
         <is>
@@ -5778,7 +5732,6 @@
         </is>
       </c>
     </row>
-    <row r="137"/>
     <row r="138" ht="22" customHeight="1">
       <c r="A138" s="1" t="inlineStr">
         <is>
@@ -5833,7 +5786,6 @@
         </is>
       </c>
     </row>
-    <row r="140"/>
     <row r="141" ht="22" customHeight="1">
       <c r="A141" s="1" t="inlineStr">
         <is>
@@ -5872,7 +5824,6 @@
         </is>
       </c>
     </row>
-    <row r="143"/>
     <row r="144" ht="22" customHeight="1">
       <c r="A144" s="1" t="inlineStr">
         <is>

</xml_diff>